<commit_message>
Refine chart styling: soft ggplot2 colors, cleaner layout
- Soft ggplot2-inspired colors: blue, coral, green
- Pie chart: smaller, no text labels inside (legend only)
- Line chart: smaller, no overlap with pie, wider lines (~2.2pt)
- Very faint gray gridlines (E0E0E0)
- Removed axis titles (Year, Dollars)
- Y-axis ticks formatted as $300K, $200K, etc.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/mortgage-amortization-calculator/mortgage_amortization_calculator.xlsx
+++ b/mortgage-amortization-calculator/mortgage_amortization_calculator.xlsx
@@ -270,7 +270,7 @@
             <idx val="0"/>
             <spPr>
               <a:solidFill>
-                <a:srgbClr val="2F5496"/>
+                <a:srgbClr val="619CFF"/>
               </a:solidFill>
               <a:ln>
                 <a:prstDash val="solid"/>
@@ -281,7 +281,7 @@
             <idx val="1"/>
             <spPr>
               <a:solidFill>
-                <a:srgbClr val="C00000"/>
+                <a:srgbClr val="F8766D"/>
               </a:solidFill>
               <a:ln>
                 <a:prstDash val="solid"/>
@@ -290,8 +290,9 @@
           </dPt>
           <dLbls>
             <showVal val="0"/>
-            <showCatName val="1"/>
-            <showPercent val="1"/>
+            <showCatName val="0"/>
+            <showSerName val="0"/>
+            <showPercent val="0"/>
           </dLbls>
           <cat>
             <numRef>
@@ -347,9 +348,9 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="20000">
+            <a:ln w="28000">
               <a:solidFill>
-                <a:srgbClr val="2F5496"/>
+                <a:srgbClr val="619CFF"/>
               </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -383,9 +384,9 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="20000">
+            <a:ln w="28000">
               <a:solidFill>
-                <a:srgbClr val="C00000"/>
+                <a:srgbClr val="F8766D"/>
               </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -419,9 +420,9 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="20000">
+            <a:ln w="28000">
               <a:solidFill>
-                <a:srgbClr val="006600"/>
+                <a:srgbClr val="00BA38"/>
               </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -456,21 +457,16 @@
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Year</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
+        <majorGridlines>
+          <spPr>
+            <a:ln w="6350">
+              <a:solidFill>
+                <a:srgbClr val="E0E0E0"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+        </majorGridlines>
         <numFmt formatCode="YYYY" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
@@ -484,23 +480,17 @@
           <orientation val="minMax"/>
         </scaling>
         <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Dollars ($)</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <numFmt formatCode="#,##0" sourceLinked="0"/>
+        <majorGridlines>
+          <spPr>
+            <a:ln w="6350">
+              <a:solidFill>
+                <a:srgbClr val="E0E0E0"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+        </majorGridlines>
+        <numFmt formatCode="$#,##0,K" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
@@ -524,7 +514,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6480000" cy="5040000"/>
+    <ext cx="5040000" cy="3960000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -543,10 +533,10 @@
     <from>
       <col>16</col>
       <colOff>0</colOff>
-      <row>15</row>
+      <row>13</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="10080000" cy="5760000"/>
+    <ext cx="7920000" cy="4680000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="2" name="Chart 2"/>

</xml_diff>

<commit_message>
Chart tweaks: 75% size, 5-year x-axis ticks, dollar y-axis
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/mortgage-amortization-calculator/mortgage_amortization_calculator.xlsx
+++ b/mortgage-amortization-calculator/mortgage_amortization_calculator.xlsx
@@ -480,6 +480,7 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
@@ -515,7 +516,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5040000" cy="3960000"/>
+    <ext cx="3780000" cy="2970000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -537,7 +538,7 @@
       <row>13</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7920000" cy="4680000"/>
+    <ext cx="5940000" cy="3510000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="2" name="Chart 2"/>

</xml_diff>

<commit_message>
Move both charts down 3 rows
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/mortgage-amortization-calculator/mortgage_amortization_calculator.xlsx
+++ b/mortgage-amortization-calculator/mortgage_amortization_calculator.xlsx
@@ -513,7 +513,7 @@
     <from>
       <col>18</col>
       <colOff>0</colOff>
-      <row>0</row>
+      <row>3</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="3780000" cy="2970000"/>
@@ -535,7 +535,7 @@
     <from>
       <col>18</col>
       <colOff>0</colOff>
-      <row>18</row>
+      <row>21</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5940000" cy="3510000"/>

</xml_diff>

<commit_message>
Add current monthly payment row to loan details
- Rename 'Monthly Payment' to 'Min Monthly Payment'
- Add 'Current Monthly Payment' row (row 7) showing base payment + monthly recurring extras

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/mortgage-amortization-calculator/mortgage_amortization_calculator.xlsx
+++ b/mortgage-amortization-calculator/mortgage_amortization_calculator.xlsx
@@ -1104,7 +1104,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Monthly Payment</t>
+          <t>Min Monthly Payment</t>
         </is>
       </c>
       <c r="B6" s="16">
@@ -1145,6 +1145,15 @@
       </c>
     </row>
     <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Current Monthly Payment</t>
+        </is>
+      </c>
+      <c r="B7" s="16">
+        <f>B6+SUMPRODUCT(($E$21:$E$30="Monthly")*($D$21:$D$30&lt;&gt;"")*$D$21:$D$30)</f>
+        <v/>
+      </c>
       <c r="H7" s="7">
         <f>IF(AND(L6&gt;0.005,H6&lt;&gt;""),5,"")</f>
         <v/>

</xml_diff>

<commit_message>
Rename to Base Monthly Payment, shift lower sections down one row
- Rename 'Min Monthly Payment' to 'Base Monthly Payment'
- Add gap row (row 8) between Loan Details and Loan Summary
- Shift Loan Summary, Recurring Extra Payments, and One-Time Extra Payments sections down by one row
- Update all cross-cell formula references for new row positions

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/mortgage-amortization-calculator/mortgage_amortization_calculator.xlsx
+++ b/mortgage-amortization-calculator/mortgage_amortization_calculator.xlsx
@@ -988,7 +988,7 @@
         <v/>
       </c>
       <c r="K3" s="9">
-        <f>IF(H3&lt;&gt;"",MIN(LoanAmount,(M3-J3)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I3)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I3))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I3)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I3))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I3))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I3))*(MONTH($B$34:$B$48)=MONTH(I3))*$C$34:$C$48)),"")</f>
+        <f>IF(H3&lt;&gt;"",MIN(LoanAmount,(M3-J3)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I3)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I3))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I3)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I3))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I3))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I3))*(MONTH($B$35:$B$49)=MONTH(I3))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L3" s="9">
@@ -1013,7 +1013,7 @@
         </is>
       </c>
       <c r="Q3" s="2">
-        <f>B13</f>
+        <f>B14</f>
         <v/>
       </c>
     </row>
@@ -1039,7 +1039,7 @@
         <v/>
       </c>
       <c r="K4" s="14">
-        <f>IF(H4&lt;&gt;"",MIN(L3,(M4-J4)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I4)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I4))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I4)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I4))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I4))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I4))*(MONTH($B$34:$B$48)=MONTH(I4))*$C$34:$C$48)),"")</f>
+        <f>IF(H4&lt;&gt;"",MIN(L3,(M4-J4)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I4)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I4))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I4)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I4))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I4))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I4))*(MONTH($B$35:$B$49)=MONTH(I4))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L4" s="14">
@@ -1081,7 +1081,7 @@
         <v/>
       </c>
       <c r="K5" s="9">
-        <f>IF(H5&lt;&gt;"",MIN(L4,(M5-J5)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I5)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I5))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I5)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I5))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I5))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I5))*(MONTH($B$34:$B$48)=MONTH(I5))*$C$34:$C$48)),"")</f>
+        <f>IF(H5&lt;&gt;"",MIN(L4,(M5-J5)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I5)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I5))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I5)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I5))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I5))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I5))*(MONTH($B$35:$B$49)=MONTH(I5))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L5" s="9">
@@ -1104,7 +1104,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Min Monthly Payment</t>
+          <t>Base Monthly Payment</t>
         </is>
       </c>
       <c r="B6" s="16">
@@ -1124,7 +1124,7 @@
         <v/>
       </c>
       <c r="K6" s="14">
-        <f>IF(H6&lt;&gt;"",MIN(L5,(M6-J6)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I6)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I6))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I6)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I6))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I6))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I6))*(MONTH($B$34:$B$48)=MONTH(I6))*$C$34:$C$48)),"")</f>
+        <f>IF(H6&lt;&gt;"",MIN(L5,(M6-J6)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I6)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I6))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I6)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I6))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I6))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I6))*(MONTH($B$35:$B$49)=MONTH(I6))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L6" s="14">
@@ -1151,7 +1151,7 @@
         </is>
       </c>
       <c r="B7" s="16">
-        <f>B6+SUMPRODUCT(($E$21:$E$30="Monthly")*($D$21:$D$30&lt;&gt;"")*$D$21:$D$30)</f>
+        <f>B6+SUMPRODUCT(($E$22:$E$31="Monthly")*($D$22:$D$31&lt;&gt;"")*$D$22:$D$31)</f>
         <v/>
       </c>
       <c r="H7" s="7">
@@ -1167,7 +1167,7 @@
         <v/>
       </c>
       <c r="K7" s="9">
-        <f>IF(H7&lt;&gt;"",MIN(L6,(M7-J7)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I7)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I7))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I7)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I7))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I7))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I7))*(MONTH($B$34:$B$48)=MONTH(I7))*$C$34:$C$48)),"")</f>
+        <f>IF(H7&lt;&gt;"",MIN(L6,(M7-J7)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I7)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I7))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I7)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I7))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I7))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I7))*(MONTH($B$35:$B$49)=MONTH(I7))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L7" s="9">
@@ -1188,432 +1188,432 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="inlineStr">
+      <c r="H8" s="12">
+        <f>IF(AND(L7&gt;0.005,H7&lt;&gt;""),6,"")</f>
+        <v/>
+      </c>
+      <c r="I8" s="13">
+        <f>IF(H8&lt;&gt;"",EDATE(StartDate,5),"")</f>
+        <v/>
+      </c>
+      <c r="J8" s="14">
+        <f>IF(H8&lt;&gt;"",ROUND(L7*AnnualRate/12,2),"")</f>
+        <v/>
+      </c>
+      <c r="K8" s="14">
+        <f>IF(H8&lt;&gt;"",MIN(L7,(M8-J8)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I8)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I8))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I8)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I8))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I8))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I8))*(MONTH($B$35:$B$49)=MONTH(I8))*$C$35:$C$49)),"")</f>
+        <v/>
+      </c>
+      <c r="L8" s="14">
+        <f>IF(H8&lt;&gt;"",ROUND(L7-K8,2),"")</f>
+        <v/>
+      </c>
+      <c r="M8" s="10">
+        <f>IF(H8&lt;&gt;"",MIN(MonthlyPmt,L7+J8),"")</f>
+        <v/>
+      </c>
+      <c r="N8" s="10">
+        <f>IF(H8&lt;&gt;"",N7+K8,"")</f>
+        <v/>
+      </c>
+      <c r="O8" s="10">
+        <f>IF(H8&lt;&gt;"",O7+J8,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
         <is>
           <t>LOAN SUMMARY</t>
         </is>
       </c>
-      <c r="H8" s="12">
-        <f>IF(AND(L7&gt;0.005,H7&lt;&gt;""),6,"")</f>
-        <v/>
-      </c>
-      <c r="I8" s="13">
-        <f>IF(H8&lt;&gt;"",EDATE(StartDate,5),"")</f>
-        <v/>
-      </c>
-      <c r="J8" s="14">
-        <f>IF(H8&lt;&gt;"",ROUND(L7*AnnualRate/12,2),"")</f>
-        <v/>
-      </c>
-      <c r="K8" s="14">
-        <f>IF(H8&lt;&gt;"",MIN(L7,(M8-J8)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I8)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I8))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I8)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I8))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I8))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I8))*(MONTH($B$34:$B$48)=MONTH(I8))*$C$34:$C$48)),"")</f>
-        <v/>
-      </c>
-      <c r="L8" s="14">
-        <f>IF(H8&lt;&gt;"",ROUND(L7-K8,2),"")</f>
-        <v/>
-      </c>
-      <c r="M8" s="10">
-        <f>IF(H8&lt;&gt;"",MIN(MonthlyPmt,L7+J8),"")</f>
-        <v/>
-      </c>
-      <c r="N8" s="10">
-        <f>IF(H8&lt;&gt;"",N7+K8,"")</f>
-        <v/>
-      </c>
-      <c r="O8" s="10">
-        <f>IF(H8&lt;&gt;"",O7+J8,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="H9" s="7">
+        <f>IF(AND(L8&gt;0.005,H8&lt;&gt;""),7,"")</f>
+        <v/>
+      </c>
+      <c r="I9" s="8">
+        <f>IF(H9&lt;&gt;"",EDATE(StartDate,6),"")</f>
+        <v/>
+      </c>
+      <c r="J9" s="9">
+        <f>IF(H9&lt;&gt;"",ROUND(L8*AnnualRate/12,2),"")</f>
+        <v/>
+      </c>
+      <c r="K9" s="9">
+        <f>IF(H9&lt;&gt;"",MIN(L8,(M9-J9)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I9)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I9))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I9)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I9))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I9))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I9))*(MONTH($B$35:$B$49)=MONTH(I9))*$C$35:$C$49)),"")</f>
+        <v/>
+      </c>
+      <c r="L9" s="9">
+        <f>IF(H9&lt;&gt;"",ROUND(L8-K9,2),"")</f>
+        <v/>
+      </c>
+      <c r="M9" s="10">
+        <f>IF(H9&lt;&gt;"",MIN(MonthlyPmt,L8+J9),"")</f>
+        <v/>
+      </c>
+      <c r="N9" s="10">
+        <f>IF(H9&lt;&gt;"",N8+K9,"")</f>
+        <v/>
+      </c>
+      <c r="O9" s="10">
+        <f>IF(H9&lt;&gt;"",O8+J9,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>Original Payoff Date</t>
         </is>
       </c>
-      <c r="B9" s="17">
+      <c r="B10" s="17">
         <f>EDATE(StartDate,TermYears*12-1)</f>
         <v/>
       </c>
-      <c r="H9" s="7">
-        <f>IF(AND(L8&gt;0.005,H8&lt;&gt;""),7,"")</f>
-        <v/>
-      </c>
-      <c r="I9" s="8">
-        <f>IF(H9&lt;&gt;"",EDATE(StartDate,6),"")</f>
-        <v/>
-      </c>
-      <c r="J9" s="9">
-        <f>IF(H9&lt;&gt;"",ROUND(L8*AnnualRate/12,2),"")</f>
-        <v/>
-      </c>
-      <c r="K9" s="9">
-        <f>IF(H9&lt;&gt;"",MIN(L8,(M9-J9)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I9)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I9))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I9)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I9))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I9))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I9))*(MONTH($B$34:$B$48)=MONTH(I9))*$C$34:$C$48)),"")</f>
-        <v/>
-      </c>
-      <c r="L9" s="9">
-        <f>IF(H9&lt;&gt;"",ROUND(L8-K9,2),"")</f>
-        <v/>
-      </c>
-      <c r="M9" s="10">
-        <f>IF(H9&lt;&gt;"",MIN(MonthlyPmt,L8+J9),"")</f>
-        <v/>
-      </c>
-      <c r="N9" s="10">
-        <f>IF(H9&lt;&gt;"",N8+K9,"")</f>
-        <v/>
-      </c>
-      <c r="O9" s="10">
-        <f>IF(H9&lt;&gt;"",O8+J9,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="H10" s="12">
+        <f>IF(AND(L9&gt;0.005,H9&lt;&gt;""),8,"")</f>
+        <v/>
+      </c>
+      <c r="I10" s="13">
+        <f>IF(H10&lt;&gt;"",EDATE(StartDate,7),"")</f>
+        <v/>
+      </c>
+      <c r="J10" s="14">
+        <f>IF(H10&lt;&gt;"",ROUND(L9*AnnualRate/12,2),"")</f>
+        <v/>
+      </c>
+      <c r="K10" s="14">
+        <f>IF(H10&lt;&gt;"",MIN(L9,(M10-J10)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I10)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I10))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I10)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I10))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I10))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I10))*(MONTH($B$35:$B$49)=MONTH(I10))*$C$35:$C$49)),"")</f>
+        <v/>
+      </c>
+      <c r="L10" s="14">
+        <f>IF(H10&lt;&gt;"",ROUND(L9-K10,2),"")</f>
+        <v/>
+      </c>
+      <c r="M10" s="10">
+        <f>IF(H10&lt;&gt;"",MIN(MonthlyPmt,L9+J10),"")</f>
+        <v/>
+      </c>
+      <c r="N10" s="10">
+        <f>IF(H10&lt;&gt;"",N9+K10,"")</f>
+        <v/>
+      </c>
+      <c r="O10" s="10">
+        <f>IF(H10&lt;&gt;"",O9+J10,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>Accelerated Payoff Date</t>
         </is>
       </c>
-      <c r="B10" s="17">
+      <c r="B11" s="17">
         <f>LOOKUP(2,1/(I3:I362&lt;&gt;""),I3:I362)</f>
         <v/>
       </c>
-      <c r="H10" s="12">
-        <f>IF(AND(L9&gt;0.005,H9&lt;&gt;""),8,"")</f>
-        <v/>
-      </c>
-      <c r="I10" s="13">
-        <f>IF(H10&lt;&gt;"",EDATE(StartDate,7),"")</f>
-        <v/>
-      </c>
-      <c r="J10" s="14">
-        <f>IF(H10&lt;&gt;"",ROUND(L9*AnnualRate/12,2),"")</f>
-        <v/>
-      </c>
-      <c r="K10" s="14">
-        <f>IF(H10&lt;&gt;"",MIN(L9,(M10-J10)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I10)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I10))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I10)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I10))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I10))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I10))*(MONTH($B$34:$B$48)=MONTH(I10))*$C$34:$C$48)),"")</f>
-        <v/>
-      </c>
-      <c r="L10" s="14">
-        <f>IF(H10&lt;&gt;"",ROUND(L9-K10,2),"")</f>
-        <v/>
-      </c>
-      <c r="M10" s="10">
-        <f>IF(H10&lt;&gt;"",MIN(MonthlyPmt,L9+J10),"")</f>
-        <v/>
-      </c>
-      <c r="N10" s="10">
-        <f>IF(H10&lt;&gt;"",N9+K10,"")</f>
-        <v/>
-      </c>
-      <c r="O10" s="10">
-        <f>IF(H10&lt;&gt;"",O9+J10,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="H11" s="7">
+        <f>IF(AND(L10&gt;0.005,H10&lt;&gt;""),9,"")</f>
+        <v/>
+      </c>
+      <c r="I11" s="8">
+        <f>IF(H11&lt;&gt;"",EDATE(StartDate,8),"")</f>
+        <v/>
+      </c>
+      <c r="J11" s="9">
+        <f>IF(H11&lt;&gt;"",ROUND(L10*AnnualRate/12,2),"")</f>
+        <v/>
+      </c>
+      <c r="K11" s="9">
+        <f>IF(H11&lt;&gt;"",MIN(L10,(M11-J11)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I11)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I11))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I11)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I11))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I11))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I11))*(MONTH($B$35:$B$49)=MONTH(I11))*$C$35:$C$49)),"")</f>
+        <v/>
+      </c>
+      <c r="L11" s="9">
+        <f>IF(H11&lt;&gt;"",ROUND(L10-K11,2),"")</f>
+        <v/>
+      </c>
+      <c r="M11" s="10">
+        <f>IF(H11&lt;&gt;"",MIN(MonthlyPmt,L10+J11),"")</f>
+        <v/>
+      </c>
+      <c r="N11" s="10">
+        <f>IF(H11&lt;&gt;"",N10+K11,"")</f>
+        <v/>
+      </c>
+      <c r="O11" s="10">
+        <f>IF(H11&lt;&gt;"",O10+J11,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Accelerated Payoff Time</t>
         </is>
       </c>
-      <c r="B11" s="18">
+      <c r="B12" s="18">
         <f>INT(SUMPRODUCT(1*(ISNUMBER(H3:H362)))/12)&amp;" years, "&amp;MOD(SUMPRODUCT(1*(ISNUMBER(H3:H362))),12)&amp;" months"</f>
         <v/>
       </c>
-      <c r="H11" s="7">
-        <f>IF(AND(L10&gt;0.005,H10&lt;&gt;""),9,"")</f>
-        <v/>
-      </c>
-      <c r="I11" s="8">
-        <f>IF(H11&lt;&gt;"",EDATE(StartDate,8),"")</f>
-        <v/>
-      </c>
-      <c r="J11" s="9">
-        <f>IF(H11&lt;&gt;"",ROUND(L10*AnnualRate/12,2),"")</f>
-        <v/>
-      </c>
-      <c r="K11" s="9">
-        <f>IF(H11&lt;&gt;"",MIN(L10,(M11-J11)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I11)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I11))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I11)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I11))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I11))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I11))*(MONTH($B$34:$B$48)=MONTH(I11))*$C$34:$C$48)),"")</f>
-        <v/>
-      </c>
-      <c r="L11" s="9">
-        <f>IF(H11&lt;&gt;"",ROUND(L10-K11,2),"")</f>
-        <v/>
-      </c>
-      <c r="M11" s="10">
-        <f>IF(H11&lt;&gt;"",MIN(MonthlyPmt,L10+J11),"")</f>
-        <v/>
-      </c>
-      <c r="N11" s="10">
-        <f>IF(H11&lt;&gt;"",N10+K11,"")</f>
-        <v/>
-      </c>
-      <c r="O11" s="10">
-        <f>IF(H11&lt;&gt;"",O10+J11,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="H12" s="12">
+        <f>IF(AND(L11&gt;0.005,H11&lt;&gt;""),10,"")</f>
+        <v/>
+      </c>
+      <c r="I12" s="13">
+        <f>IF(H12&lt;&gt;"",EDATE(StartDate,9),"")</f>
+        <v/>
+      </c>
+      <c r="J12" s="14">
+        <f>IF(H12&lt;&gt;"",ROUND(L11*AnnualRate/12,2),"")</f>
+        <v/>
+      </c>
+      <c r="K12" s="14">
+        <f>IF(H12&lt;&gt;"",MIN(L11,(M12-J12)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I12)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I12))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I12)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I12))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I12))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I12))*(MONTH($B$35:$B$49)=MONTH(I12))*$C$35:$C$49)),"")</f>
+        <v/>
+      </c>
+      <c r="L12" s="14">
+        <f>IF(H12&lt;&gt;"",ROUND(L11-K12,2),"")</f>
+        <v/>
+      </c>
+      <c r="M12" s="10">
+        <f>IF(H12&lt;&gt;"",MIN(MonthlyPmt,L11+J12),"")</f>
+        <v/>
+      </c>
+      <c r="N12" s="10">
+        <f>IF(H12&lt;&gt;"",N11+K12,"")</f>
+        <v/>
+      </c>
+      <c r="O12" s="10">
+        <f>IF(H12&lt;&gt;"",O11+J12,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Original Total Interest</t>
         </is>
       </c>
-      <c r="B12" s="19">
+      <c r="B13" s="19">
         <f>ROUND(MonthlyPmt*TermYears*12-LoanAmount,2)</f>
         <v/>
       </c>
-      <c r="H12" s="12">
-        <f>IF(AND(L11&gt;0.005,H11&lt;&gt;""),10,"")</f>
-        <v/>
-      </c>
-      <c r="I12" s="13">
-        <f>IF(H12&lt;&gt;"",EDATE(StartDate,9),"")</f>
-        <v/>
-      </c>
-      <c r="J12" s="14">
-        <f>IF(H12&lt;&gt;"",ROUND(L11*AnnualRate/12,2),"")</f>
-        <v/>
-      </c>
-      <c r="K12" s="14">
-        <f>IF(H12&lt;&gt;"",MIN(L11,(M12-J12)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I12)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I12))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I12)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I12))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I12))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I12))*(MONTH($B$34:$B$48)=MONTH(I12))*$C$34:$C$48)),"")</f>
-        <v/>
-      </c>
-      <c r="L12" s="14">
-        <f>IF(H12&lt;&gt;"",ROUND(L11-K12,2),"")</f>
-        <v/>
-      </c>
-      <c r="M12" s="10">
-        <f>IF(H12&lt;&gt;"",MIN(MonthlyPmt,L11+J12),"")</f>
-        <v/>
-      </c>
-      <c r="N12" s="10">
-        <f>IF(H12&lt;&gt;"",N11+K12,"")</f>
-        <v/>
-      </c>
-      <c r="O12" s="10">
-        <f>IF(H12&lt;&gt;"",O11+J12,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="H13" s="7">
+        <f>IF(AND(L12&gt;0.005,H12&lt;&gt;""),11,"")</f>
+        <v/>
+      </c>
+      <c r="I13" s="8">
+        <f>IF(H13&lt;&gt;"",EDATE(StartDate,10),"")</f>
+        <v/>
+      </c>
+      <c r="J13" s="9">
+        <f>IF(H13&lt;&gt;"",ROUND(L12*AnnualRate/12,2),"")</f>
+        <v/>
+      </c>
+      <c r="K13" s="9">
+        <f>IF(H13&lt;&gt;"",MIN(L12,(M13-J13)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I13)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I13))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I13)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I13))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I13))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I13))*(MONTH($B$35:$B$49)=MONTH(I13))*$C$35:$C$49)),"")</f>
+        <v/>
+      </c>
+      <c r="L13" s="9">
+        <f>IF(H13&lt;&gt;"",ROUND(L12-K13,2),"")</f>
+        <v/>
+      </c>
+      <c r="M13" s="10">
+        <f>IF(H13&lt;&gt;"",MIN(MonthlyPmt,L12+J13),"")</f>
+        <v/>
+      </c>
+      <c r="N13" s="10">
+        <f>IF(H13&lt;&gt;"",N12+K13,"")</f>
+        <v/>
+      </c>
+      <c r="O13" s="10">
+        <f>IF(H13&lt;&gt;"",O12+J13,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>Accelerated Total Interest</t>
         </is>
       </c>
-      <c r="B13" s="19">
+      <c r="B14" s="19">
         <f>ROUND(SUM(J3:J362),2)</f>
         <v/>
       </c>
-      <c r="H13" s="7">
-        <f>IF(AND(L12&gt;0.005,H12&lt;&gt;""),11,"")</f>
-        <v/>
-      </c>
-      <c r="I13" s="8">
-        <f>IF(H13&lt;&gt;"",EDATE(StartDate,10),"")</f>
-        <v/>
-      </c>
-      <c r="J13" s="9">
-        <f>IF(H13&lt;&gt;"",ROUND(L12*AnnualRate/12,2),"")</f>
-        <v/>
-      </c>
-      <c r="K13" s="9">
-        <f>IF(H13&lt;&gt;"",MIN(L12,(M13-J13)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I13)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I13))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I13)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I13))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I13))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I13))*(MONTH($B$34:$B$48)=MONTH(I13))*$C$34:$C$48)),"")</f>
-        <v/>
-      </c>
-      <c r="L13" s="9">
-        <f>IF(H13&lt;&gt;"",ROUND(L12-K13,2),"")</f>
-        <v/>
-      </c>
-      <c r="M13" s="10">
-        <f>IF(H13&lt;&gt;"",MIN(MonthlyPmt,L12+J13),"")</f>
-        <v/>
-      </c>
-      <c r="N13" s="10">
-        <f>IF(H13&lt;&gt;"",N12+K13,"")</f>
-        <v/>
-      </c>
-      <c r="O13" s="10">
-        <f>IF(H13&lt;&gt;"",O12+J13,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="H14" s="12">
+        <f>IF(AND(L13&gt;0.005,H13&lt;&gt;""),12,"")</f>
+        <v/>
+      </c>
+      <c r="I14" s="13">
+        <f>IF(H14&lt;&gt;"",EDATE(StartDate,11),"")</f>
+        <v/>
+      </c>
+      <c r="J14" s="14">
+        <f>IF(H14&lt;&gt;"",ROUND(L13*AnnualRate/12,2),"")</f>
+        <v/>
+      </c>
+      <c r="K14" s="14">
+        <f>IF(H14&lt;&gt;"",MIN(L13,(M14-J14)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I14)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I14))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I14)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I14))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I14))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I14))*(MONTH($B$35:$B$49)=MONTH(I14))*$C$35:$C$49)),"")</f>
+        <v/>
+      </c>
+      <c r="L14" s="14">
+        <f>IF(H14&lt;&gt;"",ROUND(L13-K14,2),"")</f>
+        <v/>
+      </c>
+      <c r="M14" s="10">
+        <f>IF(H14&lt;&gt;"",MIN(MonthlyPmt,L13+J14),"")</f>
+        <v/>
+      </c>
+      <c r="N14" s="10">
+        <f>IF(H14&lt;&gt;"",N13+K14,"")</f>
+        <v/>
+      </c>
+      <c r="O14" s="10">
+        <f>IF(H14&lt;&gt;"",O13+J14,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>Interest Saved</t>
         </is>
       </c>
-      <c r="B14" s="20">
-        <f>B12-B13</f>
-        <v/>
-      </c>
-      <c r="H14" s="12">
-        <f>IF(AND(L13&gt;0.005,H13&lt;&gt;""),12,"")</f>
-        <v/>
-      </c>
-      <c r="I14" s="13">
-        <f>IF(H14&lt;&gt;"",EDATE(StartDate,11),"")</f>
-        <v/>
-      </c>
-      <c r="J14" s="14">
-        <f>IF(H14&lt;&gt;"",ROUND(L13*AnnualRate/12,2),"")</f>
-        <v/>
-      </c>
-      <c r="K14" s="14">
-        <f>IF(H14&lt;&gt;"",MIN(L13,(M14-J14)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I14)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I14))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I14)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I14))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I14))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I14))*(MONTH($B$34:$B$48)=MONTH(I14))*$C$34:$C$48)),"")</f>
-        <v/>
-      </c>
-      <c r="L14" s="14">
-        <f>IF(H14&lt;&gt;"",ROUND(L13-K14,2),"")</f>
-        <v/>
-      </c>
-      <c r="M14" s="10">
-        <f>IF(H14&lt;&gt;"",MIN(MonthlyPmt,L13+J14),"")</f>
-        <v/>
-      </c>
-      <c r="N14" s="10">
-        <f>IF(H14&lt;&gt;"",N13+K14,"")</f>
-        <v/>
-      </c>
-      <c r="O14" s="10">
-        <f>IF(H14&lt;&gt;"",O13+J14,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="B15" s="20">
+        <f>B13-B14</f>
+        <v/>
+      </c>
+      <c r="H15" s="7">
+        <f>IF(AND(L14&gt;0.005,H14&lt;&gt;""),13,"")</f>
+        <v/>
+      </c>
+      <c r="I15" s="8">
+        <f>IF(H15&lt;&gt;"",EDATE(StartDate,12),"")</f>
+        <v/>
+      </c>
+      <c r="J15" s="9">
+        <f>IF(H15&lt;&gt;"",ROUND(L14*AnnualRate/12,2),"")</f>
+        <v/>
+      </c>
+      <c r="K15" s="9">
+        <f>IF(H15&lt;&gt;"",MIN(L14,(M15-J15)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I15)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I15))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I15)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I15))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I15))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I15))*(MONTH($B$35:$B$49)=MONTH(I15))*$C$35:$C$49)),"")</f>
+        <v/>
+      </c>
+      <c r="L15" s="9">
+        <f>IF(H15&lt;&gt;"",ROUND(L14-K15,2),"")</f>
+        <v/>
+      </c>
+      <c r="M15" s="10">
+        <f>IF(H15&lt;&gt;"",MIN(MonthlyPmt,L14+J15),"")</f>
+        <v/>
+      </c>
+      <c r="N15" s="10">
+        <f>IF(H15&lt;&gt;"",N14+K15,"")</f>
+        <v/>
+      </c>
+      <c r="O15" s="10">
+        <f>IF(H15&lt;&gt;"",O14+J15,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Payoff Time Saved</t>
         </is>
       </c>
-      <c r="B15" s="21">
+      <c r="B16" s="21">
         <f>INT((TermYears*12-SUMPRODUCT(1*(ISNUMBER(H3:H362))))/12)&amp;" years, "&amp;MOD((TermYears*12-SUMPRODUCT(1*(ISNUMBER(H3:H362)))),12)&amp;" months"</f>
         <v/>
       </c>
-      <c r="H15" s="7">
-        <f>IF(AND(L14&gt;0.005,H14&lt;&gt;""),13,"")</f>
-        <v/>
-      </c>
-      <c r="I15" s="8">
-        <f>IF(H15&lt;&gt;"",EDATE(StartDate,12),"")</f>
-        <v/>
-      </c>
-      <c r="J15" s="9">
-        <f>IF(H15&lt;&gt;"",ROUND(L14*AnnualRate/12,2),"")</f>
-        <v/>
-      </c>
-      <c r="K15" s="9">
-        <f>IF(H15&lt;&gt;"",MIN(L14,(M15-J15)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I15)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I15))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I15)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I15))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I15))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I15))*(MONTH($B$34:$B$48)=MONTH(I15))*$C$34:$C$48)),"")</f>
-        <v/>
-      </c>
-      <c r="L15" s="9">
-        <f>IF(H15&lt;&gt;"",ROUND(L14-K15,2),"")</f>
-        <v/>
-      </c>
-      <c r="M15" s="10">
-        <f>IF(H15&lt;&gt;"",MIN(MonthlyPmt,L14+J15),"")</f>
-        <v/>
-      </c>
-      <c r="N15" s="10">
-        <f>IF(H15&lt;&gt;"",N14+K15,"")</f>
-        <v/>
-      </c>
-      <c r="O15" s="10">
-        <f>IF(H15&lt;&gt;"",O14+J15,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="H16" s="12">
+        <f>IF(AND(L15&gt;0.005,H15&lt;&gt;""),14,"")</f>
+        <v/>
+      </c>
+      <c r="I16" s="13">
+        <f>IF(H16&lt;&gt;"",EDATE(StartDate,13),"")</f>
+        <v/>
+      </c>
+      <c r="J16" s="14">
+        <f>IF(H16&lt;&gt;"",ROUND(L15*AnnualRate/12,2),"")</f>
+        <v/>
+      </c>
+      <c r="K16" s="14">
+        <f>IF(H16&lt;&gt;"",MIN(L15,(M16-J16)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I16)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I16))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I16)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I16))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I16))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I16))*(MONTH($B$35:$B$49)=MONTH(I16))*$C$35:$C$49)),"")</f>
+        <v/>
+      </c>
+      <c r="L16" s="14">
+        <f>IF(H16&lt;&gt;"",ROUND(L15-K16,2),"")</f>
+        <v/>
+      </c>
+      <c r="M16" s="10">
+        <f>IF(H16&lt;&gt;"",MIN(MonthlyPmt,L15+J16),"")</f>
+        <v/>
+      </c>
+      <c r="N16" s="10">
+        <f>IF(H16&lt;&gt;"",N15+K16,"")</f>
+        <v/>
+      </c>
+      <c r="O16" s="10">
+        <f>IF(H16&lt;&gt;"",O15+J16,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>Total of Payments (P+I)</t>
         </is>
       </c>
-      <c r="B16" s="19">
+      <c r="B17" s="19">
         <f>ROUND(SUM(M3:M362),2)</f>
         <v/>
       </c>
-      <c r="H16" s="12">
-        <f>IF(AND(L15&gt;0.005,H15&lt;&gt;""),14,"")</f>
-        <v/>
-      </c>
-      <c r="I16" s="13">
-        <f>IF(H16&lt;&gt;"",EDATE(StartDate,13),"")</f>
-        <v/>
-      </c>
-      <c r="J16" s="14">
-        <f>IF(H16&lt;&gt;"",ROUND(L15*AnnualRate/12,2),"")</f>
-        <v/>
-      </c>
-      <c r="K16" s="14">
-        <f>IF(H16&lt;&gt;"",MIN(L15,(M16-J16)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I16)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I16))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I16)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I16))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I16))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I16))*(MONTH($B$34:$B$48)=MONTH(I16))*$C$34:$C$48)),"")</f>
-        <v/>
-      </c>
-      <c r="L16" s="14">
-        <f>IF(H16&lt;&gt;"",ROUND(L15-K16,2),"")</f>
-        <v/>
-      </c>
-      <c r="M16" s="10">
-        <f>IF(H16&lt;&gt;"",MIN(MonthlyPmt,L15+J16),"")</f>
-        <v/>
-      </c>
-      <c r="N16" s="10">
-        <f>IF(H16&lt;&gt;"",N15+K16,"")</f>
-        <v/>
-      </c>
-      <c r="O16" s="10">
-        <f>IF(H16&lt;&gt;"",O15+J16,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="H17" s="7">
+        <f>IF(AND(L16&gt;0.005,H16&lt;&gt;""),15,"")</f>
+        <v/>
+      </c>
+      <c r="I17" s="8">
+        <f>IF(H17&lt;&gt;"",EDATE(StartDate,14),"")</f>
+        <v/>
+      </c>
+      <c r="J17" s="9">
+        <f>IF(H17&lt;&gt;"",ROUND(L16*AnnualRate/12,2),"")</f>
+        <v/>
+      </c>
+      <c r="K17" s="9">
+        <f>IF(H17&lt;&gt;"",MIN(L16,(M17-J17)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I17)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I17))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I17)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I17))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I17))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I17))*(MONTH($B$35:$B$49)=MONTH(I17))*$C$35:$C$49)),"")</f>
+        <v/>
+      </c>
+      <c r="L17" s="9">
+        <f>IF(H17&lt;&gt;"",ROUND(L16-K17,2),"")</f>
+        <v/>
+      </c>
+      <c r="M17" s="10">
+        <f>IF(H17&lt;&gt;"",MIN(MonthlyPmt,L16+J17),"")</f>
+        <v/>
+      </c>
+      <c r="N17" s="10">
+        <f>IF(H17&lt;&gt;"",N16+K17,"")</f>
+        <v/>
+      </c>
+      <c r="O17" s="10">
+        <f>IF(H17&lt;&gt;"",O16+J17,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>Total Extra Payments</t>
         </is>
       </c>
-      <c r="B17" s="19">
+      <c r="B18" s="19">
         <f>ROUND(SUM(K3:K362)-SUM(M3:M362)+SUM(J3:J362),2)</f>
         <v/>
       </c>
-      <c r="H17" s="7">
-        <f>IF(AND(L16&gt;0.005,H16&lt;&gt;""),15,"")</f>
-        <v/>
-      </c>
-      <c r="I17" s="8">
-        <f>IF(H17&lt;&gt;"",EDATE(StartDate,14),"")</f>
-        <v/>
-      </c>
-      <c r="J17" s="9">
-        <f>IF(H17&lt;&gt;"",ROUND(L16*AnnualRate/12,2),"")</f>
-        <v/>
-      </c>
-      <c r="K17" s="9">
-        <f>IF(H17&lt;&gt;"",MIN(L16,(M17-J17)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I17)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I17))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I17)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I17))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I17))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I17))*(MONTH($B$34:$B$48)=MONTH(I17))*$C$34:$C$48)),"")</f>
-        <v/>
-      </c>
-      <c r="L17" s="9">
-        <f>IF(H17&lt;&gt;"",ROUND(L16-K17,2),"")</f>
-        <v/>
-      </c>
-      <c r="M17" s="10">
-        <f>IF(H17&lt;&gt;"",MIN(MonthlyPmt,L16+J17),"")</f>
-        <v/>
-      </c>
-      <c r="N17" s="10">
-        <f>IF(H17&lt;&gt;"",N16+K17,"")</f>
-        <v/>
-      </c>
-      <c r="O17" s="10">
-        <f>IF(H17&lt;&gt;"",O16+J17,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
       <c r="H18" s="12">
         <f>IF(AND(L17&gt;0.005,H17&lt;&gt;""),16,"")</f>
         <v/>
@@ -1627,7 +1627,7 @@
         <v/>
       </c>
       <c r="K18" s="14">
-        <f>IF(H18&lt;&gt;"",MIN(L17,(M18-J18)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I18)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I18))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I18)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I18))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I18))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I18))*(MONTH($B$34:$B$48)=MONTH(I18))*$C$34:$C$48)),"")</f>
+        <f>IF(H18&lt;&gt;"",MIN(L17,(M18-J18)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I18)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I18))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I18)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I18))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I18))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I18))*(MONTH($B$35:$B$49)=MONTH(I18))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L18" s="14">
@@ -1648,111 +1648,104 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="inlineStr">
+      <c r="H19" s="7">
+        <f>IF(AND(L18&gt;0.005,H18&lt;&gt;""),17,"")</f>
+        <v/>
+      </c>
+      <c r="I19" s="8">
+        <f>IF(H19&lt;&gt;"",EDATE(StartDate,16),"")</f>
+        <v/>
+      </c>
+      <c r="J19" s="9">
+        <f>IF(H19&lt;&gt;"",ROUND(L18*AnnualRate/12,2),"")</f>
+        <v/>
+      </c>
+      <c r="K19" s="9">
+        <f>IF(H19&lt;&gt;"",MIN(L18,(M19-J19)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I19)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I19))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I19)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I19))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I19))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I19))*(MONTH($B$35:$B$49)=MONTH(I19))*$C$35:$C$49)),"")</f>
+        <v/>
+      </c>
+      <c r="L19" s="9">
+        <f>IF(H19&lt;&gt;"",ROUND(L18-K19,2),"")</f>
+        <v/>
+      </c>
+      <c r="M19" s="10">
+        <f>IF(H19&lt;&gt;"",MIN(MonthlyPmt,L18+J19),"")</f>
+        <v/>
+      </c>
+      <c r="N19" s="10">
+        <f>IF(H19&lt;&gt;"",N18+K19,"")</f>
+        <v/>
+      </c>
+      <c r="O19" s="10">
+        <f>IF(H19&lt;&gt;"",O18+J19,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
         <is>
           <t>RECURRING EXTRA PAYMENTS</t>
         </is>
       </c>
-      <c r="H19" s="7">
-        <f>IF(AND(L18&gt;0.005,H18&lt;&gt;""),17,"")</f>
-        <v/>
-      </c>
-      <c r="I19" s="8">
-        <f>IF(H19&lt;&gt;"",EDATE(StartDate,16),"")</f>
-        <v/>
-      </c>
-      <c r="J19" s="9">
-        <f>IF(H19&lt;&gt;"",ROUND(L18*AnnualRate/12,2),"")</f>
-        <v/>
-      </c>
-      <c r="K19" s="9">
-        <f>IF(H19&lt;&gt;"",MIN(L18,(M19-J19)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I19)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I19))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I19)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I19))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I19))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I19))*(MONTH($B$34:$B$48)=MONTH(I19))*$C$34:$C$48)),"")</f>
-        <v/>
-      </c>
-      <c r="L19" s="9">
-        <f>IF(H19&lt;&gt;"",ROUND(L18-K19,2),"")</f>
-        <v/>
-      </c>
-      <c r="M19" s="10">
-        <f>IF(H19&lt;&gt;"",MIN(MonthlyPmt,L18+J19),"")</f>
-        <v/>
-      </c>
-      <c r="N19" s="10">
-        <f>IF(H19&lt;&gt;"",N18+K19,"")</f>
-        <v/>
-      </c>
-      <c r="O19" s="10">
-        <f>IF(H19&lt;&gt;"",O18+J19,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="5" t="inlineStr">
+      <c r="H20" s="12">
+        <f>IF(AND(L19&gt;0.005,H19&lt;&gt;""),18,"")</f>
+        <v/>
+      </c>
+      <c r="I20" s="13">
+        <f>IF(H20&lt;&gt;"",EDATE(StartDate,17),"")</f>
+        <v/>
+      </c>
+      <c r="J20" s="14">
+        <f>IF(H20&lt;&gt;"",ROUND(L19*AnnualRate/12,2),"")</f>
+        <v/>
+      </c>
+      <c r="K20" s="14">
+        <f>IF(H20&lt;&gt;"",MIN(L19,(M20-J20)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I20)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I20))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I20)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I20))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I20))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I20))*(MONTH($B$35:$B$49)=MONTH(I20))*$C$35:$C$49)),"")</f>
+        <v/>
+      </c>
+      <c r="L20" s="14">
+        <f>IF(H20&lt;&gt;"",ROUND(L19-K20,2),"")</f>
+        <v/>
+      </c>
+      <c r="M20" s="10">
+        <f>IF(H20&lt;&gt;"",MIN(MonthlyPmt,L19+J20),"")</f>
+        <v/>
+      </c>
+      <c r="N20" s="10">
+        <f>IF(H20&lt;&gt;"",N19+K20,"")</f>
+        <v/>
+      </c>
+      <c r="O20" s="10">
+        <f>IF(H20&lt;&gt;"",O19+J20,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>Start Date</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="C21" s="5" t="inlineStr">
         <is>
           <t>End Date (optional)</t>
         </is>
       </c>
-      <c r="D20" s="5" t="inlineStr">
+      <c r="D21" s="5" t="inlineStr">
         <is>
           <t>Amount ($)</t>
         </is>
       </c>
-      <c r="E20" s="5" t="inlineStr">
+      <c r="E21" s="5" t="inlineStr">
         <is>
           <t>Frequency</t>
         </is>
       </c>
-      <c r="H20" s="12">
-        <f>IF(AND(L19&gt;0.005,H19&lt;&gt;""),18,"")</f>
-        <v/>
-      </c>
-      <c r="I20" s="13">
-        <f>IF(H20&lt;&gt;"",EDATE(StartDate,17),"")</f>
-        <v/>
-      </c>
-      <c r="J20" s="14">
-        <f>IF(H20&lt;&gt;"",ROUND(L19*AnnualRate/12,2),"")</f>
-        <v/>
-      </c>
-      <c r="K20" s="14">
-        <f>IF(H20&lt;&gt;"",MIN(L19,(M20-J20)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I20)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I20))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I20)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I20))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I20))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I20))*(MONTH($B$34:$B$48)=MONTH(I20))*$C$34:$C$48)),"")</f>
-        <v/>
-      </c>
-      <c r="L20" s="14">
-        <f>IF(H20&lt;&gt;"",ROUND(L19-K20,2),"")</f>
-        <v/>
-      </c>
-      <c r="M20" s="10">
-        <f>IF(H20&lt;&gt;"",MIN(MonthlyPmt,L19+J20),"")</f>
-        <v/>
-      </c>
-      <c r="N20" s="10">
-        <f>IF(H20&lt;&gt;"",N19+K20,"")</f>
-        <v/>
-      </c>
-      <c r="O20" s="10">
-        <f>IF(H20&lt;&gt;"",O19+J20,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="B21" s="22" t="n"/>
-      <c r="C21" s="22" t="n"/>
-      <c r="D21" s="23" t="n"/>
-      <c r="E21" s="24" t="n"/>
       <c r="H21" s="7">
         <f>IF(AND(L20&gt;0.005,H20&lt;&gt;""),19,"")</f>
         <v/>
@@ -1766,7 +1759,7 @@
         <v/>
       </c>
       <c r="K21" s="9">
-        <f>IF(H21&lt;&gt;"",MIN(L20,(M21-J21)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I21)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I21))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I21)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I21))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I21))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I21))*(MONTH($B$34:$B$48)=MONTH(I21))*$C$34:$C$48)),"")</f>
+        <f>IF(H21&lt;&gt;"",MIN(L20,(M21-J21)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I21)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I21))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I21)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I21))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I21))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I21))*(MONTH($B$35:$B$49)=MONTH(I21))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L21" s="9">
@@ -1788,7 +1781,7 @@
     </row>
     <row r="22">
       <c r="A22" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B22" s="22" t="n"/>
       <c r="C22" s="22" t="n"/>
@@ -1807,7 +1800,7 @@
         <v/>
       </c>
       <c r="K22" s="14">
-        <f>IF(H22&lt;&gt;"",MIN(L21,(M22-J22)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I22)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I22))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I22)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I22))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I22))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I22))*(MONTH($B$34:$B$48)=MONTH(I22))*$C$34:$C$48)),"")</f>
+        <f>IF(H22&lt;&gt;"",MIN(L21,(M22-J22)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I22)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I22))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I22)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I22))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I22))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I22))*(MONTH($B$35:$B$49)=MONTH(I22))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L22" s="14">
@@ -1829,7 +1822,7 @@
     </row>
     <row r="23">
       <c r="A23" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B23" s="22" t="n"/>
       <c r="C23" s="22" t="n"/>
@@ -1848,7 +1841,7 @@
         <v/>
       </c>
       <c r="K23" s="9">
-        <f>IF(H23&lt;&gt;"",MIN(L22,(M23-J23)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I23)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I23))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I23)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I23))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I23))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I23))*(MONTH($B$34:$B$48)=MONTH(I23))*$C$34:$C$48)),"")</f>
+        <f>IF(H23&lt;&gt;"",MIN(L22,(M23-J23)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I23)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I23))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I23)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I23))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I23))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I23))*(MONTH($B$35:$B$49)=MONTH(I23))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L23" s="9">
@@ -1870,7 +1863,7 @@
     </row>
     <row r="24">
       <c r="A24" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B24" s="22" t="n"/>
       <c r="C24" s="22" t="n"/>
@@ -1889,7 +1882,7 @@
         <v/>
       </c>
       <c r="K24" s="14">
-        <f>IF(H24&lt;&gt;"",MIN(L23,(M24-J24)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I24)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I24))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I24)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I24))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I24))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I24))*(MONTH($B$34:$B$48)=MONTH(I24))*$C$34:$C$48)),"")</f>
+        <f>IF(H24&lt;&gt;"",MIN(L23,(M24-J24)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I24)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I24))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I24)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I24))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I24))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I24))*(MONTH($B$35:$B$49)=MONTH(I24))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L24" s="14">
@@ -1911,7 +1904,7 @@
     </row>
     <row r="25">
       <c r="A25" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B25" s="22" t="n"/>
       <c r="C25" s="22" t="n"/>
@@ -1930,7 +1923,7 @@
         <v/>
       </c>
       <c r="K25" s="9">
-        <f>IF(H25&lt;&gt;"",MIN(L24,(M25-J25)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I25)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I25))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I25)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I25))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I25))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I25))*(MONTH($B$34:$B$48)=MONTH(I25))*$C$34:$C$48)),"")</f>
+        <f>IF(H25&lt;&gt;"",MIN(L24,(M25-J25)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I25)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I25))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I25)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I25))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I25))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I25))*(MONTH($B$35:$B$49)=MONTH(I25))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L25" s="9">
@@ -1952,7 +1945,7 @@
     </row>
     <row r="26">
       <c r="A26" s="7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B26" s="22" t="n"/>
       <c r="C26" s="22" t="n"/>
@@ -1971,7 +1964,7 @@
         <v/>
       </c>
       <c r="K26" s="14">
-        <f>IF(H26&lt;&gt;"",MIN(L25,(M26-J26)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I26)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I26))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I26)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I26))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I26))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I26))*(MONTH($B$34:$B$48)=MONTH(I26))*$C$34:$C$48)),"")</f>
+        <f>IF(H26&lt;&gt;"",MIN(L25,(M26-J26)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I26)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I26))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I26)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I26))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I26))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I26))*(MONTH($B$35:$B$49)=MONTH(I26))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L26" s="14">
@@ -1993,7 +1986,7 @@
     </row>
     <row r="27">
       <c r="A27" s="7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B27" s="22" t="n"/>
       <c r="C27" s="22" t="n"/>
@@ -2012,7 +2005,7 @@
         <v/>
       </c>
       <c r="K27" s="9">
-        <f>IF(H27&lt;&gt;"",MIN(L26,(M27-J27)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I27)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I27))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I27)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I27))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I27))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I27))*(MONTH($B$34:$B$48)=MONTH(I27))*$C$34:$C$48)),"")</f>
+        <f>IF(H27&lt;&gt;"",MIN(L26,(M27-J27)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I27)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I27))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I27)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I27))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I27))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I27))*(MONTH($B$35:$B$49)=MONTH(I27))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L27" s="9">
@@ -2034,7 +2027,7 @@
     </row>
     <row r="28">
       <c r="A28" s="7" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B28" s="22" t="n"/>
       <c r="C28" s="22" t="n"/>
@@ -2053,7 +2046,7 @@
         <v/>
       </c>
       <c r="K28" s="14">
-        <f>IF(H28&lt;&gt;"",MIN(L27,(M28-J28)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I28)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I28))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I28)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I28))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I28))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I28))*(MONTH($B$34:$B$48)=MONTH(I28))*$C$34:$C$48)),"")</f>
+        <f>IF(H28&lt;&gt;"",MIN(L27,(M28-J28)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I28)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I28))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I28)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I28))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I28))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I28))*(MONTH($B$35:$B$49)=MONTH(I28))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L28" s="14">
@@ -2075,7 +2068,7 @@
     </row>
     <row r="29">
       <c r="A29" s="7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B29" s="22" t="n"/>
       <c r="C29" s="22" t="n"/>
@@ -2094,7 +2087,7 @@
         <v/>
       </c>
       <c r="K29" s="9">
-        <f>IF(H29&lt;&gt;"",MIN(L28,(M29-J29)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I29)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I29))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I29)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I29))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I29))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I29))*(MONTH($B$34:$B$48)=MONTH(I29))*$C$34:$C$48)),"")</f>
+        <f>IF(H29&lt;&gt;"",MIN(L28,(M29-J29)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I29)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I29))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I29)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I29))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I29))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I29))*(MONTH($B$35:$B$49)=MONTH(I29))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L29" s="9">
@@ -2116,7 +2109,7 @@
     </row>
     <row r="30">
       <c r="A30" s="7" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B30" s="22" t="n"/>
       <c r="C30" s="22" t="n"/>
@@ -2135,7 +2128,7 @@
         <v/>
       </c>
       <c r="K30" s="14">
-        <f>IF(H30&lt;&gt;"",MIN(L29,(M30-J30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I30)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I30))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I30)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I30))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I30))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I30))*(MONTH($B$34:$B$48)=MONTH(I30))*$C$34:$C$48)),"")</f>
+        <f>IF(H30&lt;&gt;"",MIN(L29,(M30-J30)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I30)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I30))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I30)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I30))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I30))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I30))*(MONTH($B$35:$B$49)=MONTH(I30))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L30" s="14">
@@ -2156,6 +2149,13 @@
       </c>
     </row>
     <row r="31">
+      <c r="A31" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="B31" s="22" t="n"/>
+      <c r="C31" s="22" t="n"/>
+      <c r="D31" s="23" t="n"/>
+      <c r="E31" s="24" t="n"/>
       <c r="H31" s="7">
         <f>IF(AND(L30&gt;0.005,H30&lt;&gt;""),29,"")</f>
         <v/>
@@ -2169,7 +2169,7 @@
         <v/>
       </c>
       <c r="K31" s="9">
-        <f>IF(H31&lt;&gt;"",MIN(L30,(M31-J31)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I31)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I31))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I31)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I31))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I31))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I31))*(MONTH($B$34:$B$48)=MONTH(I31))*$C$34:$C$48)),"")</f>
+        <f>IF(H31&lt;&gt;"",MIN(L30,(M31-J31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I31)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I31))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I31)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I31))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I31))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I31))*(MONTH($B$35:$B$49)=MONTH(I31))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L31" s="9">
@@ -2190,99 +2190,94 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1" t="inlineStr">
+      <c r="H32" s="12">
+        <f>IF(AND(L31&gt;0.005,H31&lt;&gt;""),30,"")</f>
+        <v/>
+      </c>
+      <c r="I32" s="13">
+        <f>IF(H32&lt;&gt;"",EDATE(StartDate,29),"")</f>
+        <v/>
+      </c>
+      <c r="J32" s="14">
+        <f>IF(H32&lt;&gt;"",ROUND(L31*AnnualRate/12,2),"")</f>
+        <v/>
+      </c>
+      <c r="K32" s="14">
+        <f>IF(H32&lt;&gt;"",MIN(L31,(M32-J32)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I32)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I32))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I32)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I32))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I32))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I32))*(MONTH($B$35:$B$49)=MONTH(I32))*$C$35:$C$49)),"")</f>
+        <v/>
+      </c>
+      <c r="L32" s="14">
+        <f>IF(H32&lt;&gt;"",ROUND(L31-K32,2),"")</f>
+        <v/>
+      </c>
+      <c r="M32" s="10">
+        <f>IF(H32&lt;&gt;"",MIN(MonthlyPmt,L31+J32),"")</f>
+        <v/>
+      </c>
+      <c r="N32" s="10">
+        <f>IF(H32&lt;&gt;"",N31+K32,"")</f>
+        <v/>
+      </c>
+      <c r="O32" s="10">
+        <f>IF(H32&lt;&gt;"",O31+J32,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="inlineStr">
         <is>
           <t>ONE-TIME EXTRA PAYMENTS</t>
         </is>
       </c>
-      <c r="H32" s="12">
-        <f>IF(AND(L31&gt;0.005,H31&lt;&gt;""),30,"")</f>
-        <v/>
-      </c>
-      <c r="I32" s="13">
-        <f>IF(H32&lt;&gt;"",EDATE(StartDate,29),"")</f>
-        <v/>
-      </c>
-      <c r="J32" s="14">
-        <f>IF(H32&lt;&gt;"",ROUND(L31*AnnualRate/12,2),"")</f>
-        <v/>
-      </c>
-      <c r="K32" s="14">
-        <f>IF(H32&lt;&gt;"",MIN(L31,(M32-J32)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I32)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I32))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I32)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I32))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I32))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I32))*(MONTH($B$34:$B$48)=MONTH(I32))*$C$34:$C$48)),"")</f>
-        <v/>
-      </c>
-      <c r="L32" s="14">
-        <f>IF(H32&lt;&gt;"",ROUND(L31-K32,2),"")</f>
-        <v/>
-      </c>
-      <c r="M32" s="10">
-        <f>IF(H32&lt;&gt;"",MIN(MonthlyPmt,L31+J32),"")</f>
-        <v/>
-      </c>
-      <c r="N32" s="10">
-        <f>IF(H32&lt;&gt;"",N31+K32,"")</f>
-        <v/>
-      </c>
-      <c r="O32" s="10">
-        <f>IF(H32&lt;&gt;"",O31+J32,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="5" t="inlineStr">
+      <c r="H33" s="7">
+        <f>IF(AND(L32&gt;0.005,H32&lt;&gt;""),31,"")</f>
+        <v/>
+      </c>
+      <c r="I33" s="8">
+        <f>IF(H33&lt;&gt;"",EDATE(StartDate,30),"")</f>
+        <v/>
+      </c>
+      <c r="J33" s="9">
+        <f>IF(H33&lt;&gt;"",ROUND(L32*AnnualRate/12,2),"")</f>
+        <v/>
+      </c>
+      <c r="K33" s="9">
+        <f>IF(H33&lt;&gt;"",MIN(L32,(M33-J33)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I33)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I33))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I33)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I33))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I33))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I33))*(MONTH($B$35:$B$49)=MONTH(I33))*$C$35:$C$49)),"")</f>
+        <v/>
+      </c>
+      <c r="L33" s="9">
+        <f>IF(H33&lt;&gt;"",ROUND(L32-K33,2),"")</f>
+        <v/>
+      </c>
+      <c r="M33" s="10">
+        <f>IF(H33&lt;&gt;"",MIN(MonthlyPmt,L32+J33),"")</f>
+        <v/>
+      </c>
+      <c r="N33" s="10">
+        <f>IF(H33&lt;&gt;"",N32+K33,"")</f>
+        <v/>
+      </c>
+      <c r="O33" s="10">
+        <f>IF(H33&lt;&gt;"",O32+J33,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B33" s="5" t="inlineStr">
+      <c r="B34" s="5" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="C33" s="5" t="inlineStr">
+      <c r="C34" s="5" t="inlineStr">
         <is>
           <t>Amount ($)</t>
         </is>
       </c>
-      <c r="H33" s="7">
-        <f>IF(AND(L32&gt;0.005,H32&lt;&gt;""),31,"")</f>
-        <v/>
-      </c>
-      <c r="I33" s="8">
-        <f>IF(H33&lt;&gt;"",EDATE(StartDate,30),"")</f>
-        <v/>
-      </c>
-      <c r="J33" s="9">
-        <f>IF(H33&lt;&gt;"",ROUND(L32*AnnualRate/12,2),"")</f>
-        <v/>
-      </c>
-      <c r="K33" s="9">
-        <f>IF(H33&lt;&gt;"",MIN(L32,(M33-J33)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I33)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I33))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I33)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I33))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I33))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I33))*(MONTH($B$34:$B$48)=MONTH(I33))*$C$34:$C$48)),"")</f>
-        <v/>
-      </c>
-      <c r="L33" s="9">
-        <f>IF(H33&lt;&gt;"",ROUND(L32-K33,2),"")</f>
-        <v/>
-      </c>
-      <c r="M33" s="10">
-        <f>IF(H33&lt;&gt;"",MIN(MonthlyPmt,L32+J33),"")</f>
-        <v/>
-      </c>
-      <c r="N33" s="10">
-        <f>IF(H33&lt;&gt;"",N32+K33,"")</f>
-        <v/>
-      </c>
-      <c r="O33" s="10">
-        <f>IF(H33&lt;&gt;"",O32+J33,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="B34" s="22" t="n"/>
-      <c r="C34" s="23" t="n"/>
       <c r="H34" s="12">
         <f>IF(AND(L33&gt;0.005,H33&lt;&gt;""),32,"")</f>
         <v/>
@@ -2296,7 +2291,7 @@
         <v/>
       </c>
       <c r="K34" s="14">
-        <f>IF(H34&lt;&gt;"",MIN(L33,(M34-J34)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I34)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I34))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I34)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I34))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I34))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I34))*(MONTH($B$34:$B$48)=MONTH(I34))*$C$34:$C$48)),"")</f>
+        <f>IF(H34&lt;&gt;"",MIN(L33,(M34-J34)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I34)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I34))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I34)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I34))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I34))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I34))*(MONTH($B$35:$B$49)=MONTH(I34))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L34" s="14">
@@ -2318,7 +2313,7 @@
     </row>
     <row r="35">
       <c r="A35" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B35" s="22" t="n"/>
       <c r="C35" s="23" t="n"/>
@@ -2335,7 +2330,7 @@
         <v/>
       </c>
       <c r="K35" s="9">
-        <f>IF(H35&lt;&gt;"",MIN(L34,(M35-J35)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I35)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I35))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I35)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I35))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I35))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I35))*(MONTH($B$34:$B$48)=MONTH(I35))*$C$34:$C$48)),"")</f>
+        <f>IF(H35&lt;&gt;"",MIN(L34,(M35-J35)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I35)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I35))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I35)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I35))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I35))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I35))*(MONTH($B$35:$B$49)=MONTH(I35))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L35" s="9">
@@ -2357,7 +2352,7 @@
     </row>
     <row r="36">
       <c r="A36" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B36" s="22" t="n"/>
       <c r="C36" s="23" t="n"/>
@@ -2374,7 +2369,7 @@
         <v/>
       </c>
       <c r="K36" s="14">
-        <f>IF(H36&lt;&gt;"",MIN(L35,(M36-J36)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I36)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I36))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I36)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I36))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I36))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I36))*(MONTH($B$34:$B$48)=MONTH(I36))*$C$34:$C$48)),"")</f>
+        <f>IF(H36&lt;&gt;"",MIN(L35,(M36-J36)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I36)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I36))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I36)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I36))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I36))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I36))*(MONTH($B$35:$B$49)=MONTH(I36))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L36" s="14">
@@ -2396,7 +2391,7 @@
     </row>
     <row r="37">
       <c r="A37" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B37" s="22" t="n"/>
       <c r="C37" s="23" t="n"/>
@@ -2413,7 +2408,7 @@
         <v/>
       </c>
       <c r="K37" s="9">
-        <f>IF(H37&lt;&gt;"",MIN(L36,(M37-J37)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I37)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I37))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I37)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I37))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I37))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I37))*(MONTH($B$34:$B$48)=MONTH(I37))*$C$34:$C$48)),"")</f>
+        <f>IF(H37&lt;&gt;"",MIN(L36,(M37-J37)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I37)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I37))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I37)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I37))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I37))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I37))*(MONTH($B$35:$B$49)=MONTH(I37))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L37" s="9">
@@ -2435,7 +2430,7 @@
     </row>
     <row r="38">
       <c r="A38" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B38" s="22" t="n"/>
       <c r="C38" s="23" t="n"/>
@@ -2452,7 +2447,7 @@
         <v/>
       </c>
       <c r="K38" s="14">
-        <f>IF(H38&lt;&gt;"",MIN(L37,(M38-J38)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I38)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I38))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I38)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I38))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I38))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I38))*(MONTH($B$34:$B$48)=MONTH(I38))*$C$34:$C$48)),"")</f>
+        <f>IF(H38&lt;&gt;"",MIN(L37,(M38-J38)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I38)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I38))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I38)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I38))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I38))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I38))*(MONTH($B$35:$B$49)=MONTH(I38))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L38" s="14">
@@ -2474,7 +2469,7 @@
     </row>
     <row r="39">
       <c r="A39" s="7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B39" s="22" t="n"/>
       <c r="C39" s="23" t="n"/>
@@ -2491,7 +2486,7 @@
         <v/>
       </c>
       <c r="K39" s="9">
-        <f>IF(H39&lt;&gt;"",MIN(L38,(M39-J39)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I39)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I39))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I39)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I39))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I39))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I39))*(MONTH($B$34:$B$48)=MONTH(I39))*$C$34:$C$48)),"")</f>
+        <f>IF(H39&lt;&gt;"",MIN(L38,(M39-J39)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I39)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I39))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I39)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I39))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I39))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I39))*(MONTH($B$35:$B$49)=MONTH(I39))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L39" s="9">
@@ -2513,7 +2508,7 @@
     </row>
     <row r="40">
       <c r="A40" s="7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B40" s="22" t="n"/>
       <c r="C40" s="23" t="n"/>
@@ -2530,7 +2525,7 @@
         <v/>
       </c>
       <c r="K40" s="14">
-        <f>IF(H40&lt;&gt;"",MIN(L39,(M40-J40)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I40)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I40))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I40)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I40))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I40))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I40))*(MONTH($B$34:$B$48)=MONTH(I40))*$C$34:$C$48)),"")</f>
+        <f>IF(H40&lt;&gt;"",MIN(L39,(M40-J40)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I40)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I40))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I40)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I40))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I40))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I40))*(MONTH($B$35:$B$49)=MONTH(I40))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L40" s="14">
@@ -2552,7 +2547,7 @@
     </row>
     <row r="41">
       <c r="A41" s="7" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B41" s="22" t="n"/>
       <c r="C41" s="23" t="n"/>
@@ -2569,7 +2564,7 @@
         <v/>
       </c>
       <c r="K41" s="9">
-        <f>IF(H41&lt;&gt;"",MIN(L40,(M41-J41)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I41)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I41))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I41)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I41))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I41))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I41))*(MONTH($B$34:$B$48)=MONTH(I41))*$C$34:$C$48)),"")</f>
+        <f>IF(H41&lt;&gt;"",MIN(L40,(M41-J41)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I41)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I41))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I41)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I41))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I41))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I41))*(MONTH($B$35:$B$49)=MONTH(I41))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L41" s="9">
@@ -2591,7 +2586,7 @@
     </row>
     <row r="42">
       <c r="A42" s="7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B42" s="22" t="n"/>
       <c r="C42" s="23" t="n"/>
@@ -2608,7 +2603,7 @@
         <v/>
       </c>
       <c r="K42" s="14">
-        <f>IF(H42&lt;&gt;"",MIN(L41,(M42-J42)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I42)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I42))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I42)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I42))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I42))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I42))*(MONTH($B$34:$B$48)=MONTH(I42))*$C$34:$C$48)),"")</f>
+        <f>IF(H42&lt;&gt;"",MIN(L41,(M42-J42)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I42)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I42))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I42)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I42))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I42))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I42))*(MONTH($B$35:$B$49)=MONTH(I42))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L42" s="14">
@@ -2630,7 +2625,7 @@
     </row>
     <row r="43">
       <c r="A43" s="7" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B43" s="22" t="n"/>
       <c r="C43" s="23" t="n"/>
@@ -2647,7 +2642,7 @@
         <v/>
       </c>
       <c r="K43" s="9">
-        <f>IF(H43&lt;&gt;"",MIN(L42,(M43-J43)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I43)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I43))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I43)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I43))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I43))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I43))*(MONTH($B$34:$B$48)=MONTH(I43))*$C$34:$C$48)),"")</f>
+        <f>IF(H43&lt;&gt;"",MIN(L42,(M43-J43)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I43)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I43))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I43)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I43))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I43))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I43))*(MONTH($B$35:$B$49)=MONTH(I43))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L43" s="9">
@@ -2669,7 +2664,7 @@
     </row>
     <row r="44">
       <c r="A44" s="7" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B44" s="22" t="n"/>
       <c r="C44" s="23" t="n"/>
@@ -2686,7 +2681,7 @@
         <v/>
       </c>
       <c r="K44" s="14">
-        <f>IF(H44&lt;&gt;"",MIN(L43,(M44-J44)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I44)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I44))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I44)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I44))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I44))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I44))*(MONTH($B$34:$B$48)=MONTH(I44))*$C$34:$C$48)),"")</f>
+        <f>IF(H44&lt;&gt;"",MIN(L43,(M44-J44)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I44)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I44))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I44)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I44))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I44))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I44))*(MONTH($B$35:$B$49)=MONTH(I44))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L44" s="14">
@@ -2708,7 +2703,7 @@
     </row>
     <row r="45">
       <c r="A45" s="7" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B45" s="22" t="n"/>
       <c r="C45" s="23" t="n"/>
@@ -2725,7 +2720,7 @@
         <v/>
       </c>
       <c r="K45" s="9">
-        <f>IF(H45&lt;&gt;"",MIN(L44,(M45-J45)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I45)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I45))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I45)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I45))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I45))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I45))*(MONTH($B$34:$B$48)=MONTH(I45))*$C$34:$C$48)),"")</f>
+        <f>IF(H45&lt;&gt;"",MIN(L44,(M45-J45)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I45)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I45))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I45)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I45))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I45))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I45))*(MONTH($B$35:$B$49)=MONTH(I45))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L45" s="9">
@@ -2747,7 +2742,7 @@
     </row>
     <row r="46">
       <c r="A46" s="7" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B46" s="22" t="n"/>
       <c r="C46" s="23" t="n"/>
@@ -2764,7 +2759,7 @@
         <v/>
       </c>
       <c r="K46" s="14">
-        <f>IF(H46&lt;&gt;"",MIN(L45,(M46-J46)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I46)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I46))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I46)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I46))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I46))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I46))*(MONTH($B$34:$B$48)=MONTH(I46))*$C$34:$C$48)),"")</f>
+        <f>IF(H46&lt;&gt;"",MIN(L45,(M46-J46)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I46)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I46))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I46)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I46))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I46))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I46))*(MONTH($B$35:$B$49)=MONTH(I46))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L46" s="14">
@@ -2786,7 +2781,7 @@
     </row>
     <row r="47">
       <c r="A47" s="7" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B47" s="22" t="n"/>
       <c r="C47" s="23" t="n"/>
@@ -2803,7 +2798,7 @@
         <v/>
       </c>
       <c r="K47" s="9">
-        <f>IF(H47&lt;&gt;"",MIN(L46,(M47-J47)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I47)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I47))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I47)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I47))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I47))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I47))*(MONTH($B$34:$B$48)=MONTH(I47))*$C$34:$C$48)),"")</f>
+        <f>IF(H47&lt;&gt;"",MIN(L46,(M47-J47)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I47)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I47))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I47)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I47))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I47))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I47))*(MONTH($B$35:$B$49)=MONTH(I47))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L47" s="9">
@@ -2825,7 +2820,7 @@
     </row>
     <row r="48">
       <c r="A48" s="7" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B48" s="22" t="n"/>
       <c r="C48" s="23" t="n"/>
@@ -2842,7 +2837,7 @@
         <v/>
       </c>
       <c r="K48" s="14">
-        <f>IF(H48&lt;&gt;"",MIN(L47,(M48-J48)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I48)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I48))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I48)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I48))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I48))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I48))*(MONTH($B$34:$B$48)=MONTH(I48))*$C$34:$C$48)),"")</f>
+        <f>IF(H48&lt;&gt;"",MIN(L47,(M48-J48)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I48)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I48))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I48)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I48))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I48))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I48))*(MONTH($B$35:$B$49)=MONTH(I48))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L48" s="14">
@@ -2863,6 +2858,11 @@
       </c>
     </row>
     <row r="49">
+      <c r="A49" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="B49" s="22" t="n"/>
+      <c r="C49" s="23" t="n"/>
       <c r="H49" s="7">
         <f>IF(AND(L48&gt;0.005,H48&lt;&gt;""),47,"")</f>
         <v/>
@@ -2876,7 +2876,7 @@
         <v/>
       </c>
       <c r="K49" s="9">
-        <f>IF(H49&lt;&gt;"",MIN(L48,(M49-J49)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I49)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I49))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I49)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I49))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I49))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I49))*(MONTH($B$34:$B$48)=MONTH(I49))*$C$34:$C$48)),"")</f>
+        <f>IF(H49&lt;&gt;"",MIN(L48,(M49-J49)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I49)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I49))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I49)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I49))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I49))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I49))*(MONTH($B$35:$B$49)=MONTH(I49))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L49" s="9">
@@ -2910,7 +2910,7 @@
         <v/>
       </c>
       <c r="K50" s="14">
-        <f>IF(H50&lt;&gt;"",MIN(L49,(M50-J50)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I50)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I50))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I50)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I50))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I50))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I50))*(MONTH($B$34:$B$48)=MONTH(I50))*$C$34:$C$48)),"")</f>
+        <f>IF(H50&lt;&gt;"",MIN(L49,(M50-J50)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I50)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I50))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I50)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I50))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I50))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I50))*(MONTH($B$35:$B$49)=MONTH(I50))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L50" s="14">
@@ -2944,7 +2944,7 @@
         <v/>
       </c>
       <c r="K51" s="9">
-        <f>IF(H51&lt;&gt;"",MIN(L50,(M51-J51)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I51)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I51))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I51)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I51))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I51))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I51))*(MONTH($B$34:$B$48)=MONTH(I51))*$C$34:$C$48)),"")</f>
+        <f>IF(H51&lt;&gt;"",MIN(L50,(M51-J51)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I51)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I51))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I51)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I51))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I51))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I51))*(MONTH($B$35:$B$49)=MONTH(I51))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L51" s="9">
@@ -2978,7 +2978,7 @@
         <v/>
       </c>
       <c r="K52" s="14">
-        <f>IF(H52&lt;&gt;"",MIN(L51,(M52-J52)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I52)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I52))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I52)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I52))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I52))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I52))*(MONTH($B$34:$B$48)=MONTH(I52))*$C$34:$C$48)),"")</f>
+        <f>IF(H52&lt;&gt;"",MIN(L51,(M52-J52)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I52)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I52))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I52)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I52))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I52))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I52))*(MONTH($B$35:$B$49)=MONTH(I52))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L52" s="14">
@@ -3012,7 +3012,7 @@
         <v/>
       </c>
       <c r="K53" s="9">
-        <f>IF(H53&lt;&gt;"",MIN(L52,(M53-J53)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I53)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I53))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I53)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I53))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I53))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I53))*(MONTH($B$34:$B$48)=MONTH(I53))*$C$34:$C$48)),"")</f>
+        <f>IF(H53&lt;&gt;"",MIN(L52,(M53-J53)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I53)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I53))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I53)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I53))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I53))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I53))*(MONTH($B$35:$B$49)=MONTH(I53))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L53" s="9">
@@ -3046,7 +3046,7 @@
         <v/>
       </c>
       <c r="K54" s="14">
-        <f>IF(H54&lt;&gt;"",MIN(L53,(M54-J54)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I54)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I54))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I54)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I54))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I54))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I54))*(MONTH($B$34:$B$48)=MONTH(I54))*$C$34:$C$48)),"")</f>
+        <f>IF(H54&lt;&gt;"",MIN(L53,(M54-J54)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I54)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I54))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I54)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I54))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I54))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I54))*(MONTH($B$35:$B$49)=MONTH(I54))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L54" s="14">
@@ -3080,7 +3080,7 @@
         <v/>
       </c>
       <c r="K55" s="9">
-        <f>IF(H55&lt;&gt;"",MIN(L54,(M55-J55)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I55)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I55))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I55)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I55))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I55))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I55))*(MONTH($B$34:$B$48)=MONTH(I55))*$C$34:$C$48)),"")</f>
+        <f>IF(H55&lt;&gt;"",MIN(L54,(M55-J55)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I55)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I55))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I55)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I55))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I55))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I55))*(MONTH($B$35:$B$49)=MONTH(I55))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L55" s="9">
@@ -3114,7 +3114,7 @@
         <v/>
       </c>
       <c r="K56" s="14">
-        <f>IF(H56&lt;&gt;"",MIN(L55,(M56-J56)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I56)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I56))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I56)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I56))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I56))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I56))*(MONTH($B$34:$B$48)=MONTH(I56))*$C$34:$C$48)),"")</f>
+        <f>IF(H56&lt;&gt;"",MIN(L55,(M56-J56)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I56)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I56))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I56)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I56))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I56))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I56))*(MONTH($B$35:$B$49)=MONTH(I56))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L56" s="14">
@@ -3148,7 +3148,7 @@
         <v/>
       </c>
       <c r="K57" s="9">
-        <f>IF(H57&lt;&gt;"",MIN(L56,(M57-J57)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I57)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I57))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I57)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I57))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I57))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I57))*(MONTH($B$34:$B$48)=MONTH(I57))*$C$34:$C$48)),"")</f>
+        <f>IF(H57&lt;&gt;"",MIN(L56,(M57-J57)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I57)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I57))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I57)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I57))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I57))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I57))*(MONTH($B$35:$B$49)=MONTH(I57))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L57" s="9">
@@ -3182,7 +3182,7 @@
         <v/>
       </c>
       <c r="K58" s="14">
-        <f>IF(H58&lt;&gt;"",MIN(L57,(M58-J58)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I58)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I58))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I58)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I58))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I58))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I58))*(MONTH($B$34:$B$48)=MONTH(I58))*$C$34:$C$48)),"")</f>
+        <f>IF(H58&lt;&gt;"",MIN(L57,(M58-J58)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I58)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I58))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I58)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I58))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I58))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I58))*(MONTH($B$35:$B$49)=MONTH(I58))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L58" s="14">
@@ -3216,7 +3216,7 @@
         <v/>
       </c>
       <c r="K59" s="9">
-        <f>IF(H59&lt;&gt;"",MIN(L58,(M59-J59)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I59)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I59))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I59)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I59))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I59))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I59))*(MONTH($B$34:$B$48)=MONTH(I59))*$C$34:$C$48)),"")</f>
+        <f>IF(H59&lt;&gt;"",MIN(L58,(M59-J59)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I59)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I59))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I59)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I59))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I59))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I59))*(MONTH($B$35:$B$49)=MONTH(I59))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L59" s="9">
@@ -3250,7 +3250,7 @@
         <v/>
       </c>
       <c r="K60" s="14">
-        <f>IF(H60&lt;&gt;"",MIN(L59,(M60-J60)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I60)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I60))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I60)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I60))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I60))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I60))*(MONTH($B$34:$B$48)=MONTH(I60))*$C$34:$C$48)),"")</f>
+        <f>IF(H60&lt;&gt;"",MIN(L59,(M60-J60)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I60)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I60))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I60)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I60))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I60))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I60))*(MONTH($B$35:$B$49)=MONTH(I60))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L60" s="14">
@@ -3284,7 +3284,7 @@
         <v/>
       </c>
       <c r="K61" s="9">
-        <f>IF(H61&lt;&gt;"",MIN(L60,(M61-J61)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I61)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I61))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I61)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I61))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I61))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I61))*(MONTH($B$34:$B$48)=MONTH(I61))*$C$34:$C$48)),"")</f>
+        <f>IF(H61&lt;&gt;"",MIN(L60,(M61-J61)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I61)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I61))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I61)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I61))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I61))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I61))*(MONTH($B$35:$B$49)=MONTH(I61))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L61" s="9">
@@ -3318,7 +3318,7 @@
         <v/>
       </c>
       <c r="K62" s="14">
-        <f>IF(H62&lt;&gt;"",MIN(L61,(M62-J62)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I62)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I62))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I62)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I62))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I62))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I62))*(MONTH($B$34:$B$48)=MONTH(I62))*$C$34:$C$48)),"")</f>
+        <f>IF(H62&lt;&gt;"",MIN(L61,(M62-J62)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I62)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I62))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I62)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I62))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I62))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I62))*(MONTH($B$35:$B$49)=MONTH(I62))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L62" s="14">
@@ -3352,7 +3352,7 @@
         <v/>
       </c>
       <c r="K63" s="9">
-        <f>IF(H63&lt;&gt;"",MIN(L62,(M63-J63)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I63)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I63))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I63)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I63))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I63))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I63))*(MONTH($B$34:$B$48)=MONTH(I63))*$C$34:$C$48)),"")</f>
+        <f>IF(H63&lt;&gt;"",MIN(L62,(M63-J63)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I63)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I63))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I63)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I63))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I63))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I63))*(MONTH($B$35:$B$49)=MONTH(I63))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L63" s="9">
@@ -3386,7 +3386,7 @@
         <v/>
       </c>
       <c r="K64" s="14">
-        <f>IF(H64&lt;&gt;"",MIN(L63,(M64-J64)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I64)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I64))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I64)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I64))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I64))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I64))*(MONTH($B$34:$B$48)=MONTH(I64))*$C$34:$C$48)),"")</f>
+        <f>IF(H64&lt;&gt;"",MIN(L63,(M64-J64)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I64)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I64))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I64)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I64))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I64))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I64))*(MONTH($B$35:$B$49)=MONTH(I64))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L64" s="14">
@@ -3420,7 +3420,7 @@
         <v/>
       </c>
       <c r="K65" s="9">
-        <f>IF(H65&lt;&gt;"",MIN(L64,(M65-J65)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I65)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I65))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I65)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I65))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I65))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I65))*(MONTH($B$34:$B$48)=MONTH(I65))*$C$34:$C$48)),"")</f>
+        <f>IF(H65&lt;&gt;"",MIN(L64,(M65-J65)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I65)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I65))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I65)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I65))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I65))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I65))*(MONTH($B$35:$B$49)=MONTH(I65))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L65" s="9">
@@ -3454,7 +3454,7 @@
         <v/>
       </c>
       <c r="K66" s="14">
-        <f>IF(H66&lt;&gt;"",MIN(L65,(M66-J66)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I66)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I66))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I66)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I66))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I66))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I66))*(MONTH($B$34:$B$48)=MONTH(I66))*$C$34:$C$48)),"")</f>
+        <f>IF(H66&lt;&gt;"",MIN(L65,(M66-J66)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I66)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I66))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I66)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I66))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I66))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I66))*(MONTH($B$35:$B$49)=MONTH(I66))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L66" s="14">
@@ -3488,7 +3488,7 @@
         <v/>
       </c>
       <c r="K67" s="9">
-        <f>IF(H67&lt;&gt;"",MIN(L66,(M67-J67)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I67)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I67))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I67)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I67))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I67))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I67))*(MONTH($B$34:$B$48)=MONTH(I67))*$C$34:$C$48)),"")</f>
+        <f>IF(H67&lt;&gt;"",MIN(L66,(M67-J67)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I67)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I67))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I67)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I67))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I67))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I67))*(MONTH($B$35:$B$49)=MONTH(I67))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L67" s="9">
@@ -3522,7 +3522,7 @@
         <v/>
       </c>
       <c r="K68" s="14">
-        <f>IF(H68&lt;&gt;"",MIN(L67,(M68-J68)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I68)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I68))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I68)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I68))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I68))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I68))*(MONTH($B$34:$B$48)=MONTH(I68))*$C$34:$C$48)),"")</f>
+        <f>IF(H68&lt;&gt;"",MIN(L67,(M68-J68)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I68)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I68))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I68)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I68))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I68))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I68))*(MONTH($B$35:$B$49)=MONTH(I68))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L68" s="14">
@@ -3556,7 +3556,7 @@
         <v/>
       </c>
       <c r="K69" s="9">
-        <f>IF(H69&lt;&gt;"",MIN(L68,(M69-J69)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I69)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I69))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I69)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I69))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I69))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I69))*(MONTH($B$34:$B$48)=MONTH(I69))*$C$34:$C$48)),"")</f>
+        <f>IF(H69&lt;&gt;"",MIN(L68,(M69-J69)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I69)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I69))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I69)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I69))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I69))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I69))*(MONTH($B$35:$B$49)=MONTH(I69))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L69" s="9">
@@ -3590,7 +3590,7 @@
         <v/>
       </c>
       <c r="K70" s="14">
-        <f>IF(H70&lt;&gt;"",MIN(L69,(M70-J70)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I70)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I70))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I70)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I70))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I70))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I70))*(MONTH($B$34:$B$48)=MONTH(I70))*$C$34:$C$48)),"")</f>
+        <f>IF(H70&lt;&gt;"",MIN(L69,(M70-J70)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I70)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I70))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I70)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I70))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I70))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I70))*(MONTH($B$35:$B$49)=MONTH(I70))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L70" s="14">
@@ -3624,7 +3624,7 @@
         <v/>
       </c>
       <c r="K71" s="9">
-        <f>IF(H71&lt;&gt;"",MIN(L70,(M71-J71)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I71)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I71))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I71)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I71))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I71))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I71))*(MONTH($B$34:$B$48)=MONTH(I71))*$C$34:$C$48)),"")</f>
+        <f>IF(H71&lt;&gt;"",MIN(L70,(M71-J71)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I71)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I71))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I71)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I71))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I71))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I71))*(MONTH($B$35:$B$49)=MONTH(I71))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L71" s="9">
@@ -3658,7 +3658,7 @@
         <v/>
       </c>
       <c r="K72" s="14">
-        <f>IF(H72&lt;&gt;"",MIN(L71,(M72-J72)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I72)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I72))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I72)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I72))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I72))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I72))*(MONTH($B$34:$B$48)=MONTH(I72))*$C$34:$C$48)),"")</f>
+        <f>IF(H72&lt;&gt;"",MIN(L71,(M72-J72)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I72)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I72))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I72)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I72))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I72))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I72))*(MONTH($B$35:$B$49)=MONTH(I72))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L72" s="14">
@@ -3692,7 +3692,7 @@
         <v/>
       </c>
       <c r="K73" s="9">
-        <f>IF(H73&lt;&gt;"",MIN(L72,(M73-J73)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I73)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I73))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I73)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I73))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I73))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I73))*(MONTH($B$34:$B$48)=MONTH(I73))*$C$34:$C$48)),"")</f>
+        <f>IF(H73&lt;&gt;"",MIN(L72,(M73-J73)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I73)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I73))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I73)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I73))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I73))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I73))*(MONTH($B$35:$B$49)=MONTH(I73))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L73" s="9">
@@ -3726,7 +3726,7 @@
         <v/>
       </c>
       <c r="K74" s="14">
-        <f>IF(H74&lt;&gt;"",MIN(L73,(M74-J74)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I74)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I74))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I74)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I74))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I74))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I74))*(MONTH($B$34:$B$48)=MONTH(I74))*$C$34:$C$48)),"")</f>
+        <f>IF(H74&lt;&gt;"",MIN(L73,(M74-J74)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I74)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I74))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I74)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I74))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I74))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I74))*(MONTH($B$35:$B$49)=MONTH(I74))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L74" s="14">
@@ -3760,7 +3760,7 @@
         <v/>
       </c>
       <c r="K75" s="9">
-        <f>IF(H75&lt;&gt;"",MIN(L74,(M75-J75)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I75)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I75))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I75)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I75))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I75))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I75))*(MONTH($B$34:$B$48)=MONTH(I75))*$C$34:$C$48)),"")</f>
+        <f>IF(H75&lt;&gt;"",MIN(L74,(M75-J75)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I75)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I75))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I75)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I75))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I75))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I75))*(MONTH($B$35:$B$49)=MONTH(I75))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L75" s="9">
@@ -3794,7 +3794,7 @@
         <v/>
       </c>
       <c r="K76" s="14">
-        <f>IF(H76&lt;&gt;"",MIN(L75,(M76-J76)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I76)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I76))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I76)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I76))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I76))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I76))*(MONTH($B$34:$B$48)=MONTH(I76))*$C$34:$C$48)),"")</f>
+        <f>IF(H76&lt;&gt;"",MIN(L75,(M76-J76)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I76)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I76))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I76)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I76))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I76))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I76))*(MONTH($B$35:$B$49)=MONTH(I76))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L76" s="14">
@@ -3828,7 +3828,7 @@
         <v/>
       </c>
       <c r="K77" s="9">
-        <f>IF(H77&lt;&gt;"",MIN(L76,(M77-J77)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I77)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I77))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I77)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I77))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I77))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I77))*(MONTH($B$34:$B$48)=MONTH(I77))*$C$34:$C$48)),"")</f>
+        <f>IF(H77&lt;&gt;"",MIN(L76,(M77-J77)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I77)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I77))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I77)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I77))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I77))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I77))*(MONTH($B$35:$B$49)=MONTH(I77))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L77" s="9">
@@ -3862,7 +3862,7 @@
         <v/>
       </c>
       <c r="K78" s="14">
-        <f>IF(H78&lt;&gt;"",MIN(L77,(M78-J78)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I78)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I78))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I78)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I78))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I78))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I78))*(MONTH($B$34:$B$48)=MONTH(I78))*$C$34:$C$48)),"")</f>
+        <f>IF(H78&lt;&gt;"",MIN(L77,(M78-J78)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I78)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I78))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I78)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I78))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I78))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I78))*(MONTH($B$35:$B$49)=MONTH(I78))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L78" s="14">
@@ -3896,7 +3896,7 @@
         <v/>
       </c>
       <c r="K79" s="9">
-        <f>IF(H79&lt;&gt;"",MIN(L78,(M79-J79)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I79)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I79))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I79)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I79))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I79))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I79))*(MONTH($B$34:$B$48)=MONTH(I79))*$C$34:$C$48)),"")</f>
+        <f>IF(H79&lt;&gt;"",MIN(L78,(M79-J79)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I79)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I79))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I79)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I79))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I79))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I79))*(MONTH($B$35:$B$49)=MONTH(I79))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L79" s="9">
@@ -3930,7 +3930,7 @@
         <v/>
       </c>
       <c r="K80" s="14">
-        <f>IF(H80&lt;&gt;"",MIN(L79,(M80-J80)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I80)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I80))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I80)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I80))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I80))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I80))*(MONTH($B$34:$B$48)=MONTH(I80))*$C$34:$C$48)),"")</f>
+        <f>IF(H80&lt;&gt;"",MIN(L79,(M80-J80)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I80)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I80))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I80)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I80))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I80))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I80))*(MONTH($B$35:$B$49)=MONTH(I80))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L80" s="14">
@@ -3964,7 +3964,7 @@
         <v/>
       </c>
       <c r="K81" s="9">
-        <f>IF(H81&lt;&gt;"",MIN(L80,(M81-J81)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I81)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I81))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I81)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I81))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I81))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I81))*(MONTH($B$34:$B$48)=MONTH(I81))*$C$34:$C$48)),"")</f>
+        <f>IF(H81&lt;&gt;"",MIN(L80,(M81-J81)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I81)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I81))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I81)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I81))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I81))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I81))*(MONTH($B$35:$B$49)=MONTH(I81))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L81" s="9">
@@ -3998,7 +3998,7 @@
         <v/>
       </c>
       <c r="K82" s="14">
-        <f>IF(H82&lt;&gt;"",MIN(L81,(M82-J82)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I82)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I82))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I82)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I82))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I82))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I82))*(MONTH($B$34:$B$48)=MONTH(I82))*$C$34:$C$48)),"")</f>
+        <f>IF(H82&lt;&gt;"",MIN(L81,(M82-J82)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I82)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I82))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I82)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I82))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I82))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I82))*(MONTH($B$35:$B$49)=MONTH(I82))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L82" s="14">
@@ -4032,7 +4032,7 @@
         <v/>
       </c>
       <c r="K83" s="9">
-        <f>IF(H83&lt;&gt;"",MIN(L82,(M83-J83)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I83)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I83))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I83)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I83))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I83))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I83))*(MONTH($B$34:$B$48)=MONTH(I83))*$C$34:$C$48)),"")</f>
+        <f>IF(H83&lt;&gt;"",MIN(L82,(M83-J83)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I83)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I83))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I83)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I83))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I83))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I83))*(MONTH($B$35:$B$49)=MONTH(I83))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L83" s="9">
@@ -4066,7 +4066,7 @@
         <v/>
       </c>
       <c r="K84" s="14">
-        <f>IF(H84&lt;&gt;"",MIN(L83,(M84-J84)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I84)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I84))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I84)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I84))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I84))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I84))*(MONTH($B$34:$B$48)=MONTH(I84))*$C$34:$C$48)),"")</f>
+        <f>IF(H84&lt;&gt;"",MIN(L83,(M84-J84)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I84)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I84))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I84)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I84))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I84))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I84))*(MONTH($B$35:$B$49)=MONTH(I84))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L84" s="14">
@@ -4100,7 +4100,7 @@
         <v/>
       </c>
       <c r="K85" s="9">
-        <f>IF(H85&lt;&gt;"",MIN(L84,(M85-J85)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I85)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I85))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I85)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I85))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I85))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I85))*(MONTH($B$34:$B$48)=MONTH(I85))*$C$34:$C$48)),"")</f>
+        <f>IF(H85&lt;&gt;"",MIN(L84,(M85-J85)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I85)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I85))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I85)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I85))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I85))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I85))*(MONTH($B$35:$B$49)=MONTH(I85))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L85" s="9">
@@ -4134,7 +4134,7 @@
         <v/>
       </c>
       <c r="K86" s="14">
-        <f>IF(H86&lt;&gt;"",MIN(L85,(M86-J86)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I86)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I86))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I86)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I86))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I86))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I86))*(MONTH($B$34:$B$48)=MONTH(I86))*$C$34:$C$48)),"")</f>
+        <f>IF(H86&lt;&gt;"",MIN(L85,(M86-J86)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I86)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I86))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I86)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I86))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I86))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I86))*(MONTH($B$35:$B$49)=MONTH(I86))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L86" s="14">
@@ -4168,7 +4168,7 @@
         <v/>
       </c>
       <c r="K87" s="9">
-        <f>IF(H87&lt;&gt;"",MIN(L86,(M87-J87)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I87)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I87))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I87)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I87))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I87))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I87))*(MONTH($B$34:$B$48)=MONTH(I87))*$C$34:$C$48)),"")</f>
+        <f>IF(H87&lt;&gt;"",MIN(L86,(M87-J87)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I87)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I87))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I87)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I87))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I87))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I87))*(MONTH($B$35:$B$49)=MONTH(I87))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L87" s="9">
@@ -4202,7 +4202,7 @@
         <v/>
       </c>
       <c r="K88" s="14">
-        <f>IF(H88&lt;&gt;"",MIN(L87,(M88-J88)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I88)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I88))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I88)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I88))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I88))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I88))*(MONTH($B$34:$B$48)=MONTH(I88))*$C$34:$C$48)),"")</f>
+        <f>IF(H88&lt;&gt;"",MIN(L87,(M88-J88)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I88)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I88))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I88)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I88))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I88))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I88))*(MONTH($B$35:$B$49)=MONTH(I88))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L88" s="14">
@@ -4236,7 +4236,7 @@
         <v/>
       </c>
       <c r="K89" s="9">
-        <f>IF(H89&lt;&gt;"",MIN(L88,(M89-J89)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I89)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I89))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I89)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I89))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I89))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I89))*(MONTH($B$34:$B$48)=MONTH(I89))*$C$34:$C$48)),"")</f>
+        <f>IF(H89&lt;&gt;"",MIN(L88,(M89-J89)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I89)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I89))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I89)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I89))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I89))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I89))*(MONTH($B$35:$B$49)=MONTH(I89))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L89" s="9">
@@ -4270,7 +4270,7 @@
         <v/>
       </c>
       <c r="K90" s="14">
-        <f>IF(H90&lt;&gt;"",MIN(L89,(M90-J90)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I90)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I90))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I90)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I90))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I90))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I90))*(MONTH($B$34:$B$48)=MONTH(I90))*$C$34:$C$48)),"")</f>
+        <f>IF(H90&lt;&gt;"",MIN(L89,(M90-J90)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I90)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I90))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I90)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I90))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I90))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I90))*(MONTH($B$35:$B$49)=MONTH(I90))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L90" s="14">
@@ -4304,7 +4304,7 @@
         <v/>
       </c>
       <c r="K91" s="9">
-        <f>IF(H91&lt;&gt;"",MIN(L90,(M91-J91)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I91)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I91))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I91)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I91))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I91))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I91))*(MONTH($B$34:$B$48)=MONTH(I91))*$C$34:$C$48)),"")</f>
+        <f>IF(H91&lt;&gt;"",MIN(L90,(M91-J91)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I91)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I91))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I91)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I91))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I91))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I91))*(MONTH($B$35:$B$49)=MONTH(I91))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L91" s="9">
@@ -4338,7 +4338,7 @@
         <v/>
       </c>
       <c r="K92" s="14">
-        <f>IF(H92&lt;&gt;"",MIN(L91,(M92-J92)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I92)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I92))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I92)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I92))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I92))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I92))*(MONTH($B$34:$B$48)=MONTH(I92))*$C$34:$C$48)),"")</f>
+        <f>IF(H92&lt;&gt;"",MIN(L91,(M92-J92)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I92)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I92))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I92)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I92))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I92))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I92))*(MONTH($B$35:$B$49)=MONTH(I92))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L92" s="14">
@@ -4372,7 +4372,7 @@
         <v/>
       </c>
       <c r="K93" s="9">
-        <f>IF(H93&lt;&gt;"",MIN(L92,(M93-J93)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I93)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I93))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I93)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I93))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I93))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I93))*(MONTH($B$34:$B$48)=MONTH(I93))*$C$34:$C$48)),"")</f>
+        <f>IF(H93&lt;&gt;"",MIN(L92,(M93-J93)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I93)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I93))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I93)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I93))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I93))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I93))*(MONTH($B$35:$B$49)=MONTH(I93))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L93" s="9">
@@ -4406,7 +4406,7 @@
         <v/>
       </c>
       <c r="K94" s="14">
-        <f>IF(H94&lt;&gt;"",MIN(L93,(M94-J94)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I94)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I94))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I94)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I94))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I94))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I94))*(MONTH($B$34:$B$48)=MONTH(I94))*$C$34:$C$48)),"")</f>
+        <f>IF(H94&lt;&gt;"",MIN(L93,(M94-J94)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I94)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I94))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I94)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I94))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I94))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I94))*(MONTH($B$35:$B$49)=MONTH(I94))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L94" s="14">
@@ -4440,7 +4440,7 @@
         <v/>
       </c>
       <c r="K95" s="9">
-        <f>IF(H95&lt;&gt;"",MIN(L94,(M95-J95)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I95)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I95))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I95)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I95))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I95))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I95))*(MONTH($B$34:$B$48)=MONTH(I95))*$C$34:$C$48)),"")</f>
+        <f>IF(H95&lt;&gt;"",MIN(L94,(M95-J95)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I95)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I95))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I95)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I95))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I95))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I95))*(MONTH($B$35:$B$49)=MONTH(I95))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L95" s="9">
@@ -4474,7 +4474,7 @@
         <v/>
       </c>
       <c r="K96" s="14">
-        <f>IF(H96&lt;&gt;"",MIN(L95,(M96-J96)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I96)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I96))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I96)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I96))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I96))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I96))*(MONTH($B$34:$B$48)=MONTH(I96))*$C$34:$C$48)),"")</f>
+        <f>IF(H96&lt;&gt;"",MIN(L95,(M96-J96)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I96)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I96))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I96)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I96))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I96))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I96))*(MONTH($B$35:$B$49)=MONTH(I96))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L96" s="14">
@@ -4508,7 +4508,7 @@
         <v/>
       </c>
       <c r="K97" s="9">
-        <f>IF(H97&lt;&gt;"",MIN(L96,(M97-J97)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I97)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I97))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I97)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I97))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I97))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I97))*(MONTH($B$34:$B$48)=MONTH(I97))*$C$34:$C$48)),"")</f>
+        <f>IF(H97&lt;&gt;"",MIN(L96,(M97-J97)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I97)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I97))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I97)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I97))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I97))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I97))*(MONTH($B$35:$B$49)=MONTH(I97))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L97" s="9">
@@ -4542,7 +4542,7 @@
         <v/>
       </c>
       <c r="K98" s="14">
-        <f>IF(H98&lt;&gt;"",MIN(L97,(M98-J98)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I98)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I98))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I98)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I98))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I98))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I98))*(MONTH($B$34:$B$48)=MONTH(I98))*$C$34:$C$48)),"")</f>
+        <f>IF(H98&lt;&gt;"",MIN(L97,(M98-J98)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I98)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I98))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I98)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I98))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I98))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I98))*(MONTH($B$35:$B$49)=MONTH(I98))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L98" s="14">
@@ -4576,7 +4576,7 @@
         <v/>
       </c>
       <c r="K99" s="9">
-        <f>IF(H99&lt;&gt;"",MIN(L98,(M99-J99)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I99)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I99))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I99)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I99))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I99))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I99))*(MONTH($B$34:$B$48)=MONTH(I99))*$C$34:$C$48)),"")</f>
+        <f>IF(H99&lt;&gt;"",MIN(L98,(M99-J99)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I99)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I99))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I99)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I99))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I99))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I99))*(MONTH($B$35:$B$49)=MONTH(I99))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L99" s="9">
@@ -4610,7 +4610,7 @@
         <v/>
       </c>
       <c r="K100" s="14">
-        <f>IF(H100&lt;&gt;"",MIN(L99,(M100-J100)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I100)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I100))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I100)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I100))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I100))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I100))*(MONTH($B$34:$B$48)=MONTH(I100))*$C$34:$C$48)),"")</f>
+        <f>IF(H100&lt;&gt;"",MIN(L99,(M100-J100)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I100)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I100))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I100)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I100))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I100))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I100))*(MONTH($B$35:$B$49)=MONTH(I100))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L100" s="14">
@@ -4644,7 +4644,7 @@
         <v/>
       </c>
       <c r="K101" s="9">
-        <f>IF(H101&lt;&gt;"",MIN(L100,(M101-J101)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I101)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I101))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I101)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I101))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I101))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I101))*(MONTH($B$34:$B$48)=MONTH(I101))*$C$34:$C$48)),"")</f>
+        <f>IF(H101&lt;&gt;"",MIN(L100,(M101-J101)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I101)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I101))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I101)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I101))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I101))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I101))*(MONTH($B$35:$B$49)=MONTH(I101))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L101" s="9">
@@ -4678,7 +4678,7 @@
         <v/>
       </c>
       <c r="K102" s="14">
-        <f>IF(H102&lt;&gt;"",MIN(L101,(M102-J102)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I102)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I102))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I102)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I102))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I102))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I102))*(MONTH($B$34:$B$48)=MONTH(I102))*$C$34:$C$48)),"")</f>
+        <f>IF(H102&lt;&gt;"",MIN(L101,(M102-J102)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I102)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I102))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I102)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I102))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I102))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I102))*(MONTH($B$35:$B$49)=MONTH(I102))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L102" s="14">
@@ -4712,7 +4712,7 @@
         <v/>
       </c>
       <c r="K103" s="9">
-        <f>IF(H103&lt;&gt;"",MIN(L102,(M103-J103)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I103)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I103))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I103)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I103))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I103))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I103))*(MONTH($B$34:$B$48)=MONTH(I103))*$C$34:$C$48)),"")</f>
+        <f>IF(H103&lt;&gt;"",MIN(L102,(M103-J103)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I103)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I103))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I103)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I103))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I103))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I103))*(MONTH($B$35:$B$49)=MONTH(I103))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L103" s="9">
@@ -4746,7 +4746,7 @@
         <v/>
       </c>
       <c r="K104" s="14">
-        <f>IF(H104&lt;&gt;"",MIN(L103,(M104-J104)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I104)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I104))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I104)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I104))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I104))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I104))*(MONTH($B$34:$B$48)=MONTH(I104))*$C$34:$C$48)),"")</f>
+        <f>IF(H104&lt;&gt;"",MIN(L103,(M104-J104)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I104)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I104))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I104)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I104))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I104))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I104))*(MONTH($B$35:$B$49)=MONTH(I104))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L104" s="14">
@@ -4780,7 +4780,7 @@
         <v/>
       </c>
       <c r="K105" s="9">
-        <f>IF(H105&lt;&gt;"",MIN(L104,(M105-J105)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I105)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I105))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I105)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I105))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I105))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I105))*(MONTH($B$34:$B$48)=MONTH(I105))*$C$34:$C$48)),"")</f>
+        <f>IF(H105&lt;&gt;"",MIN(L104,(M105-J105)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I105)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I105))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I105)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I105))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I105))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I105))*(MONTH($B$35:$B$49)=MONTH(I105))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L105" s="9">
@@ -4814,7 +4814,7 @@
         <v/>
       </c>
       <c r="K106" s="14">
-        <f>IF(H106&lt;&gt;"",MIN(L105,(M106-J106)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I106)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I106))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I106)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I106))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I106))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I106))*(MONTH($B$34:$B$48)=MONTH(I106))*$C$34:$C$48)),"")</f>
+        <f>IF(H106&lt;&gt;"",MIN(L105,(M106-J106)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I106)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I106))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I106)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I106))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I106))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I106))*(MONTH($B$35:$B$49)=MONTH(I106))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L106" s="14">
@@ -4848,7 +4848,7 @@
         <v/>
       </c>
       <c r="K107" s="9">
-        <f>IF(H107&lt;&gt;"",MIN(L106,(M107-J107)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I107)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I107))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I107)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I107))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I107))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I107))*(MONTH($B$34:$B$48)=MONTH(I107))*$C$34:$C$48)),"")</f>
+        <f>IF(H107&lt;&gt;"",MIN(L106,(M107-J107)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I107)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I107))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I107)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I107))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I107))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I107))*(MONTH($B$35:$B$49)=MONTH(I107))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L107" s="9">
@@ -4882,7 +4882,7 @@
         <v/>
       </c>
       <c r="K108" s="14">
-        <f>IF(H108&lt;&gt;"",MIN(L107,(M108-J108)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I108)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I108))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I108)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I108))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I108))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I108))*(MONTH($B$34:$B$48)=MONTH(I108))*$C$34:$C$48)),"")</f>
+        <f>IF(H108&lt;&gt;"",MIN(L107,(M108-J108)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I108)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I108))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I108)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I108))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I108))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I108))*(MONTH($B$35:$B$49)=MONTH(I108))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L108" s="14">
@@ -4916,7 +4916,7 @@
         <v/>
       </c>
       <c r="K109" s="9">
-        <f>IF(H109&lt;&gt;"",MIN(L108,(M109-J109)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I109)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I109))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I109)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I109))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I109))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I109))*(MONTH($B$34:$B$48)=MONTH(I109))*$C$34:$C$48)),"")</f>
+        <f>IF(H109&lt;&gt;"",MIN(L108,(M109-J109)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I109)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I109))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I109)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I109))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I109))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I109))*(MONTH($B$35:$B$49)=MONTH(I109))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L109" s="9">
@@ -4950,7 +4950,7 @@
         <v/>
       </c>
       <c r="K110" s="14">
-        <f>IF(H110&lt;&gt;"",MIN(L109,(M110-J110)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I110)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I110))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I110)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I110))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I110))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I110))*(MONTH($B$34:$B$48)=MONTH(I110))*$C$34:$C$48)),"")</f>
+        <f>IF(H110&lt;&gt;"",MIN(L109,(M110-J110)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I110)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I110))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I110)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I110))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I110))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I110))*(MONTH($B$35:$B$49)=MONTH(I110))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L110" s="14">
@@ -4984,7 +4984,7 @@
         <v/>
       </c>
       <c r="K111" s="9">
-        <f>IF(H111&lt;&gt;"",MIN(L110,(M111-J111)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I111)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I111))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I111)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I111))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I111))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I111))*(MONTH($B$34:$B$48)=MONTH(I111))*$C$34:$C$48)),"")</f>
+        <f>IF(H111&lt;&gt;"",MIN(L110,(M111-J111)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I111)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I111))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I111)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I111))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I111))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I111))*(MONTH($B$35:$B$49)=MONTH(I111))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L111" s="9">
@@ -5018,7 +5018,7 @@
         <v/>
       </c>
       <c r="K112" s="14">
-        <f>IF(H112&lt;&gt;"",MIN(L111,(M112-J112)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I112)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I112))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I112)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I112))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I112))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I112))*(MONTH($B$34:$B$48)=MONTH(I112))*$C$34:$C$48)),"")</f>
+        <f>IF(H112&lt;&gt;"",MIN(L111,(M112-J112)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I112)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I112))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I112)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I112))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I112))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I112))*(MONTH($B$35:$B$49)=MONTH(I112))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L112" s="14">
@@ -5052,7 +5052,7 @@
         <v/>
       </c>
       <c r="K113" s="9">
-        <f>IF(H113&lt;&gt;"",MIN(L112,(M113-J113)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I113)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I113))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I113)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I113))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I113))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I113))*(MONTH($B$34:$B$48)=MONTH(I113))*$C$34:$C$48)),"")</f>
+        <f>IF(H113&lt;&gt;"",MIN(L112,(M113-J113)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I113)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I113))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I113)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I113))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I113))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I113))*(MONTH($B$35:$B$49)=MONTH(I113))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L113" s="9">
@@ -5086,7 +5086,7 @@
         <v/>
       </c>
       <c r="K114" s="14">
-        <f>IF(H114&lt;&gt;"",MIN(L113,(M114-J114)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I114)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I114))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I114)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I114))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I114))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I114))*(MONTH($B$34:$B$48)=MONTH(I114))*$C$34:$C$48)),"")</f>
+        <f>IF(H114&lt;&gt;"",MIN(L113,(M114-J114)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I114)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I114))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I114)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I114))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I114))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I114))*(MONTH($B$35:$B$49)=MONTH(I114))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L114" s="14">
@@ -5120,7 +5120,7 @@
         <v/>
       </c>
       <c r="K115" s="9">
-        <f>IF(H115&lt;&gt;"",MIN(L114,(M115-J115)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I115)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I115))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I115)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I115))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I115))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I115))*(MONTH($B$34:$B$48)=MONTH(I115))*$C$34:$C$48)),"")</f>
+        <f>IF(H115&lt;&gt;"",MIN(L114,(M115-J115)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I115)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I115))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I115)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I115))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I115))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I115))*(MONTH($B$35:$B$49)=MONTH(I115))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L115" s="9">
@@ -5154,7 +5154,7 @@
         <v/>
       </c>
       <c r="K116" s="14">
-        <f>IF(H116&lt;&gt;"",MIN(L115,(M116-J116)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I116)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I116))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I116)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I116))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I116))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I116))*(MONTH($B$34:$B$48)=MONTH(I116))*$C$34:$C$48)),"")</f>
+        <f>IF(H116&lt;&gt;"",MIN(L115,(M116-J116)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I116)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I116))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I116)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I116))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I116))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I116))*(MONTH($B$35:$B$49)=MONTH(I116))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L116" s="14">
@@ -5188,7 +5188,7 @@
         <v/>
       </c>
       <c r="K117" s="9">
-        <f>IF(H117&lt;&gt;"",MIN(L116,(M117-J117)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I117)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I117))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I117)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I117))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I117))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I117))*(MONTH($B$34:$B$48)=MONTH(I117))*$C$34:$C$48)),"")</f>
+        <f>IF(H117&lt;&gt;"",MIN(L116,(M117-J117)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I117)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I117))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I117)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I117))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I117))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I117))*(MONTH($B$35:$B$49)=MONTH(I117))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L117" s="9">
@@ -5222,7 +5222,7 @@
         <v/>
       </c>
       <c r="K118" s="14">
-        <f>IF(H118&lt;&gt;"",MIN(L117,(M118-J118)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I118)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I118))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I118)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I118))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I118))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I118))*(MONTH($B$34:$B$48)=MONTH(I118))*$C$34:$C$48)),"")</f>
+        <f>IF(H118&lt;&gt;"",MIN(L117,(M118-J118)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I118)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I118))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I118)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I118))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I118))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I118))*(MONTH($B$35:$B$49)=MONTH(I118))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L118" s="14">
@@ -5256,7 +5256,7 @@
         <v/>
       </c>
       <c r="K119" s="9">
-        <f>IF(H119&lt;&gt;"",MIN(L118,(M119-J119)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I119)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I119))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I119)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I119))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I119))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I119))*(MONTH($B$34:$B$48)=MONTH(I119))*$C$34:$C$48)),"")</f>
+        <f>IF(H119&lt;&gt;"",MIN(L118,(M119-J119)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I119)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I119))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I119)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I119))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I119))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I119))*(MONTH($B$35:$B$49)=MONTH(I119))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L119" s="9">
@@ -5290,7 +5290,7 @@
         <v/>
       </c>
       <c r="K120" s="14">
-        <f>IF(H120&lt;&gt;"",MIN(L119,(M120-J120)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I120)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I120))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I120)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I120))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I120))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I120))*(MONTH($B$34:$B$48)=MONTH(I120))*$C$34:$C$48)),"")</f>
+        <f>IF(H120&lt;&gt;"",MIN(L119,(M120-J120)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I120)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I120))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I120)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I120))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I120))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I120))*(MONTH($B$35:$B$49)=MONTH(I120))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L120" s="14">
@@ -5324,7 +5324,7 @@
         <v/>
       </c>
       <c r="K121" s="9">
-        <f>IF(H121&lt;&gt;"",MIN(L120,(M121-J121)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I121)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I121))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I121)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I121))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I121))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I121))*(MONTH($B$34:$B$48)=MONTH(I121))*$C$34:$C$48)),"")</f>
+        <f>IF(H121&lt;&gt;"",MIN(L120,(M121-J121)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I121)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I121))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I121)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I121))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I121))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I121))*(MONTH($B$35:$B$49)=MONTH(I121))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L121" s="9">
@@ -5358,7 +5358,7 @@
         <v/>
       </c>
       <c r="K122" s="14">
-        <f>IF(H122&lt;&gt;"",MIN(L121,(M122-J122)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I122)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I122))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I122)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I122))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I122))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I122))*(MONTH($B$34:$B$48)=MONTH(I122))*$C$34:$C$48)),"")</f>
+        <f>IF(H122&lt;&gt;"",MIN(L121,(M122-J122)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I122)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I122))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I122)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I122))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I122))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I122))*(MONTH($B$35:$B$49)=MONTH(I122))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L122" s="14">
@@ -5392,7 +5392,7 @@
         <v/>
       </c>
       <c r="K123" s="9">
-        <f>IF(H123&lt;&gt;"",MIN(L122,(M123-J123)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I123)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I123))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I123)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I123))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I123))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I123))*(MONTH($B$34:$B$48)=MONTH(I123))*$C$34:$C$48)),"")</f>
+        <f>IF(H123&lt;&gt;"",MIN(L122,(M123-J123)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I123)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I123))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I123)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I123))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I123))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I123))*(MONTH($B$35:$B$49)=MONTH(I123))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L123" s="9">
@@ -5426,7 +5426,7 @@
         <v/>
       </c>
       <c r="K124" s="14">
-        <f>IF(H124&lt;&gt;"",MIN(L123,(M124-J124)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I124)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I124))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I124)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I124))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I124))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I124))*(MONTH($B$34:$B$48)=MONTH(I124))*$C$34:$C$48)),"")</f>
+        <f>IF(H124&lt;&gt;"",MIN(L123,(M124-J124)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I124)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I124))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I124)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I124))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I124))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I124))*(MONTH($B$35:$B$49)=MONTH(I124))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L124" s="14">
@@ -5460,7 +5460,7 @@
         <v/>
       </c>
       <c r="K125" s="9">
-        <f>IF(H125&lt;&gt;"",MIN(L124,(M125-J125)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I125)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I125))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I125)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I125))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I125))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I125))*(MONTH($B$34:$B$48)=MONTH(I125))*$C$34:$C$48)),"")</f>
+        <f>IF(H125&lt;&gt;"",MIN(L124,(M125-J125)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I125)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I125))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I125)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I125))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I125))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I125))*(MONTH($B$35:$B$49)=MONTH(I125))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L125" s="9">
@@ -5494,7 +5494,7 @@
         <v/>
       </c>
       <c r="K126" s="14">
-        <f>IF(H126&lt;&gt;"",MIN(L125,(M126-J126)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I126)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I126))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I126)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I126))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I126))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I126))*(MONTH($B$34:$B$48)=MONTH(I126))*$C$34:$C$48)),"")</f>
+        <f>IF(H126&lt;&gt;"",MIN(L125,(M126-J126)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I126)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I126))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I126)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I126))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I126))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I126))*(MONTH($B$35:$B$49)=MONTH(I126))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L126" s="14">
@@ -5528,7 +5528,7 @@
         <v/>
       </c>
       <c r="K127" s="9">
-        <f>IF(H127&lt;&gt;"",MIN(L126,(M127-J127)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I127)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I127))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I127)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I127))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I127))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I127))*(MONTH($B$34:$B$48)=MONTH(I127))*$C$34:$C$48)),"")</f>
+        <f>IF(H127&lt;&gt;"",MIN(L126,(M127-J127)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I127)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I127))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I127)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I127))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I127))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I127))*(MONTH($B$35:$B$49)=MONTH(I127))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L127" s="9">
@@ -5562,7 +5562,7 @@
         <v/>
       </c>
       <c r="K128" s="14">
-        <f>IF(H128&lt;&gt;"",MIN(L127,(M128-J128)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I128)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I128))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I128)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I128))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I128))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I128))*(MONTH($B$34:$B$48)=MONTH(I128))*$C$34:$C$48)),"")</f>
+        <f>IF(H128&lt;&gt;"",MIN(L127,(M128-J128)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I128)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I128))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I128)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I128))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I128))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I128))*(MONTH($B$35:$B$49)=MONTH(I128))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L128" s="14">
@@ -5596,7 +5596,7 @@
         <v/>
       </c>
       <c r="K129" s="9">
-        <f>IF(H129&lt;&gt;"",MIN(L128,(M129-J129)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I129)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I129))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I129)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I129))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I129))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I129))*(MONTH($B$34:$B$48)=MONTH(I129))*$C$34:$C$48)),"")</f>
+        <f>IF(H129&lt;&gt;"",MIN(L128,(M129-J129)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I129)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I129))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I129)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I129))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I129))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I129))*(MONTH($B$35:$B$49)=MONTH(I129))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L129" s="9">
@@ -5630,7 +5630,7 @@
         <v/>
       </c>
       <c r="K130" s="14">
-        <f>IF(H130&lt;&gt;"",MIN(L129,(M130-J130)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I130)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I130))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I130)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I130))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I130))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I130))*(MONTH($B$34:$B$48)=MONTH(I130))*$C$34:$C$48)),"")</f>
+        <f>IF(H130&lt;&gt;"",MIN(L129,(M130-J130)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I130)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I130))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I130)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I130))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I130))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I130))*(MONTH($B$35:$B$49)=MONTH(I130))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L130" s="14">
@@ -5664,7 +5664,7 @@
         <v/>
       </c>
       <c r="K131" s="9">
-        <f>IF(H131&lt;&gt;"",MIN(L130,(M131-J131)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I131)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I131))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I131)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I131))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I131))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I131))*(MONTH($B$34:$B$48)=MONTH(I131))*$C$34:$C$48)),"")</f>
+        <f>IF(H131&lt;&gt;"",MIN(L130,(M131-J131)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I131)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I131))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I131)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I131))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I131))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I131))*(MONTH($B$35:$B$49)=MONTH(I131))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L131" s="9">
@@ -5698,7 +5698,7 @@
         <v/>
       </c>
       <c r="K132" s="14">
-        <f>IF(H132&lt;&gt;"",MIN(L131,(M132-J132)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I132)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I132))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I132)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I132))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I132))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I132))*(MONTH($B$34:$B$48)=MONTH(I132))*$C$34:$C$48)),"")</f>
+        <f>IF(H132&lt;&gt;"",MIN(L131,(M132-J132)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I132)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I132))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I132)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I132))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I132))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I132))*(MONTH($B$35:$B$49)=MONTH(I132))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L132" s="14">
@@ -5732,7 +5732,7 @@
         <v/>
       </c>
       <c r="K133" s="9">
-        <f>IF(H133&lt;&gt;"",MIN(L132,(M133-J133)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I133)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I133))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I133)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I133))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I133))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I133))*(MONTH($B$34:$B$48)=MONTH(I133))*$C$34:$C$48)),"")</f>
+        <f>IF(H133&lt;&gt;"",MIN(L132,(M133-J133)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I133)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I133))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I133)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I133))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I133))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I133))*(MONTH($B$35:$B$49)=MONTH(I133))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L133" s="9">
@@ -5766,7 +5766,7 @@
         <v/>
       </c>
       <c r="K134" s="14">
-        <f>IF(H134&lt;&gt;"",MIN(L133,(M134-J134)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I134)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I134))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I134)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I134))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I134))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I134))*(MONTH($B$34:$B$48)=MONTH(I134))*$C$34:$C$48)),"")</f>
+        <f>IF(H134&lt;&gt;"",MIN(L133,(M134-J134)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I134)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I134))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I134)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I134))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I134))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I134))*(MONTH($B$35:$B$49)=MONTH(I134))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L134" s="14">
@@ -5800,7 +5800,7 @@
         <v/>
       </c>
       <c r="K135" s="9">
-        <f>IF(H135&lt;&gt;"",MIN(L134,(M135-J135)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I135)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I135))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I135)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I135))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I135))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I135))*(MONTH($B$34:$B$48)=MONTH(I135))*$C$34:$C$48)),"")</f>
+        <f>IF(H135&lt;&gt;"",MIN(L134,(M135-J135)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I135)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I135))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I135)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I135))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I135))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I135))*(MONTH($B$35:$B$49)=MONTH(I135))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L135" s="9">
@@ -5834,7 +5834,7 @@
         <v/>
       </c>
       <c r="K136" s="14">
-        <f>IF(H136&lt;&gt;"",MIN(L135,(M136-J136)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I136)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I136))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I136)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I136))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I136))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I136))*(MONTH($B$34:$B$48)=MONTH(I136))*$C$34:$C$48)),"")</f>
+        <f>IF(H136&lt;&gt;"",MIN(L135,(M136-J136)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I136)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I136))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I136)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I136))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I136))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I136))*(MONTH($B$35:$B$49)=MONTH(I136))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L136" s="14">
@@ -5868,7 +5868,7 @@
         <v/>
       </c>
       <c r="K137" s="9">
-        <f>IF(H137&lt;&gt;"",MIN(L136,(M137-J137)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I137)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I137))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I137)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I137))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I137))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I137))*(MONTH($B$34:$B$48)=MONTH(I137))*$C$34:$C$48)),"")</f>
+        <f>IF(H137&lt;&gt;"",MIN(L136,(M137-J137)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I137)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I137))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I137)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I137))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I137))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I137))*(MONTH($B$35:$B$49)=MONTH(I137))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L137" s="9">
@@ -5902,7 +5902,7 @@
         <v/>
       </c>
       <c r="K138" s="14">
-        <f>IF(H138&lt;&gt;"",MIN(L137,(M138-J138)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I138)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I138))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I138)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I138))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I138))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I138))*(MONTH($B$34:$B$48)=MONTH(I138))*$C$34:$C$48)),"")</f>
+        <f>IF(H138&lt;&gt;"",MIN(L137,(M138-J138)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I138)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I138))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I138)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I138))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I138))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I138))*(MONTH($B$35:$B$49)=MONTH(I138))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L138" s="14">
@@ -5936,7 +5936,7 @@
         <v/>
       </c>
       <c r="K139" s="9">
-        <f>IF(H139&lt;&gt;"",MIN(L138,(M139-J139)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I139)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I139))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I139)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I139))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I139))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I139))*(MONTH($B$34:$B$48)=MONTH(I139))*$C$34:$C$48)),"")</f>
+        <f>IF(H139&lt;&gt;"",MIN(L138,(M139-J139)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I139)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I139))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I139)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I139))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I139))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I139))*(MONTH($B$35:$B$49)=MONTH(I139))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L139" s="9">
@@ -5970,7 +5970,7 @@
         <v/>
       </c>
       <c r="K140" s="14">
-        <f>IF(H140&lt;&gt;"",MIN(L139,(M140-J140)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I140)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I140))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I140)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I140))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I140))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I140))*(MONTH($B$34:$B$48)=MONTH(I140))*$C$34:$C$48)),"")</f>
+        <f>IF(H140&lt;&gt;"",MIN(L139,(M140-J140)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I140)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I140))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I140)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I140))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I140))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I140))*(MONTH($B$35:$B$49)=MONTH(I140))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L140" s="14">
@@ -6004,7 +6004,7 @@
         <v/>
       </c>
       <c r="K141" s="9">
-        <f>IF(H141&lt;&gt;"",MIN(L140,(M141-J141)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I141)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I141))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I141)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I141))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I141))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I141))*(MONTH($B$34:$B$48)=MONTH(I141))*$C$34:$C$48)),"")</f>
+        <f>IF(H141&lt;&gt;"",MIN(L140,(M141-J141)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I141)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I141))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I141)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I141))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I141))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I141))*(MONTH($B$35:$B$49)=MONTH(I141))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L141" s="9">
@@ -6038,7 +6038,7 @@
         <v/>
       </c>
       <c r="K142" s="14">
-        <f>IF(H142&lt;&gt;"",MIN(L141,(M142-J142)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I142)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I142))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I142)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I142))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I142))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I142))*(MONTH($B$34:$B$48)=MONTH(I142))*$C$34:$C$48)),"")</f>
+        <f>IF(H142&lt;&gt;"",MIN(L141,(M142-J142)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I142)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I142))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I142)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I142))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I142))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I142))*(MONTH($B$35:$B$49)=MONTH(I142))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L142" s="14">
@@ -6072,7 +6072,7 @@
         <v/>
       </c>
       <c r="K143" s="9">
-        <f>IF(H143&lt;&gt;"",MIN(L142,(M143-J143)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I143)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I143))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I143)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I143))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I143))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I143))*(MONTH($B$34:$B$48)=MONTH(I143))*$C$34:$C$48)),"")</f>
+        <f>IF(H143&lt;&gt;"",MIN(L142,(M143-J143)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I143)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I143))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I143)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I143))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I143))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I143))*(MONTH($B$35:$B$49)=MONTH(I143))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L143" s="9">
@@ -6106,7 +6106,7 @@
         <v/>
       </c>
       <c r="K144" s="14">
-        <f>IF(H144&lt;&gt;"",MIN(L143,(M144-J144)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I144)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I144))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I144)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I144))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I144))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I144))*(MONTH($B$34:$B$48)=MONTH(I144))*$C$34:$C$48)),"")</f>
+        <f>IF(H144&lt;&gt;"",MIN(L143,(M144-J144)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I144)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I144))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I144)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I144))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I144))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I144))*(MONTH($B$35:$B$49)=MONTH(I144))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L144" s="14">
@@ -6140,7 +6140,7 @@
         <v/>
       </c>
       <c r="K145" s="9">
-        <f>IF(H145&lt;&gt;"",MIN(L144,(M145-J145)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I145)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I145))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I145)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I145))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I145))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I145))*(MONTH($B$34:$B$48)=MONTH(I145))*$C$34:$C$48)),"")</f>
+        <f>IF(H145&lt;&gt;"",MIN(L144,(M145-J145)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I145)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I145))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I145)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I145))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I145))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I145))*(MONTH($B$35:$B$49)=MONTH(I145))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L145" s="9">
@@ -6174,7 +6174,7 @@
         <v/>
       </c>
       <c r="K146" s="14">
-        <f>IF(H146&lt;&gt;"",MIN(L145,(M146-J146)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I146)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I146))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I146)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I146))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I146))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I146))*(MONTH($B$34:$B$48)=MONTH(I146))*$C$34:$C$48)),"")</f>
+        <f>IF(H146&lt;&gt;"",MIN(L145,(M146-J146)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I146)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I146))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I146)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I146))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I146))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I146))*(MONTH($B$35:$B$49)=MONTH(I146))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L146" s="14">
@@ -6208,7 +6208,7 @@
         <v/>
       </c>
       <c r="K147" s="9">
-        <f>IF(H147&lt;&gt;"",MIN(L146,(M147-J147)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I147)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I147))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I147)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I147))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I147))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I147))*(MONTH($B$34:$B$48)=MONTH(I147))*$C$34:$C$48)),"")</f>
+        <f>IF(H147&lt;&gt;"",MIN(L146,(M147-J147)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I147)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I147))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I147)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I147))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I147))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I147))*(MONTH($B$35:$B$49)=MONTH(I147))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L147" s="9">
@@ -6242,7 +6242,7 @@
         <v/>
       </c>
       <c r="K148" s="14">
-        <f>IF(H148&lt;&gt;"",MIN(L147,(M148-J148)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I148)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I148))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I148)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I148))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I148))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I148))*(MONTH($B$34:$B$48)=MONTH(I148))*$C$34:$C$48)),"")</f>
+        <f>IF(H148&lt;&gt;"",MIN(L147,(M148-J148)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I148)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I148))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I148)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I148))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I148))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I148))*(MONTH($B$35:$B$49)=MONTH(I148))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L148" s="14">
@@ -6276,7 +6276,7 @@
         <v/>
       </c>
       <c r="K149" s="9">
-        <f>IF(H149&lt;&gt;"",MIN(L148,(M149-J149)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I149)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I149))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I149)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I149))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I149))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I149))*(MONTH($B$34:$B$48)=MONTH(I149))*$C$34:$C$48)),"")</f>
+        <f>IF(H149&lt;&gt;"",MIN(L148,(M149-J149)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I149)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I149))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I149)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I149))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I149))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I149))*(MONTH($B$35:$B$49)=MONTH(I149))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L149" s="9">
@@ -6310,7 +6310,7 @@
         <v/>
       </c>
       <c r="K150" s="14">
-        <f>IF(H150&lt;&gt;"",MIN(L149,(M150-J150)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I150)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I150))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I150)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I150))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I150))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I150))*(MONTH($B$34:$B$48)=MONTH(I150))*$C$34:$C$48)),"")</f>
+        <f>IF(H150&lt;&gt;"",MIN(L149,(M150-J150)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I150)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I150))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I150)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I150))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I150))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I150))*(MONTH($B$35:$B$49)=MONTH(I150))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L150" s="14">
@@ -6344,7 +6344,7 @@
         <v/>
       </c>
       <c r="K151" s="9">
-        <f>IF(H151&lt;&gt;"",MIN(L150,(M151-J151)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I151)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I151))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I151)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I151))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I151))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I151))*(MONTH($B$34:$B$48)=MONTH(I151))*$C$34:$C$48)),"")</f>
+        <f>IF(H151&lt;&gt;"",MIN(L150,(M151-J151)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I151)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I151))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I151)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I151))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I151))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I151))*(MONTH($B$35:$B$49)=MONTH(I151))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L151" s="9">
@@ -6378,7 +6378,7 @@
         <v/>
       </c>
       <c r="K152" s="14">
-        <f>IF(H152&lt;&gt;"",MIN(L151,(M152-J152)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I152)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I152))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I152)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I152))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I152))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I152))*(MONTH($B$34:$B$48)=MONTH(I152))*$C$34:$C$48)),"")</f>
+        <f>IF(H152&lt;&gt;"",MIN(L151,(M152-J152)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I152)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I152))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I152)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I152))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I152))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I152))*(MONTH($B$35:$B$49)=MONTH(I152))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L152" s="14">
@@ -6412,7 +6412,7 @@
         <v/>
       </c>
       <c r="K153" s="9">
-        <f>IF(H153&lt;&gt;"",MIN(L152,(M153-J153)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I153)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I153))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I153)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I153))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I153))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I153))*(MONTH($B$34:$B$48)=MONTH(I153))*$C$34:$C$48)),"")</f>
+        <f>IF(H153&lt;&gt;"",MIN(L152,(M153-J153)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I153)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I153))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I153)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I153))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I153))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I153))*(MONTH($B$35:$B$49)=MONTH(I153))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L153" s="9">
@@ -6446,7 +6446,7 @@
         <v/>
       </c>
       <c r="K154" s="14">
-        <f>IF(H154&lt;&gt;"",MIN(L153,(M154-J154)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I154)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I154))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I154)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I154))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I154))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I154))*(MONTH($B$34:$B$48)=MONTH(I154))*$C$34:$C$48)),"")</f>
+        <f>IF(H154&lt;&gt;"",MIN(L153,(M154-J154)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I154)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I154))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I154)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I154))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I154))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I154))*(MONTH($B$35:$B$49)=MONTH(I154))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L154" s="14">
@@ -6480,7 +6480,7 @@
         <v/>
       </c>
       <c r="K155" s="9">
-        <f>IF(H155&lt;&gt;"",MIN(L154,(M155-J155)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I155)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I155))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I155)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I155))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I155))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I155))*(MONTH($B$34:$B$48)=MONTH(I155))*$C$34:$C$48)),"")</f>
+        <f>IF(H155&lt;&gt;"",MIN(L154,(M155-J155)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I155)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I155))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I155)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I155))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I155))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I155))*(MONTH($B$35:$B$49)=MONTH(I155))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L155" s="9">
@@ -6514,7 +6514,7 @@
         <v/>
       </c>
       <c r="K156" s="14">
-        <f>IF(H156&lt;&gt;"",MIN(L155,(M156-J156)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I156)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I156))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I156)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I156))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I156))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I156))*(MONTH($B$34:$B$48)=MONTH(I156))*$C$34:$C$48)),"")</f>
+        <f>IF(H156&lt;&gt;"",MIN(L155,(M156-J156)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I156)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I156))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I156)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I156))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I156))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I156))*(MONTH($B$35:$B$49)=MONTH(I156))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L156" s="14">
@@ -6548,7 +6548,7 @@
         <v/>
       </c>
       <c r="K157" s="9">
-        <f>IF(H157&lt;&gt;"",MIN(L156,(M157-J157)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I157)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I157))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I157)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I157))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I157))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I157))*(MONTH($B$34:$B$48)=MONTH(I157))*$C$34:$C$48)),"")</f>
+        <f>IF(H157&lt;&gt;"",MIN(L156,(M157-J157)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I157)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I157))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I157)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I157))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I157))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I157))*(MONTH($B$35:$B$49)=MONTH(I157))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L157" s="9">
@@ -6582,7 +6582,7 @@
         <v/>
       </c>
       <c r="K158" s="14">
-        <f>IF(H158&lt;&gt;"",MIN(L157,(M158-J158)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I158)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I158))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I158)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I158))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I158))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I158))*(MONTH($B$34:$B$48)=MONTH(I158))*$C$34:$C$48)),"")</f>
+        <f>IF(H158&lt;&gt;"",MIN(L157,(M158-J158)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I158)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I158))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I158)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I158))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I158))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I158))*(MONTH($B$35:$B$49)=MONTH(I158))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L158" s="14">
@@ -6616,7 +6616,7 @@
         <v/>
       </c>
       <c r="K159" s="9">
-        <f>IF(H159&lt;&gt;"",MIN(L158,(M159-J159)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I159)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I159))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I159)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I159))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I159))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I159))*(MONTH($B$34:$B$48)=MONTH(I159))*$C$34:$C$48)),"")</f>
+        <f>IF(H159&lt;&gt;"",MIN(L158,(M159-J159)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I159)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I159))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I159)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I159))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I159))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I159))*(MONTH($B$35:$B$49)=MONTH(I159))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L159" s="9">
@@ -6650,7 +6650,7 @@
         <v/>
       </c>
       <c r="K160" s="14">
-        <f>IF(H160&lt;&gt;"",MIN(L159,(M160-J160)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I160)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I160))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I160)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I160))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I160))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I160))*(MONTH($B$34:$B$48)=MONTH(I160))*$C$34:$C$48)),"")</f>
+        <f>IF(H160&lt;&gt;"",MIN(L159,(M160-J160)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I160)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I160))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I160)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I160))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I160))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I160))*(MONTH($B$35:$B$49)=MONTH(I160))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L160" s="14">
@@ -6684,7 +6684,7 @@
         <v/>
       </c>
       <c r="K161" s="9">
-        <f>IF(H161&lt;&gt;"",MIN(L160,(M161-J161)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I161)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I161))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I161)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I161))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I161))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I161))*(MONTH($B$34:$B$48)=MONTH(I161))*$C$34:$C$48)),"")</f>
+        <f>IF(H161&lt;&gt;"",MIN(L160,(M161-J161)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I161)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I161))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I161)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I161))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I161))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I161))*(MONTH($B$35:$B$49)=MONTH(I161))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L161" s="9">
@@ -6718,7 +6718,7 @@
         <v/>
       </c>
       <c r="K162" s="14">
-        <f>IF(H162&lt;&gt;"",MIN(L161,(M162-J162)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I162)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I162))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I162)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I162))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I162))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I162))*(MONTH($B$34:$B$48)=MONTH(I162))*$C$34:$C$48)),"")</f>
+        <f>IF(H162&lt;&gt;"",MIN(L161,(M162-J162)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I162)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I162))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I162)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I162))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I162))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I162))*(MONTH($B$35:$B$49)=MONTH(I162))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L162" s="14">
@@ -6752,7 +6752,7 @@
         <v/>
       </c>
       <c r="K163" s="9">
-        <f>IF(H163&lt;&gt;"",MIN(L162,(M163-J163)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I163)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I163))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I163)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I163))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I163))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I163))*(MONTH($B$34:$B$48)=MONTH(I163))*$C$34:$C$48)),"")</f>
+        <f>IF(H163&lt;&gt;"",MIN(L162,(M163-J163)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I163)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I163))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I163)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I163))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I163))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I163))*(MONTH($B$35:$B$49)=MONTH(I163))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L163" s="9">
@@ -6786,7 +6786,7 @@
         <v/>
       </c>
       <c r="K164" s="14">
-        <f>IF(H164&lt;&gt;"",MIN(L163,(M164-J164)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I164)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I164))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I164)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I164))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I164))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I164))*(MONTH($B$34:$B$48)=MONTH(I164))*$C$34:$C$48)),"")</f>
+        <f>IF(H164&lt;&gt;"",MIN(L163,(M164-J164)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I164)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I164))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I164)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I164))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I164))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I164))*(MONTH($B$35:$B$49)=MONTH(I164))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L164" s="14">
@@ -6820,7 +6820,7 @@
         <v/>
       </c>
       <c r="K165" s="9">
-        <f>IF(H165&lt;&gt;"",MIN(L164,(M165-J165)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I165)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I165))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I165)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I165))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I165))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I165))*(MONTH($B$34:$B$48)=MONTH(I165))*$C$34:$C$48)),"")</f>
+        <f>IF(H165&lt;&gt;"",MIN(L164,(M165-J165)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I165)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I165))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I165)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I165))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I165))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I165))*(MONTH($B$35:$B$49)=MONTH(I165))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L165" s="9">
@@ -6854,7 +6854,7 @@
         <v/>
       </c>
       <c r="K166" s="14">
-        <f>IF(H166&lt;&gt;"",MIN(L165,(M166-J166)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I166)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I166))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I166)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I166))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I166))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I166))*(MONTH($B$34:$B$48)=MONTH(I166))*$C$34:$C$48)),"")</f>
+        <f>IF(H166&lt;&gt;"",MIN(L165,(M166-J166)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I166)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I166))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I166)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I166))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I166))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I166))*(MONTH($B$35:$B$49)=MONTH(I166))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L166" s="14">
@@ -6888,7 +6888,7 @@
         <v/>
       </c>
       <c r="K167" s="9">
-        <f>IF(H167&lt;&gt;"",MIN(L166,(M167-J167)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I167)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I167))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I167)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I167))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I167))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I167))*(MONTH($B$34:$B$48)=MONTH(I167))*$C$34:$C$48)),"")</f>
+        <f>IF(H167&lt;&gt;"",MIN(L166,(M167-J167)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I167)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I167))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I167)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I167))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I167))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I167))*(MONTH($B$35:$B$49)=MONTH(I167))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L167" s="9">
@@ -6922,7 +6922,7 @@
         <v/>
       </c>
       <c r="K168" s="14">
-        <f>IF(H168&lt;&gt;"",MIN(L167,(M168-J168)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I168)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I168))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I168)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I168))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I168))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I168))*(MONTH($B$34:$B$48)=MONTH(I168))*$C$34:$C$48)),"")</f>
+        <f>IF(H168&lt;&gt;"",MIN(L167,(M168-J168)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I168)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I168))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I168)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I168))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I168))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I168))*(MONTH($B$35:$B$49)=MONTH(I168))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L168" s="14">
@@ -6956,7 +6956,7 @@
         <v/>
       </c>
       <c r="K169" s="9">
-        <f>IF(H169&lt;&gt;"",MIN(L168,(M169-J169)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I169)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I169))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I169)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I169))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I169))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I169))*(MONTH($B$34:$B$48)=MONTH(I169))*$C$34:$C$48)),"")</f>
+        <f>IF(H169&lt;&gt;"",MIN(L168,(M169-J169)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I169)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I169))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I169)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I169))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I169))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I169))*(MONTH($B$35:$B$49)=MONTH(I169))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L169" s="9">
@@ -6990,7 +6990,7 @@
         <v/>
       </c>
       <c r="K170" s="14">
-        <f>IF(H170&lt;&gt;"",MIN(L169,(M170-J170)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I170)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I170))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I170)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I170))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I170))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I170))*(MONTH($B$34:$B$48)=MONTH(I170))*$C$34:$C$48)),"")</f>
+        <f>IF(H170&lt;&gt;"",MIN(L169,(M170-J170)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I170)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I170))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I170)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I170))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I170))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I170))*(MONTH($B$35:$B$49)=MONTH(I170))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L170" s="14">
@@ -7024,7 +7024,7 @@
         <v/>
       </c>
       <c r="K171" s="9">
-        <f>IF(H171&lt;&gt;"",MIN(L170,(M171-J171)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I171)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I171))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I171)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I171))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I171))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I171))*(MONTH($B$34:$B$48)=MONTH(I171))*$C$34:$C$48)),"")</f>
+        <f>IF(H171&lt;&gt;"",MIN(L170,(M171-J171)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I171)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I171))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I171)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I171))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I171))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I171))*(MONTH($B$35:$B$49)=MONTH(I171))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L171" s="9">
@@ -7058,7 +7058,7 @@
         <v/>
       </c>
       <c r="K172" s="14">
-        <f>IF(H172&lt;&gt;"",MIN(L171,(M172-J172)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I172)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I172))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I172)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I172))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I172))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I172))*(MONTH($B$34:$B$48)=MONTH(I172))*$C$34:$C$48)),"")</f>
+        <f>IF(H172&lt;&gt;"",MIN(L171,(M172-J172)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I172)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I172))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I172)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I172))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I172))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I172))*(MONTH($B$35:$B$49)=MONTH(I172))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L172" s="14">
@@ -7092,7 +7092,7 @@
         <v/>
       </c>
       <c r="K173" s="9">
-        <f>IF(H173&lt;&gt;"",MIN(L172,(M173-J173)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I173)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I173))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I173)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I173))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I173))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I173))*(MONTH($B$34:$B$48)=MONTH(I173))*$C$34:$C$48)),"")</f>
+        <f>IF(H173&lt;&gt;"",MIN(L172,(M173-J173)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I173)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I173))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I173)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I173))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I173))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I173))*(MONTH($B$35:$B$49)=MONTH(I173))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L173" s="9">
@@ -7126,7 +7126,7 @@
         <v/>
       </c>
       <c r="K174" s="14">
-        <f>IF(H174&lt;&gt;"",MIN(L173,(M174-J174)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I174)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I174))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I174)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I174))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I174))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I174))*(MONTH($B$34:$B$48)=MONTH(I174))*$C$34:$C$48)),"")</f>
+        <f>IF(H174&lt;&gt;"",MIN(L173,(M174-J174)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I174)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I174))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I174)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I174))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I174))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I174))*(MONTH($B$35:$B$49)=MONTH(I174))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L174" s="14">
@@ -7160,7 +7160,7 @@
         <v/>
       </c>
       <c r="K175" s="9">
-        <f>IF(H175&lt;&gt;"",MIN(L174,(M175-J175)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I175)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I175))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I175)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I175))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I175))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I175))*(MONTH($B$34:$B$48)=MONTH(I175))*$C$34:$C$48)),"")</f>
+        <f>IF(H175&lt;&gt;"",MIN(L174,(M175-J175)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I175)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I175))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I175)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I175))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I175))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I175))*(MONTH($B$35:$B$49)=MONTH(I175))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L175" s="9">
@@ -7194,7 +7194,7 @@
         <v/>
       </c>
       <c r="K176" s="14">
-        <f>IF(H176&lt;&gt;"",MIN(L175,(M176-J176)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I176)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I176))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I176)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I176))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I176))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I176))*(MONTH($B$34:$B$48)=MONTH(I176))*$C$34:$C$48)),"")</f>
+        <f>IF(H176&lt;&gt;"",MIN(L175,(M176-J176)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I176)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I176))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I176)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I176))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I176))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I176))*(MONTH($B$35:$B$49)=MONTH(I176))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L176" s="14">
@@ -7228,7 +7228,7 @@
         <v/>
       </c>
       <c r="K177" s="9">
-        <f>IF(H177&lt;&gt;"",MIN(L176,(M177-J177)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I177)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I177))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I177)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I177))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I177))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I177))*(MONTH($B$34:$B$48)=MONTH(I177))*$C$34:$C$48)),"")</f>
+        <f>IF(H177&lt;&gt;"",MIN(L176,(M177-J177)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I177)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I177))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I177)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I177))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I177))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I177))*(MONTH($B$35:$B$49)=MONTH(I177))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L177" s="9">
@@ -7262,7 +7262,7 @@
         <v/>
       </c>
       <c r="K178" s="14">
-        <f>IF(H178&lt;&gt;"",MIN(L177,(M178-J178)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I178)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I178))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I178)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I178))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I178))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I178))*(MONTH($B$34:$B$48)=MONTH(I178))*$C$34:$C$48)),"")</f>
+        <f>IF(H178&lt;&gt;"",MIN(L177,(M178-J178)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I178)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I178))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I178)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I178))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I178))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I178))*(MONTH($B$35:$B$49)=MONTH(I178))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L178" s="14">
@@ -7296,7 +7296,7 @@
         <v/>
       </c>
       <c r="K179" s="9">
-        <f>IF(H179&lt;&gt;"",MIN(L178,(M179-J179)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I179)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I179))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I179)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I179))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I179))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I179))*(MONTH($B$34:$B$48)=MONTH(I179))*$C$34:$C$48)),"")</f>
+        <f>IF(H179&lt;&gt;"",MIN(L178,(M179-J179)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I179)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I179))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I179)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I179))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I179))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I179))*(MONTH($B$35:$B$49)=MONTH(I179))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L179" s="9">
@@ -7330,7 +7330,7 @@
         <v/>
       </c>
       <c r="K180" s="14">
-        <f>IF(H180&lt;&gt;"",MIN(L179,(M180-J180)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I180)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I180))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I180)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I180))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I180))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I180))*(MONTH($B$34:$B$48)=MONTH(I180))*$C$34:$C$48)),"")</f>
+        <f>IF(H180&lt;&gt;"",MIN(L179,(M180-J180)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I180)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I180))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I180)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I180))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I180))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I180))*(MONTH($B$35:$B$49)=MONTH(I180))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L180" s="14">
@@ -7364,7 +7364,7 @@
         <v/>
       </c>
       <c r="K181" s="9">
-        <f>IF(H181&lt;&gt;"",MIN(L180,(M181-J181)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I181)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I181))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I181)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I181))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I181))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I181))*(MONTH($B$34:$B$48)=MONTH(I181))*$C$34:$C$48)),"")</f>
+        <f>IF(H181&lt;&gt;"",MIN(L180,(M181-J181)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I181)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I181))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I181)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I181))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I181))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I181))*(MONTH($B$35:$B$49)=MONTH(I181))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L181" s="9">
@@ -7398,7 +7398,7 @@
         <v/>
       </c>
       <c r="K182" s="14">
-        <f>IF(H182&lt;&gt;"",MIN(L181,(M182-J182)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I182)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I182))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I182)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I182))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I182))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I182))*(MONTH($B$34:$B$48)=MONTH(I182))*$C$34:$C$48)),"")</f>
+        <f>IF(H182&lt;&gt;"",MIN(L181,(M182-J182)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I182)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I182))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I182)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I182))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I182))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I182))*(MONTH($B$35:$B$49)=MONTH(I182))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L182" s="14">
@@ -7432,7 +7432,7 @@
         <v/>
       </c>
       <c r="K183" s="9">
-        <f>IF(H183&lt;&gt;"",MIN(L182,(M183-J183)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I183)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I183))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I183)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I183))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I183))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I183))*(MONTH($B$34:$B$48)=MONTH(I183))*$C$34:$C$48)),"")</f>
+        <f>IF(H183&lt;&gt;"",MIN(L182,(M183-J183)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I183)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I183))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I183)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I183))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I183))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I183))*(MONTH($B$35:$B$49)=MONTH(I183))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L183" s="9">
@@ -7466,7 +7466,7 @@
         <v/>
       </c>
       <c r="K184" s="14">
-        <f>IF(H184&lt;&gt;"",MIN(L183,(M184-J184)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I184)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I184))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I184)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I184))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I184))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I184))*(MONTH($B$34:$B$48)=MONTH(I184))*$C$34:$C$48)),"")</f>
+        <f>IF(H184&lt;&gt;"",MIN(L183,(M184-J184)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I184)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I184))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I184)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I184))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I184))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I184))*(MONTH($B$35:$B$49)=MONTH(I184))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L184" s="14">
@@ -7500,7 +7500,7 @@
         <v/>
       </c>
       <c r="K185" s="9">
-        <f>IF(H185&lt;&gt;"",MIN(L184,(M185-J185)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I185)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I185))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I185)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I185))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I185))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I185))*(MONTH($B$34:$B$48)=MONTH(I185))*$C$34:$C$48)),"")</f>
+        <f>IF(H185&lt;&gt;"",MIN(L184,(M185-J185)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I185)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I185))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I185)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I185))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I185))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I185))*(MONTH($B$35:$B$49)=MONTH(I185))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L185" s="9">
@@ -7534,7 +7534,7 @@
         <v/>
       </c>
       <c r="K186" s="14">
-        <f>IF(H186&lt;&gt;"",MIN(L185,(M186-J186)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I186)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I186))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I186)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I186))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I186))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I186))*(MONTH($B$34:$B$48)=MONTH(I186))*$C$34:$C$48)),"")</f>
+        <f>IF(H186&lt;&gt;"",MIN(L185,(M186-J186)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I186)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I186))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I186)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I186))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I186))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I186))*(MONTH($B$35:$B$49)=MONTH(I186))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L186" s="14">
@@ -7568,7 +7568,7 @@
         <v/>
       </c>
       <c r="K187" s="9">
-        <f>IF(H187&lt;&gt;"",MIN(L186,(M187-J187)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I187)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I187))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I187)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I187))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I187))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I187))*(MONTH($B$34:$B$48)=MONTH(I187))*$C$34:$C$48)),"")</f>
+        <f>IF(H187&lt;&gt;"",MIN(L186,(M187-J187)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I187)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I187))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I187)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I187))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I187))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I187))*(MONTH($B$35:$B$49)=MONTH(I187))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L187" s="9">
@@ -7602,7 +7602,7 @@
         <v/>
       </c>
       <c r="K188" s="14">
-        <f>IF(H188&lt;&gt;"",MIN(L187,(M188-J188)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I188)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I188))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I188)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I188))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I188))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I188))*(MONTH($B$34:$B$48)=MONTH(I188))*$C$34:$C$48)),"")</f>
+        <f>IF(H188&lt;&gt;"",MIN(L187,(M188-J188)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I188)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I188))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I188)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I188))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I188))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I188))*(MONTH($B$35:$B$49)=MONTH(I188))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L188" s="14">
@@ -7636,7 +7636,7 @@
         <v/>
       </c>
       <c r="K189" s="9">
-        <f>IF(H189&lt;&gt;"",MIN(L188,(M189-J189)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I189)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I189))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I189)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I189))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I189))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I189))*(MONTH($B$34:$B$48)=MONTH(I189))*$C$34:$C$48)),"")</f>
+        <f>IF(H189&lt;&gt;"",MIN(L188,(M189-J189)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I189)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I189))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I189)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I189))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I189))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I189))*(MONTH($B$35:$B$49)=MONTH(I189))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L189" s="9">
@@ -7670,7 +7670,7 @@
         <v/>
       </c>
       <c r="K190" s="14">
-        <f>IF(H190&lt;&gt;"",MIN(L189,(M190-J190)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I190)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I190))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I190)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I190))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I190))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I190))*(MONTH($B$34:$B$48)=MONTH(I190))*$C$34:$C$48)),"")</f>
+        <f>IF(H190&lt;&gt;"",MIN(L189,(M190-J190)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I190)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I190))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I190)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I190))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I190))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I190))*(MONTH($B$35:$B$49)=MONTH(I190))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L190" s="14">
@@ -7704,7 +7704,7 @@
         <v/>
       </c>
       <c r="K191" s="9">
-        <f>IF(H191&lt;&gt;"",MIN(L190,(M191-J191)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I191)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I191))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I191)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I191))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I191))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I191))*(MONTH($B$34:$B$48)=MONTH(I191))*$C$34:$C$48)),"")</f>
+        <f>IF(H191&lt;&gt;"",MIN(L190,(M191-J191)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I191)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I191))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I191)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I191))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I191))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I191))*(MONTH($B$35:$B$49)=MONTH(I191))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L191" s="9">
@@ -7738,7 +7738,7 @@
         <v/>
       </c>
       <c r="K192" s="14">
-        <f>IF(H192&lt;&gt;"",MIN(L191,(M192-J192)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I192)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I192))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I192)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I192))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I192))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I192))*(MONTH($B$34:$B$48)=MONTH(I192))*$C$34:$C$48)),"")</f>
+        <f>IF(H192&lt;&gt;"",MIN(L191,(M192-J192)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I192)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I192))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I192)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I192))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I192))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I192))*(MONTH($B$35:$B$49)=MONTH(I192))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L192" s="14">
@@ -7772,7 +7772,7 @@
         <v/>
       </c>
       <c r="K193" s="9">
-        <f>IF(H193&lt;&gt;"",MIN(L192,(M193-J193)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I193)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I193))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I193)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I193))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I193))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I193))*(MONTH($B$34:$B$48)=MONTH(I193))*$C$34:$C$48)),"")</f>
+        <f>IF(H193&lt;&gt;"",MIN(L192,(M193-J193)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I193)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I193))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I193)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I193))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I193))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I193))*(MONTH($B$35:$B$49)=MONTH(I193))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L193" s="9">
@@ -7806,7 +7806,7 @@
         <v/>
       </c>
       <c r="K194" s="14">
-        <f>IF(H194&lt;&gt;"",MIN(L193,(M194-J194)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I194)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I194))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I194)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I194))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I194))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I194))*(MONTH($B$34:$B$48)=MONTH(I194))*$C$34:$C$48)),"")</f>
+        <f>IF(H194&lt;&gt;"",MIN(L193,(M194-J194)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I194)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I194))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I194)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I194))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I194))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I194))*(MONTH($B$35:$B$49)=MONTH(I194))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L194" s="14">
@@ -7840,7 +7840,7 @@
         <v/>
       </c>
       <c r="K195" s="9">
-        <f>IF(H195&lt;&gt;"",MIN(L194,(M195-J195)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I195)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I195))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I195)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I195))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I195))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I195))*(MONTH($B$34:$B$48)=MONTH(I195))*$C$34:$C$48)),"")</f>
+        <f>IF(H195&lt;&gt;"",MIN(L194,(M195-J195)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I195)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I195))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I195)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I195))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I195))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I195))*(MONTH($B$35:$B$49)=MONTH(I195))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L195" s="9">
@@ -7874,7 +7874,7 @@
         <v/>
       </c>
       <c r="K196" s="14">
-        <f>IF(H196&lt;&gt;"",MIN(L195,(M196-J196)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I196)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I196))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I196)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I196))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I196))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I196))*(MONTH($B$34:$B$48)=MONTH(I196))*$C$34:$C$48)),"")</f>
+        <f>IF(H196&lt;&gt;"",MIN(L195,(M196-J196)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I196)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I196))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I196)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I196))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I196))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I196))*(MONTH($B$35:$B$49)=MONTH(I196))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L196" s="14">
@@ -7908,7 +7908,7 @@
         <v/>
       </c>
       <c r="K197" s="9">
-        <f>IF(H197&lt;&gt;"",MIN(L196,(M197-J197)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I197)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I197))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I197)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I197))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I197))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I197))*(MONTH($B$34:$B$48)=MONTH(I197))*$C$34:$C$48)),"")</f>
+        <f>IF(H197&lt;&gt;"",MIN(L196,(M197-J197)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I197)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I197))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I197)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I197))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I197))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I197))*(MONTH($B$35:$B$49)=MONTH(I197))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L197" s="9">
@@ -7942,7 +7942,7 @@
         <v/>
       </c>
       <c r="K198" s="14">
-        <f>IF(H198&lt;&gt;"",MIN(L197,(M198-J198)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I198)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I198))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I198)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I198))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I198))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I198))*(MONTH($B$34:$B$48)=MONTH(I198))*$C$34:$C$48)),"")</f>
+        <f>IF(H198&lt;&gt;"",MIN(L197,(M198-J198)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I198)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I198))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I198)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I198))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I198))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I198))*(MONTH($B$35:$B$49)=MONTH(I198))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L198" s="14">
@@ -7976,7 +7976,7 @@
         <v/>
       </c>
       <c r="K199" s="9">
-        <f>IF(H199&lt;&gt;"",MIN(L198,(M199-J199)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I199)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I199))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I199)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I199))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I199))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I199))*(MONTH($B$34:$B$48)=MONTH(I199))*$C$34:$C$48)),"")</f>
+        <f>IF(H199&lt;&gt;"",MIN(L198,(M199-J199)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I199)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I199))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I199)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I199))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I199))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I199))*(MONTH($B$35:$B$49)=MONTH(I199))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L199" s="9">
@@ -8010,7 +8010,7 @@
         <v/>
       </c>
       <c r="K200" s="14">
-        <f>IF(H200&lt;&gt;"",MIN(L199,(M200-J200)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I200)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I200))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I200)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I200))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I200))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I200))*(MONTH($B$34:$B$48)=MONTH(I200))*$C$34:$C$48)),"")</f>
+        <f>IF(H200&lt;&gt;"",MIN(L199,(M200-J200)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I200)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I200))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I200)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I200))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I200))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I200))*(MONTH($B$35:$B$49)=MONTH(I200))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L200" s="14">
@@ -8044,7 +8044,7 @@
         <v/>
       </c>
       <c r="K201" s="9">
-        <f>IF(H201&lt;&gt;"",MIN(L200,(M201-J201)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I201)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I201))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I201)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I201))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I201))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I201))*(MONTH($B$34:$B$48)=MONTH(I201))*$C$34:$C$48)),"")</f>
+        <f>IF(H201&lt;&gt;"",MIN(L200,(M201-J201)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I201)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I201))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I201)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I201))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I201))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I201))*(MONTH($B$35:$B$49)=MONTH(I201))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L201" s="9">
@@ -8078,7 +8078,7 @@
         <v/>
       </c>
       <c r="K202" s="14">
-        <f>IF(H202&lt;&gt;"",MIN(L201,(M202-J202)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I202)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I202))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I202)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I202))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I202))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I202))*(MONTH($B$34:$B$48)=MONTH(I202))*$C$34:$C$48)),"")</f>
+        <f>IF(H202&lt;&gt;"",MIN(L201,(M202-J202)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I202)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I202))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I202)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I202))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I202))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I202))*(MONTH($B$35:$B$49)=MONTH(I202))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L202" s="14">
@@ -8112,7 +8112,7 @@
         <v/>
       </c>
       <c r="K203" s="9">
-        <f>IF(H203&lt;&gt;"",MIN(L202,(M203-J203)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I203)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I203))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I203)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I203))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I203))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I203))*(MONTH($B$34:$B$48)=MONTH(I203))*$C$34:$C$48)),"")</f>
+        <f>IF(H203&lt;&gt;"",MIN(L202,(M203-J203)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I203)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I203))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I203)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I203))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I203))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I203))*(MONTH($B$35:$B$49)=MONTH(I203))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L203" s="9">
@@ -8146,7 +8146,7 @@
         <v/>
       </c>
       <c r="K204" s="14">
-        <f>IF(H204&lt;&gt;"",MIN(L203,(M204-J204)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I204)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I204))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I204)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I204))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I204))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I204))*(MONTH($B$34:$B$48)=MONTH(I204))*$C$34:$C$48)),"")</f>
+        <f>IF(H204&lt;&gt;"",MIN(L203,(M204-J204)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I204)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I204))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I204)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I204))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I204))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I204))*(MONTH($B$35:$B$49)=MONTH(I204))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L204" s="14">
@@ -8180,7 +8180,7 @@
         <v/>
       </c>
       <c r="K205" s="9">
-        <f>IF(H205&lt;&gt;"",MIN(L204,(M205-J205)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I205)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I205))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I205)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I205))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I205))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I205))*(MONTH($B$34:$B$48)=MONTH(I205))*$C$34:$C$48)),"")</f>
+        <f>IF(H205&lt;&gt;"",MIN(L204,(M205-J205)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I205)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I205))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I205)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I205))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I205))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I205))*(MONTH($B$35:$B$49)=MONTH(I205))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L205" s="9">
@@ -8214,7 +8214,7 @@
         <v/>
       </c>
       <c r="K206" s="14">
-        <f>IF(H206&lt;&gt;"",MIN(L205,(M206-J206)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I206)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I206))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I206)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I206))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I206))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I206))*(MONTH($B$34:$B$48)=MONTH(I206))*$C$34:$C$48)),"")</f>
+        <f>IF(H206&lt;&gt;"",MIN(L205,(M206-J206)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I206)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I206))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I206)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I206))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I206))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I206))*(MONTH($B$35:$B$49)=MONTH(I206))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L206" s="14">
@@ -8248,7 +8248,7 @@
         <v/>
       </c>
       <c r="K207" s="9">
-        <f>IF(H207&lt;&gt;"",MIN(L206,(M207-J207)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I207)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I207))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I207)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I207))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I207))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I207))*(MONTH($B$34:$B$48)=MONTH(I207))*$C$34:$C$48)),"")</f>
+        <f>IF(H207&lt;&gt;"",MIN(L206,(M207-J207)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I207)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I207))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I207)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I207))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I207))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I207))*(MONTH($B$35:$B$49)=MONTH(I207))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L207" s="9">
@@ -8282,7 +8282,7 @@
         <v/>
       </c>
       <c r="K208" s="14">
-        <f>IF(H208&lt;&gt;"",MIN(L207,(M208-J208)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I208)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I208))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I208)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I208))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I208))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I208))*(MONTH($B$34:$B$48)=MONTH(I208))*$C$34:$C$48)),"")</f>
+        <f>IF(H208&lt;&gt;"",MIN(L207,(M208-J208)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I208)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I208))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I208)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I208))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I208))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I208))*(MONTH($B$35:$B$49)=MONTH(I208))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L208" s="14">
@@ -8316,7 +8316,7 @@
         <v/>
       </c>
       <c r="K209" s="9">
-        <f>IF(H209&lt;&gt;"",MIN(L208,(M209-J209)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I209)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I209))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I209)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I209))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I209))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I209))*(MONTH($B$34:$B$48)=MONTH(I209))*$C$34:$C$48)),"")</f>
+        <f>IF(H209&lt;&gt;"",MIN(L208,(M209-J209)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I209)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I209))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I209)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I209))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I209))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I209))*(MONTH($B$35:$B$49)=MONTH(I209))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L209" s="9">
@@ -8350,7 +8350,7 @@
         <v/>
       </c>
       <c r="K210" s="14">
-        <f>IF(H210&lt;&gt;"",MIN(L209,(M210-J210)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I210)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I210))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I210)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I210))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I210))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I210))*(MONTH($B$34:$B$48)=MONTH(I210))*$C$34:$C$48)),"")</f>
+        <f>IF(H210&lt;&gt;"",MIN(L209,(M210-J210)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I210)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I210))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I210)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I210))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I210))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I210))*(MONTH($B$35:$B$49)=MONTH(I210))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L210" s="14">
@@ -8384,7 +8384,7 @@
         <v/>
       </c>
       <c r="K211" s="9">
-        <f>IF(H211&lt;&gt;"",MIN(L210,(M211-J211)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I211)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I211))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I211)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I211))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I211))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I211))*(MONTH($B$34:$B$48)=MONTH(I211))*$C$34:$C$48)),"")</f>
+        <f>IF(H211&lt;&gt;"",MIN(L210,(M211-J211)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I211)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I211))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I211)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I211))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I211))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I211))*(MONTH($B$35:$B$49)=MONTH(I211))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L211" s="9">
@@ -8418,7 +8418,7 @@
         <v/>
       </c>
       <c r="K212" s="14">
-        <f>IF(H212&lt;&gt;"",MIN(L211,(M212-J212)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I212)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I212))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I212)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I212))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I212))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I212))*(MONTH($B$34:$B$48)=MONTH(I212))*$C$34:$C$48)),"")</f>
+        <f>IF(H212&lt;&gt;"",MIN(L211,(M212-J212)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I212)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I212))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I212)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I212))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I212))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I212))*(MONTH($B$35:$B$49)=MONTH(I212))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L212" s="14">
@@ -8452,7 +8452,7 @@
         <v/>
       </c>
       <c r="K213" s="9">
-        <f>IF(H213&lt;&gt;"",MIN(L212,(M213-J213)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I213)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I213))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I213)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I213))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I213))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I213))*(MONTH($B$34:$B$48)=MONTH(I213))*$C$34:$C$48)),"")</f>
+        <f>IF(H213&lt;&gt;"",MIN(L212,(M213-J213)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I213)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I213))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I213)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I213))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I213))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I213))*(MONTH($B$35:$B$49)=MONTH(I213))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L213" s="9">
@@ -8486,7 +8486,7 @@
         <v/>
       </c>
       <c r="K214" s="14">
-        <f>IF(H214&lt;&gt;"",MIN(L213,(M214-J214)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I214)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I214))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I214)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I214))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I214))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I214))*(MONTH($B$34:$B$48)=MONTH(I214))*$C$34:$C$48)),"")</f>
+        <f>IF(H214&lt;&gt;"",MIN(L213,(M214-J214)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I214)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I214))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I214)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I214))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I214))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I214))*(MONTH($B$35:$B$49)=MONTH(I214))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L214" s="14">
@@ -8520,7 +8520,7 @@
         <v/>
       </c>
       <c r="K215" s="9">
-        <f>IF(H215&lt;&gt;"",MIN(L214,(M215-J215)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I215)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I215))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I215)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I215))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I215))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I215))*(MONTH($B$34:$B$48)=MONTH(I215))*$C$34:$C$48)),"")</f>
+        <f>IF(H215&lt;&gt;"",MIN(L214,(M215-J215)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I215)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I215))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I215)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I215))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I215))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I215))*(MONTH($B$35:$B$49)=MONTH(I215))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L215" s="9">
@@ -8554,7 +8554,7 @@
         <v/>
       </c>
       <c r="K216" s="14">
-        <f>IF(H216&lt;&gt;"",MIN(L215,(M216-J216)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I216)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I216))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I216)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I216))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I216))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I216))*(MONTH($B$34:$B$48)=MONTH(I216))*$C$34:$C$48)),"")</f>
+        <f>IF(H216&lt;&gt;"",MIN(L215,(M216-J216)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I216)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I216))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I216)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I216))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I216))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I216))*(MONTH($B$35:$B$49)=MONTH(I216))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L216" s="14">
@@ -8588,7 +8588,7 @@
         <v/>
       </c>
       <c r="K217" s="9">
-        <f>IF(H217&lt;&gt;"",MIN(L216,(M217-J217)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I217)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I217))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I217)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I217))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I217))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I217))*(MONTH($B$34:$B$48)=MONTH(I217))*$C$34:$C$48)),"")</f>
+        <f>IF(H217&lt;&gt;"",MIN(L216,(M217-J217)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I217)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I217))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I217)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I217))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I217))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I217))*(MONTH($B$35:$B$49)=MONTH(I217))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L217" s="9">
@@ -8622,7 +8622,7 @@
         <v/>
       </c>
       <c r="K218" s="14">
-        <f>IF(H218&lt;&gt;"",MIN(L217,(M218-J218)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I218)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I218))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I218)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I218))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I218))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I218))*(MONTH($B$34:$B$48)=MONTH(I218))*$C$34:$C$48)),"")</f>
+        <f>IF(H218&lt;&gt;"",MIN(L217,(M218-J218)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I218)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I218))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I218)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I218))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I218))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I218))*(MONTH($B$35:$B$49)=MONTH(I218))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L218" s="14">
@@ -8656,7 +8656,7 @@
         <v/>
       </c>
       <c r="K219" s="9">
-        <f>IF(H219&lt;&gt;"",MIN(L218,(M219-J219)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I219)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I219))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I219)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I219))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I219))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I219))*(MONTH($B$34:$B$48)=MONTH(I219))*$C$34:$C$48)),"")</f>
+        <f>IF(H219&lt;&gt;"",MIN(L218,(M219-J219)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I219)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I219))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I219)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I219))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I219))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I219))*(MONTH($B$35:$B$49)=MONTH(I219))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L219" s="9">
@@ -8690,7 +8690,7 @@
         <v/>
       </c>
       <c r="K220" s="14">
-        <f>IF(H220&lt;&gt;"",MIN(L219,(M220-J220)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I220)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I220))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I220)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I220))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I220))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I220))*(MONTH($B$34:$B$48)=MONTH(I220))*$C$34:$C$48)),"")</f>
+        <f>IF(H220&lt;&gt;"",MIN(L219,(M220-J220)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I220)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I220))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I220)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I220))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I220))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I220))*(MONTH($B$35:$B$49)=MONTH(I220))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L220" s="14">
@@ -8724,7 +8724,7 @@
         <v/>
       </c>
       <c r="K221" s="9">
-        <f>IF(H221&lt;&gt;"",MIN(L220,(M221-J221)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I221)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I221))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I221)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I221))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I221))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I221))*(MONTH($B$34:$B$48)=MONTH(I221))*$C$34:$C$48)),"")</f>
+        <f>IF(H221&lt;&gt;"",MIN(L220,(M221-J221)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I221)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I221))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I221)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I221))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I221))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I221))*(MONTH($B$35:$B$49)=MONTH(I221))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L221" s="9">
@@ -8758,7 +8758,7 @@
         <v/>
       </c>
       <c r="K222" s="14">
-        <f>IF(H222&lt;&gt;"",MIN(L221,(M222-J222)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I222)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I222))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I222)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I222))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I222))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I222))*(MONTH($B$34:$B$48)=MONTH(I222))*$C$34:$C$48)),"")</f>
+        <f>IF(H222&lt;&gt;"",MIN(L221,(M222-J222)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I222)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I222))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I222)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I222))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I222))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I222))*(MONTH($B$35:$B$49)=MONTH(I222))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L222" s="14">
@@ -8792,7 +8792,7 @@
         <v/>
       </c>
       <c r="K223" s="9">
-        <f>IF(H223&lt;&gt;"",MIN(L222,(M223-J223)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I223)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I223))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I223)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I223))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I223))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I223))*(MONTH($B$34:$B$48)=MONTH(I223))*$C$34:$C$48)),"")</f>
+        <f>IF(H223&lt;&gt;"",MIN(L222,(M223-J223)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I223)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I223))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I223)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I223))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I223))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I223))*(MONTH($B$35:$B$49)=MONTH(I223))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L223" s="9">
@@ -8826,7 +8826,7 @@
         <v/>
       </c>
       <c r="K224" s="14">
-        <f>IF(H224&lt;&gt;"",MIN(L223,(M224-J224)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I224)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I224))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I224)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I224))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I224))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I224))*(MONTH($B$34:$B$48)=MONTH(I224))*$C$34:$C$48)),"")</f>
+        <f>IF(H224&lt;&gt;"",MIN(L223,(M224-J224)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I224)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I224))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I224)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I224))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I224))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I224))*(MONTH($B$35:$B$49)=MONTH(I224))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L224" s="14">
@@ -8860,7 +8860,7 @@
         <v/>
       </c>
       <c r="K225" s="9">
-        <f>IF(H225&lt;&gt;"",MIN(L224,(M225-J225)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I225)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I225))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I225)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I225))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I225))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I225))*(MONTH($B$34:$B$48)=MONTH(I225))*$C$34:$C$48)),"")</f>
+        <f>IF(H225&lt;&gt;"",MIN(L224,(M225-J225)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I225)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I225))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I225)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I225))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I225))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I225))*(MONTH($B$35:$B$49)=MONTH(I225))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L225" s="9">
@@ -8894,7 +8894,7 @@
         <v/>
       </c>
       <c r="K226" s="14">
-        <f>IF(H226&lt;&gt;"",MIN(L225,(M226-J226)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I226)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I226))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I226)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I226))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I226))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I226))*(MONTH($B$34:$B$48)=MONTH(I226))*$C$34:$C$48)),"")</f>
+        <f>IF(H226&lt;&gt;"",MIN(L225,(M226-J226)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I226)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I226))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I226)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I226))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I226))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I226))*(MONTH($B$35:$B$49)=MONTH(I226))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L226" s="14">
@@ -8928,7 +8928,7 @@
         <v/>
       </c>
       <c r="K227" s="9">
-        <f>IF(H227&lt;&gt;"",MIN(L226,(M227-J227)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I227)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I227))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I227)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I227))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I227))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I227))*(MONTH($B$34:$B$48)=MONTH(I227))*$C$34:$C$48)),"")</f>
+        <f>IF(H227&lt;&gt;"",MIN(L226,(M227-J227)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I227)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I227))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I227)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I227))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I227))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I227))*(MONTH($B$35:$B$49)=MONTH(I227))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L227" s="9">
@@ -8962,7 +8962,7 @@
         <v/>
       </c>
       <c r="K228" s="14">
-        <f>IF(H228&lt;&gt;"",MIN(L227,(M228-J228)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I228)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I228))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I228)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I228))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I228))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I228))*(MONTH($B$34:$B$48)=MONTH(I228))*$C$34:$C$48)),"")</f>
+        <f>IF(H228&lt;&gt;"",MIN(L227,(M228-J228)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I228)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I228))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I228)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I228))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I228))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I228))*(MONTH($B$35:$B$49)=MONTH(I228))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L228" s="14">
@@ -8996,7 +8996,7 @@
         <v/>
       </c>
       <c r="K229" s="9">
-        <f>IF(H229&lt;&gt;"",MIN(L228,(M229-J229)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I229)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I229))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I229)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I229))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I229))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I229))*(MONTH($B$34:$B$48)=MONTH(I229))*$C$34:$C$48)),"")</f>
+        <f>IF(H229&lt;&gt;"",MIN(L228,(M229-J229)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I229)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I229))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I229)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I229))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I229))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I229))*(MONTH($B$35:$B$49)=MONTH(I229))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L229" s="9">
@@ -9030,7 +9030,7 @@
         <v/>
       </c>
       <c r="K230" s="14">
-        <f>IF(H230&lt;&gt;"",MIN(L229,(M230-J230)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I230)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I230))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I230)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I230))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I230))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I230))*(MONTH($B$34:$B$48)=MONTH(I230))*$C$34:$C$48)),"")</f>
+        <f>IF(H230&lt;&gt;"",MIN(L229,(M230-J230)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I230)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I230))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I230)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I230))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I230))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I230))*(MONTH($B$35:$B$49)=MONTH(I230))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L230" s="14">
@@ -9064,7 +9064,7 @@
         <v/>
       </c>
       <c r="K231" s="9">
-        <f>IF(H231&lt;&gt;"",MIN(L230,(M231-J231)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I231)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I231))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I231)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I231))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I231))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I231))*(MONTH($B$34:$B$48)=MONTH(I231))*$C$34:$C$48)),"")</f>
+        <f>IF(H231&lt;&gt;"",MIN(L230,(M231-J231)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I231)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I231))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I231)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I231))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I231))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I231))*(MONTH($B$35:$B$49)=MONTH(I231))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L231" s="9">
@@ -9098,7 +9098,7 @@
         <v/>
       </c>
       <c r="K232" s="14">
-        <f>IF(H232&lt;&gt;"",MIN(L231,(M232-J232)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I232)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I232))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I232)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I232))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I232))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I232))*(MONTH($B$34:$B$48)=MONTH(I232))*$C$34:$C$48)),"")</f>
+        <f>IF(H232&lt;&gt;"",MIN(L231,(M232-J232)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I232)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I232))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I232)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I232))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I232))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I232))*(MONTH($B$35:$B$49)=MONTH(I232))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L232" s="14">
@@ -9132,7 +9132,7 @@
         <v/>
       </c>
       <c r="K233" s="9">
-        <f>IF(H233&lt;&gt;"",MIN(L232,(M233-J233)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I233)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I233))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I233)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I233))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I233))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I233))*(MONTH($B$34:$B$48)=MONTH(I233))*$C$34:$C$48)),"")</f>
+        <f>IF(H233&lt;&gt;"",MIN(L232,(M233-J233)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I233)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I233))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I233)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I233))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I233))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I233))*(MONTH($B$35:$B$49)=MONTH(I233))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L233" s="9">
@@ -9166,7 +9166,7 @@
         <v/>
       </c>
       <c r="K234" s="14">
-        <f>IF(H234&lt;&gt;"",MIN(L233,(M234-J234)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I234)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I234))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I234)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I234))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I234))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I234))*(MONTH($B$34:$B$48)=MONTH(I234))*$C$34:$C$48)),"")</f>
+        <f>IF(H234&lt;&gt;"",MIN(L233,(M234-J234)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I234)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I234))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I234)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I234))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I234))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I234))*(MONTH($B$35:$B$49)=MONTH(I234))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L234" s="14">
@@ -9200,7 +9200,7 @@
         <v/>
       </c>
       <c r="K235" s="9">
-        <f>IF(H235&lt;&gt;"",MIN(L234,(M235-J235)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I235)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I235))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I235)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I235))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I235))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I235))*(MONTH($B$34:$B$48)=MONTH(I235))*$C$34:$C$48)),"")</f>
+        <f>IF(H235&lt;&gt;"",MIN(L234,(M235-J235)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I235)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I235))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I235)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I235))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I235))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I235))*(MONTH($B$35:$B$49)=MONTH(I235))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L235" s="9">
@@ -9234,7 +9234,7 @@
         <v/>
       </c>
       <c r="K236" s="14">
-        <f>IF(H236&lt;&gt;"",MIN(L235,(M236-J236)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I236)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I236))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I236)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I236))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I236))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I236))*(MONTH($B$34:$B$48)=MONTH(I236))*$C$34:$C$48)),"")</f>
+        <f>IF(H236&lt;&gt;"",MIN(L235,(M236-J236)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I236)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I236))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I236)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I236))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I236))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I236))*(MONTH($B$35:$B$49)=MONTH(I236))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L236" s="14">
@@ -9268,7 +9268,7 @@
         <v/>
       </c>
       <c r="K237" s="9">
-        <f>IF(H237&lt;&gt;"",MIN(L236,(M237-J237)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I237)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I237))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I237)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I237))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I237))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I237))*(MONTH($B$34:$B$48)=MONTH(I237))*$C$34:$C$48)),"")</f>
+        <f>IF(H237&lt;&gt;"",MIN(L236,(M237-J237)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I237)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I237))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I237)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I237))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I237))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I237))*(MONTH($B$35:$B$49)=MONTH(I237))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L237" s="9">
@@ -9302,7 +9302,7 @@
         <v/>
       </c>
       <c r="K238" s="14">
-        <f>IF(H238&lt;&gt;"",MIN(L237,(M238-J238)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I238)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I238))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I238)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I238))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I238))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I238))*(MONTH($B$34:$B$48)=MONTH(I238))*$C$34:$C$48)),"")</f>
+        <f>IF(H238&lt;&gt;"",MIN(L237,(M238-J238)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I238)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I238))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I238)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I238))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I238))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I238))*(MONTH($B$35:$B$49)=MONTH(I238))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L238" s="14">
@@ -9336,7 +9336,7 @@
         <v/>
       </c>
       <c r="K239" s="9">
-        <f>IF(H239&lt;&gt;"",MIN(L238,(M239-J239)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I239)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I239))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I239)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I239))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I239))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I239))*(MONTH($B$34:$B$48)=MONTH(I239))*$C$34:$C$48)),"")</f>
+        <f>IF(H239&lt;&gt;"",MIN(L238,(M239-J239)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I239)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I239))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I239)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I239))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I239))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I239))*(MONTH($B$35:$B$49)=MONTH(I239))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L239" s="9">
@@ -9370,7 +9370,7 @@
         <v/>
       </c>
       <c r="K240" s="14">
-        <f>IF(H240&lt;&gt;"",MIN(L239,(M240-J240)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I240)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I240))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I240)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I240))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I240))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I240))*(MONTH($B$34:$B$48)=MONTH(I240))*$C$34:$C$48)),"")</f>
+        <f>IF(H240&lt;&gt;"",MIN(L239,(M240-J240)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I240)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I240))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I240)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I240))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I240))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I240))*(MONTH($B$35:$B$49)=MONTH(I240))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L240" s="14">
@@ -9404,7 +9404,7 @@
         <v/>
       </c>
       <c r="K241" s="9">
-        <f>IF(H241&lt;&gt;"",MIN(L240,(M241-J241)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I241)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I241))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I241)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I241))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I241))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I241))*(MONTH($B$34:$B$48)=MONTH(I241))*$C$34:$C$48)),"")</f>
+        <f>IF(H241&lt;&gt;"",MIN(L240,(M241-J241)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I241)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I241))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I241)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I241))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I241))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I241))*(MONTH($B$35:$B$49)=MONTH(I241))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L241" s="9">
@@ -9438,7 +9438,7 @@
         <v/>
       </c>
       <c r="K242" s="14">
-        <f>IF(H242&lt;&gt;"",MIN(L241,(M242-J242)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I242)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I242))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I242)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I242))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I242))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I242))*(MONTH($B$34:$B$48)=MONTH(I242))*$C$34:$C$48)),"")</f>
+        <f>IF(H242&lt;&gt;"",MIN(L241,(M242-J242)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I242)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I242))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I242)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I242))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I242))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I242))*(MONTH($B$35:$B$49)=MONTH(I242))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L242" s="14">
@@ -9472,7 +9472,7 @@
         <v/>
       </c>
       <c r="K243" s="9">
-        <f>IF(H243&lt;&gt;"",MIN(L242,(M243-J243)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I243)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I243))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I243)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I243))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I243))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I243))*(MONTH($B$34:$B$48)=MONTH(I243))*$C$34:$C$48)),"")</f>
+        <f>IF(H243&lt;&gt;"",MIN(L242,(M243-J243)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I243)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I243))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I243)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I243))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I243))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I243))*(MONTH($B$35:$B$49)=MONTH(I243))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L243" s="9">
@@ -9506,7 +9506,7 @@
         <v/>
       </c>
       <c r="K244" s="14">
-        <f>IF(H244&lt;&gt;"",MIN(L243,(M244-J244)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I244)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I244))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I244)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I244))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I244))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I244))*(MONTH($B$34:$B$48)=MONTH(I244))*$C$34:$C$48)),"")</f>
+        <f>IF(H244&lt;&gt;"",MIN(L243,(M244-J244)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I244)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I244))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I244)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I244))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I244))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I244))*(MONTH($B$35:$B$49)=MONTH(I244))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L244" s="14">
@@ -9540,7 +9540,7 @@
         <v/>
       </c>
       <c r="K245" s="9">
-        <f>IF(H245&lt;&gt;"",MIN(L244,(M245-J245)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I245)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I245))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I245)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I245))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I245))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I245))*(MONTH($B$34:$B$48)=MONTH(I245))*$C$34:$C$48)),"")</f>
+        <f>IF(H245&lt;&gt;"",MIN(L244,(M245-J245)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I245)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I245))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I245)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I245))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I245))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I245))*(MONTH($B$35:$B$49)=MONTH(I245))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L245" s="9">
@@ -9574,7 +9574,7 @@
         <v/>
       </c>
       <c r="K246" s="14">
-        <f>IF(H246&lt;&gt;"",MIN(L245,(M246-J246)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I246)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I246))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I246)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I246))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I246))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I246))*(MONTH($B$34:$B$48)=MONTH(I246))*$C$34:$C$48)),"")</f>
+        <f>IF(H246&lt;&gt;"",MIN(L245,(M246-J246)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I246)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I246))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I246)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I246))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I246))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I246))*(MONTH($B$35:$B$49)=MONTH(I246))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L246" s="14">
@@ -9608,7 +9608,7 @@
         <v/>
       </c>
       <c r="K247" s="9">
-        <f>IF(H247&lt;&gt;"",MIN(L246,(M247-J247)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I247)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I247))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I247)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I247))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I247))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I247))*(MONTH($B$34:$B$48)=MONTH(I247))*$C$34:$C$48)),"")</f>
+        <f>IF(H247&lt;&gt;"",MIN(L246,(M247-J247)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I247)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I247))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I247)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I247))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I247))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I247))*(MONTH($B$35:$B$49)=MONTH(I247))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L247" s="9">
@@ -9642,7 +9642,7 @@
         <v/>
       </c>
       <c r="K248" s="14">
-        <f>IF(H248&lt;&gt;"",MIN(L247,(M248-J248)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I248)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I248))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I248)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I248))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I248))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I248))*(MONTH($B$34:$B$48)=MONTH(I248))*$C$34:$C$48)),"")</f>
+        <f>IF(H248&lt;&gt;"",MIN(L247,(M248-J248)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I248)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I248))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I248)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I248))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I248))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I248))*(MONTH($B$35:$B$49)=MONTH(I248))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L248" s="14">
@@ -9676,7 +9676,7 @@
         <v/>
       </c>
       <c r="K249" s="9">
-        <f>IF(H249&lt;&gt;"",MIN(L248,(M249-J249)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I249)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I249))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I249)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I249))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I249))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I249))*(MONTH($B$34:$B$48)=MONTH(I249))*$C$34:$C$48)),"")</f>
+        <f>IF(H249&lt;&gt;"",MIN(L248,(M249-J249)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I249)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I249))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I249)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I249))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I249))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I249))*(MONTH($B$35:$B$49)=MONTH(I249))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L249" s="9">
@@ -9710,7 +9710,7 @@
         <v/>
       </c>
       <c r="K250" s="14">
-        <f>IF(H250&lt;&gt;"",MIN(L249,(M250-J250)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I250)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I250))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I250)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I250))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I250))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I250))*(MONTH($B$34:$B$48)=MONTH(I250))*$C$34:$C$48)),"")</f>
+        <f>IF(H250&lt;&gt;"",MIN(L249,(M250-J250)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I250)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I250))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I250)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I250))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I250))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I250))*(MONTH($B$35:$B$49)=MONTH(I250))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L250" s="14">
@@ -9744,7 +9744,7 @@
         <v/>
       </c>
       <c r="K251" s="9">
-        <f>IF(H251&lt;&gt;"",MIN(L250,(M251-J251)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I251)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I251))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I251)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I251))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I251))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I251))*(MONTH($B$34:$B$48)=MONTH(I251))*$C$34:$C$48)),"")</f>
+        <f>IF(H251&lt;&gt;"",MIN(L250,(M251-J251)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I251)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I251))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I251)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I251))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I251))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I251))*(MONTH($B$35:$B$49)=MONTH(I251))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L251" s="9">
@@ -9778,7 +9778,7 @@
         <v/>
       </c>
       <c r="K252" s="14">
-        <f>IF(H252&lt;&gt;"",MIN(L251,(M252-J252)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I252)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I252))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I252)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I252))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I252))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I252))*(MONTH($B$34:$B$48)=MONTH(I252))*$C$34:$C$48)),"")</f>
+        <f>IF(H252&lt;&gt;"",MIN(L251,(M252-J252)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I252)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I252))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I252)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I252))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I252))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I252))*(MONTH($B$35:$B$49)=MONTH(I252))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L252" s="14">
@@ -9812,7 +9812,7 @@
         <v/>
       </c>
       <c r="K253" s="9">
-        <f>IF(H253&lt;&gt;"",MIN(L252,(M253-J253)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I253)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I253))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I253)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I253))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I253))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I253))*(MONTH($B$34:$B$48)=MONTH(I253))*$C$34:$C$48)),"")</f>
+        <f>IF(H253&lt;&gt;"",MIN(L252,(M253-J253)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I253)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I253))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I253)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I253))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I253))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I253))*(MONTH($B$35:$B$49)=MONTH(I253))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L253" s="9">
@@ -9846,7 +9846,7 @@
         <v/>
       </c>
       <c r="K254" s="14">
-        <f>IF(H254&lt;&gt;"",MIN(L253,(M254-J254)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I254)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I254))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I254)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I254))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I254))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I254))*(MONTH($B$34:$B$48)=MONTH(I254))*$C$34:$C$48)),"")</f>
+        <f>IF(H254&lt;&gt;"",MIN(L253,(M254-J254)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I254)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I254))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I254)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I254))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I254))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I254))*(MONTH($B$35:$B$49)=MONTH(I254))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L254" s="14">
@@ -9880,7 +9880,7 @@
         <v/>
       </c>
       <c r="K255" s="9">
-        <f>IF(H255&lt;&gt;"",MIN(L254,(M255-J255)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I255)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I255))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I255)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I255))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I255))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I255))*(MONTH($B$34:$B$48)=MONTH(I255))*$C$34:$C$48)),"")</f>
+        <f>IF(H255&lt;&gt;"",MIN(L254,(M255-J255)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I255)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I255))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I255)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I255))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I255))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I255))*(MONTH($B$35:$B$49)=MONTH(I255))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L255" s="9">
@@ -9914,7 +9914,7 @@
         <v/>
       </c>
       <c r="K256" s="14">
-        <f>IF(H256&lt;&gt;"",MIN(L255,(M256-J256)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I256)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I256))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I256)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I256))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I256))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I256))*(MONTH($B$34:$B$48)=MONTH(I256))*$C$34:$C$48)),"")</f>
+        <f>IF(H256&lt;&gt;"",MIN(L255,(M256-J256)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I256)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I256))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I256)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I256))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I256))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I256))*(MONTH($B$35:$B$49)=MONTH(I256))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L256" s="14">
@@ -9948,7 +9948,7 @@
         <v/>
       </c>
       <c r="K257" s="9">
-        <f>IF(H257&lt;&gt;"",MIN(L256,(M257-J257)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I257)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I257))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I257)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I257))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I257))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I257))*(MONTH($B$34:$B$48)=MONTH(I257))*$C$34:$C$48)),"")</f>
+        <f>IF(H257&lt;&gt;"",MIN(L256,(M257-J257)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I257)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I257))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I257)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I257))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I257))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I257))*(MONTH($B$35:$B$49)=MONTH(I257))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L257" s="9">
@@ -9982,7 +9982,7 @@
         <v/>
       </c>
       <c r="K258" s="14">
-        <f>IF(H258&lt;&gt;"",MIN(L257,(M258-J258)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I258)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I258))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I258)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I258))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I258))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I258))*(MONTH($B$34:$B$48)=MONTH(I258))*$C$34:$C$48)),"")</f>
+        <f>IF(H258&lt;&gt;"",MIN(L257,(M258-J258)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I258)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I258))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I258)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I258))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I258))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I258))*(MONTH($B$35:$B$49)=MONTH(I258))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L258" s="14">
@@ -10016,7 +10016,7 @@
         <v/>
       </c>
       <c r="K259" s="9">
-        <f>IF(H259&lt;&gt;"",MIN(L258,(M259-J259)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I259)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I259))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I259)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I259))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I259))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I259))*(MONTH($B$34:$B$48)=MONTH(I259))*$C$34:$C$48)),"")</f>
+        <f>IF(H259&lt;&gt;"",MIN(L258,(M259-J259)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I259)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I259))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I259)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I259))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I259))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I259))*(MONTH($B$35:$B$49)=MONTH(I259))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L259" s="9">
@@ -10050,7 +10050,7 @@
         <v/>
       </c>
       <c r="K260" s="14">
-        <f>IF(H260&lt;&gt;"",MIN(L259,(M260-J260)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I260)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I260))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I260)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I260))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I260))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I260))*(MONTH($B$34:$B$48)=MONTH(I260))*$C$34:$C$48)),"")</f>
+        <f>IF(H260&lt;&gt;"",MIN(L259,(M260-J260)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I260)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I260))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I260)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I260))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I260))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I260))*(MONTH($B$35:$B$49)=MONTH(I260))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L260" s="14">
@@ -10084,7 +10084,7 @@
         <v/>
       </c>
       <c r="K261" s="9">
-        <f>IF(H261&lt;&gt;"",MIN(L260,(M261-J261)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I261)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I261))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I261)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I261))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I261))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I261))*(MONTH($B$34:$B$48)=MONTH(I261))*$C$34:$C$48)),"")</f>
+        <f>IF(H261&lt;&gt;"",MIN(L260,(M261-J261)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I261)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I261))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I261)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I261))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I261))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I261))*(MONTH($B$35:$B$49)=MONTH(I261))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L261" s="9">
@@ -10118,7 +10118,7 @@
         <v/>
       </c>
       <c r="K262" s="14">
-        <f>IF(H262&lt;&gt;"",MIN(L261,(M262-J262)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I262)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I262))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I262)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I262))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I262))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I262))*(MONTH($B$34:$B$48)=MONTH(I262))*$C$34:$C$48)),"")</f>
+        <f>IF(H262&lt;&gt;"",MIN(L261,(M262-J262)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I262)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I262))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I262)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I262))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I262))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I262))*(MONTH($B$35:$B$49)=MONTH(I262))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L262" s="14">
@@ -10152,7 +10152,7 @@
         <v/>
       </c>
       <c r="K263" s="9">
-        <f>IF(H263&lt;&gt;"",MIN(L262,(M263-J263)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I263)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I263))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I263)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I263))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I263))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I263))*(MONTH($B$34:$B$48)=MONTH(I263))*$C$34:$C$48)),"")</f>
+        <f>IF(H263&lt;&gt;"",MIN(L262,(M263-J263)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I263)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I263))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I263)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I263))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I263))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I263))*(MONTH($B$35:$B$49)=MONTH(I263))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L263" s="9">
@@ -10186,7 +10186,7 @@
         <v/>
       </c>
       <c r="K264" s="14">
-        <f>IF(H264&lt;&gt;"",MIN(L263,(M264-J264)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I264)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I264))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I264)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I264))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I264))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I264))*(MONTH($B$34:$B$48)=MONTH(I264))*$C$34:$C$48)),"")</f>
+        <f>IF(H264&lt;&gt;"",MIN(L263,(M264-J264)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I264)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I264))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I264)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I264))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I264))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I264))*(MONTH($B$35:$B$49)=MONTH(I264))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L264" s="14">
@@ -10220,7 +10220,7 @@
         <v/>
       </c>
       <c r="K265" s="9">
-        <f>IF(H265&lt;&gt;"",MIN(L264,(M265-J265)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I265)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I265))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I265)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I265))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I265))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I265))*(MONTH($B$34:$B$48)=MONTH(I265))*$C$34:$C$48)),"")</f>
+        <f>IF(H265&lt;&gt;"",MIN(L264,(M265-J265)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I265)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I265))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I265)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I265))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I265))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I265))*(MONTH($B$35:$B$49)=MONTH(I265))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L265" s="9">
@@ -10254,7 +10254,7 @@
         <v/>
       </c>
       <c r="K266" s="14">
-        <f>IF(H266&lt;&gt;"",MIN(L265,(M266-J266)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I266)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I266))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I266)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I266))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I266))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I266))*(MONTH($B$34:$B$48)=MONTH(I266))*$C$34:$C$48)),"")</f>
+        <f>IF(H266&lt;&gt;"",MIN(L265,(M266-J266)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I266)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I266))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I266)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I266))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I266))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I266))*(MONTH($B$35:$B$49)=MONTH(I266))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L266" s="14">
@@ -10288,7 +10288,7 @@
         <v/>
       </c>
       <c r="K267" s="9">
-        <f>IF(H267&lt;&gt;"",MIN(L266,(M267-J267)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I267)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I267))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I267)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I267))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I267))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I267))*(MONTH($B$34:$B$48)=MONTH(I267))*$C$34:$C$48)),"")</f>
+        <f>IF(H267&lt;&gt;"",MIN(L266,(M267-J267)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I267)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I267))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I267)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I267))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I267))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I267))*(MONTH($B$35:$B$49)=MONTH(I267))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L267" s="9">
@@ -10322,7 +10322,7 @@
         <v/>
       </c>
       <c r="K268" s="14">
-        <f>IF(H268&lt;&gt;"",MIN(L267,(M268-J268)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I268)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I268))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I268)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I268))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I268))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I268))*(MONTH($B$34:$B$48)=MONTH(I268))*$C$34:$C$48)),"")</f>
+        <f>IF(H268&lt;&gt;"",MIN(L267,(M268-J268)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I268)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I268))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I268)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I268))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I268))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I268))*(MONTH($B$35:$B$49)=MONTH(I268))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L268" s="14">
@@ -10356,7 +10356,7 @@
         <v/>
       </c>
       <c r="K269" s="9">
-        <f>IF(H269&lt;&gt;"",MIN(L268,(M269-J269)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I269)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I269))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I269)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I269))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I269))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I269))*(MONTH($B$34:$B$48)=MONTH(I269))*$C$34:$C$48)),"")</f>
+        <f>IF(H269&lt;&gt;"",MIN(L268,(M269-J269)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I269)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I269))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I269)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I269))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I269))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I269))*(MONTH($B$35:$B$49)=MONTH(I269))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L269" s="9">
@@ -10390,7 +10390,7 @@
         <v/>
       </c>
       <c r="K270" s="14">
-        <f>IF(H270&lt;&gt;"",MIN(L269,(M270-J270)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I270)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I270))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I270)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I270))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I270))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I270))*(MONTH($B$34:$B$48)=MONTH(I270))*$C$34:$C$48)),"")</f>
+        <f>IF(H270&lt;&gt;"",MIN(L269,(M270-J270)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I270)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I270))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I270)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I270))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I270))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I270))*(MONTH($B$35:$B$49)=MONTH(I270))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L270" s="14">
@@ -10424,7 +10424,7 @@
         <v/>
       </c>
       <c r="K271" s="9">
-        <f>IF(H271&lt;&gt;"",MIN(L270,(M271-J271)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I271)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I271))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I271)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I271))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I271))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I271))*(MONTH($B$34:$B$48)=MONTH(I271))*$C$34:$C$48)),"")</f>
+        <f>IF(H271&lt;&gt;"",MIN(L270,(M271-J271)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I271)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I271))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I271)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I271))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I271))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I271))*(MONTH($B$35:$B$49)=MONTH(I271))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L271" s="9">
@@ -10458,7 +10458,7 @@
         <v/>
       </c>
       <c r="K272" s="14">
-        <f>IF(H272&lt;&gt;"",MIN(L271,(M272-J272)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I272)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I272))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I272)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I272))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I272))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I272))*(MONTH($B$34:$B$48)=MONTH(I272))*$C$34:$C$48)),"")</f>
+        <f>IF(H272&lt;&gt;"",MIN(L271,(M272-J272)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I272)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I272))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I272)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I272))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I272))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I272))*(MONTH($B$35:$B$49)=MONTH(I272))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L272" s="14">
@@ -10492,7 +10492,7 @@
         <v/>
       </c>
       <c r="K273" s="9">
-        <f>IF(H273&lt;&gt;"",MIN(L272,(M273-J273)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I273)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I273))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I273)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I273))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I273))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I273))*(MONTH($B$34:$B$48)=MONTH(I273))*$C$34:$C$48)),"")</f>
+        <f>IF(H273&lt;&gt;"",MIN(L272,(M273-J273)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I273)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I273))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I273)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I273))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I273))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I273))*(MONTH($B$35:$B$49)=MONTH(I273))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L273" s="9">
@@ -10526,7 +10526,7 @@
         <v/>
       </c>
       <c r="K274" s="14">
-        <f>IF(H274&lt;&gt;"",MIN(L273,(M274-J274)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I274)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I274))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I274)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I274))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I274))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I274))*(MONTH($B$34:$B$48)=MONTH(I274))*$C$34:$C$48)),"")</f>
+        <f>IF(H274&lt;&gt;"",MIN(L273,(M274-J274)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I274)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I274))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I274)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I274))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I274))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I274))*(MONTH($B$35:$B$49)=MONTH(I274))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L274" s="14">
@@ -10560,7 +10560,7 @@
         <v/>
       </c>
       <c r="K275" s="9">
-        <f>IF(H275&lt;&gt;"",MIN(L274,(M275-J275)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I275)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I275))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I275)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I275))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I275))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I275))*(MONTH($B$34:$B$48)=MONTH(I275))*$C$34:$C$48)),"")</f>
+        <f>IF(H275&lt;&gt;"",MIN(L274,(M275-J275)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I275)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I275))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I275)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I275))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I275))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I275))*(MONTH($B$35:$B$49)=MONTH(I275))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L275" s="9">
@@ -10594,7 +10594,7 @@
         <v/>
       </c>
       <c r="K276" s="14">
-        <f>IF(H276&lt;&gt;"",MIN(L275,(M276-J276)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I276)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I276))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I276)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I276))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I276))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I276))*(MONTH($B$34:$B$48)=MONTH(I276))*$C$34:$C$48)),"")</f>
+        <f>IF(H276&lt;&gt;"",MIN(L275,(M276-J276)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I276)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I276))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I276)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I276))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I276))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I276))*(MONTH($B$35:$B$49)=MONTH(I276))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L276" s="14">
@@ -10628,7 +10628,7 @@
         <v/>
       </c>
       <c r="K277" s="9">
-        <f>IF(H277&lt;&gt;"",MIN(L276,(M277-J277)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I277)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I277))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I277)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I277))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I277))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I277))*(MONTH($B$34:$B$48)=MONTH(I277))*$C$34:$C$48)),"")</f>
+        <f>IF(H277&lt;&gt;"",MIN(L276,(M277-J277)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I277)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I277))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I277)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I277))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I277))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I277))*(MONTH($B$35:$B$49)=MONTH(I277))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L277" s="9">
@@ -10662,7 +10662,7 @@
         <v/>
       </c>
       <c r="K278" s="14">
-        <f>IF(H278&lt;&gt;"",MIN(L277,(M278-J278)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I278)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I278))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I278)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I278))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I278))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I278))*(MONTH($B$34:$B$48)=MONTH(I278))*$C$34:$C$48)),"")</f>
+        <f>IF(H278&lt;&gt;"",MIN(L277,(M278-J278)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I278)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I278))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I278)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I278))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I278))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I278))*(MONTH($B$35:$B$49)=MONTH(I278))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L278" s="14">
@@ -10696,7 +10696,7 @@
         <v/>
       </c>
       <c r="K279" s="9">
-        <f>IF(H279&lt;&gt;"",MIN(L278,(M279-J279)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I279)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I279))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I279)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I279))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I279))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I279))*(MONTH($B$34:$B$48)=MONTH(I279))*$C$34:$C$48)),"")</f>
+        <f>IF(H279&lt;&gt;"",MIN(L278,(M279-J279)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I279)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I279))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I279)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I279))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I279))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I279))*(MONTH($B$35:$B$49)=MONTH(I279))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L279" s="9">
@@ -10730,7 +10730,7 @@
         <v/>
       </c>
       <c r="K280" s="14">
-        <f>IF(H280&lt;&gt;"",MIN(L279,(M280-J280)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I280)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I280))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I280)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I280))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I280))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I280))*(MONTH($B$34:$B$48)=MONTH(I280))*$C$34:$C$48)),"")</f>
+        <f>IF(H280&lt;&gt;"",MIN(L279,(M280-J280)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I280)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I280))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I280)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I280))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I280))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I280))*(MONTH($B$35:$B$49)=MONTH(I280))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L280" s="14">
@@ -10764,7 +10764,7 @@
         <v/>
       </c>
       <c r="K281" s="9">
-        <f>IF(H281&lt;&gt;"",MIN(L280,(M281-J281)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I281)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I281))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I281)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I281))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I281))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I281))*(MONTH($B$34:$B$48)=MONTH(I281))*$C$34:$C$48)),"")</f>
+        <f>IF(H281&lt;&gt;"",MIN(L280,(M281-J281)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I281)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I281))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I281)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I281))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I281))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I281))*(MONTH($B$35:$B$49)=MONTH(I281))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L281" s="9">
@@ -10798,7 +10798,7 @@
         <v/>
       </c>
       <c r="K282" s="14">
-        <f>IF(H282&lt;&gt;"",MIN(L281,(M282-J282)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I282)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I282))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I282)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I282))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I282))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I282))*(MONTH($B$34:$B$48)=MONTH(I282))*$C$34:$C$48)),"")</f>
+        <f>IF(H282&lt;&gt;"",MIN(L281,(M282-J282)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I282)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I282))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I282)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I282))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I282))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I282))*(MONTH($B$35:$B$49)=MONTH(I282))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L282" s="14">
@@ -10832,7 +10832,7 @@
         <v/>
       </c>
       <c r="K283" s="9">
-        <f>IF(H283&lt;&gt;"",MIN(L282,(M283-J283)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I283)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I283))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I283)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I283))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I283))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I283))*(MONTH($B$34:$B$48)=MONTH(I283))*$C$34:$C$48)),"")</f>
+        <f>IF(H283&lt;&gt;"",MIN(L282,(M283-J283)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I283)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I283))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I283)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I283))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I283))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I283))*(MONTH($B$35:$B$49)=MONTH(I283))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L283" s="9">
@@ -10866,7 +10866,7 @@
         <v/>
       </c>
       <c r="K284" s="14">
-        <f>IF(H284&lt;&gt;"",MIN(L283,(M284-J284)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I284)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I284))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I284)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I284))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I284))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I284))*(MONTH($B$34:$B$48)=MONTH(I284))*$C$34:$C$48)),"")</f>
+        <f>IF(H284&lt;&gt;"",MIN(L283,(M284-J284)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I284)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I284))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I284)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I284))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I284))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I284))*(MONTH($B$35:$B$49)=MONTH(I284))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L284" s="14">
@@ -10900,7 +10900,7 @@
         <v/>
       </c>
       <c r="K285" s="9">
-        <f>IF(H285&lt;&gt;"",MIN(L284,(M285-J285)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I285)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I285))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I285)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I285))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I285))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I285))*(MONTH($B$34:$B$48)=MONTH(I285))*$C$34:$C$48)),"")</f>
+        <f>IF(H285&lt;&gt;"",MIN(L284,(M285-J285)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I285)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I285))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I285)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I285))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I285))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I285))*(MONTH($B$35:$B$49)=MONTH(I285))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L285" s="9">
@@ -10934,7 +10934,7 @@
         <v/>
       </c>
       <c r="K286" s="14">
-        <f>IF(H286&lt;&gt;"",MIN(L285,(M286-J286)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I286)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I286))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I286)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I286))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I286))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I286))*(MONTH($B$34:$B$48)=MONTH(I286))*$C$34:$C$48)),"")</f>
+        <f>IF(H286&lt;&gt;"",MIN(L285,(M286-J286)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I286)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I286))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I286)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I286))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I286))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I286))*(MONTH($B$35:$B$49)=MONTH(I286))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L286" s="14">
@@ -10968,7 +10968,7 @@
         <v/>
       </c>
       <c r="K287" s="9">
-        <f>IF(H287&lt;&gt;"",MIN(L286,(M287-J287)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I287)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I287))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I287)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I287))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I287))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I287))*(MONTH($B$34:$B$48)=MONTH(I287))*$C$34:$C$48)),"")</f>
+        <f>IF(H287&lt;&gt;"",MIN(L286,(M287-J287)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I287)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I287))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I287)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I287))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I287))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I287))*(MONTH($B$35:$B$49)=MONTH(I287))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L287" s="9">
@@ -11002,7 +11002,7 @@
         <v/>
       </c>
       <c r="K288" s="14">
-        <f>IF(H288&lt;&gt;"",MIN(L287,(M288-J288)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I288)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I288))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I288)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I288))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I288))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I288))*(MONTH($B$34:$B$48)=MONTH(I288))*$C$34:$C$48)),"")</f>
+        <f>IF(H288&lt;&gt;"",MIN(L287,(M288-J288)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I288)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I288))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I288)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I288))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I288))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I288))*(MONTH($B$35:$B$49)=MONTH(I288))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L288" s="14">
@@ -11036,7 +11036,7 @@
         <v/>
       </c>
       <c r="K289" s="9">
-        <f>IF(H289&lt;&gt;"",MIN(L288,(M289-J289)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I289)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I289))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I289)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I289))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I289))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I289))*(MONTH($B$34:$B$48)=MONTH(I289))*$C$34:$C$48)),"")</f>
+        <f>IF(H289&lt;&gt;"",MIN(L288,(M289-J289)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I289)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I289))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I289)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I289))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I289))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I289))*(MONTH($B$35:$B$49)=MONTH(I289))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L289" s="9">
@@ -11070,7 +11070,7 @@
         <v/>
       </c>
       <c r="K290" s="14">
-        <f>IF(H290&lt;&gt;"",MIN(L289,(M290-J290)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I290)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I290))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I290)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I290))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I290))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I290))*(MONTH($B$34:$B$48)=MONTH(I290))*$C$34:$C$48)),"")</f>
+        <f>IF(H290&lt;&gt;"",MIN(L289,(M290-J290)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I290)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I290))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I290)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I290))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I290))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I290))*(MONTH($B$35:$B$49)=MONTH(I290))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L290" s="14">
@@ -11104,7 +11104,7 @@
         <v/>
       </c>
       <c r="K291" s="9">
-        <f>IF(H291&lt;&gt;"",MIN(L290,(M291-J291)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I291)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I291))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I291)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I291))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I291))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I291))*(MONTH($B$34:$B$48)=MONTH(I291))*$C$34:$C$48)),"")</f>
+        <f>IF(H291&lt;&gt;"",MIN(L290,(M291-J291)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I291)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I291))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I291)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I291))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I291))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I291))*(MONTH($B$35:$B$49)=MONTH(I291))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L291" s="9">
@@ -11138,7 +11138,7 @@
         <v/>
       </c>
       <c r="K292" s="14">
-        <f>IF(H292&lt;&gt;"",MIN(L291,(M292-J292)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I292)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I292))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I292)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I292))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I292))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I292))*(MONTH($B$34:$B$48)=MONTH(I292))*$C$34:$C$48)),"")</f>
+        <f>IF(H292&lt;&gt;"",MIN(L291,(M292-J292)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I292)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I292))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I292)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I292))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I292))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I292))*(MONTH($B$35:$B$49)=MONTH(I292))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L292" s="14">
@@ -11172,7 +11172,7 @@
         <v/>
       </c>
       <c r="K293" s="9">
-        <f>IF(H293&lt;&gt;"",MIN(L292,(M293-J293)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I293)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I293))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I293)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I293))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I293))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I293))*(MONTH($B$34:$B$48)=MONTH(I293))*$C$34:$C$48)),"")</f>
+        <f>IF(H293&lt;&gt;"",MIN(L292,(M293-J293)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I293)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I293))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I293)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I293))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I293))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I293))*(MONTH($B$35:$B$49)=MONTH(I293))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L293" s="9">
@@ -11206,7 +11206,7 @@
         <v/>
       </c>
       <c r="K294" s="14">
-        <f>IF(H294&lt;&gt;"",MIN(L293,(M294-J294)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I294)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I294))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I294)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I294))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I294))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I294))*(MONTH($B$34:$B$48)=MONTH(I294))*$C$34:$C$48)),"")</f>
+        <f>IF(H294&lt;&gt;"",MIN(L293,(M294-J294)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I294)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I294))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I294)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I294))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I294))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I294))*(MONTH($B$35:$B$49)=MONTH(I294))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L294" s="14">
@@ -11240,7 +11240,7 @@
         <v/>
       </c>
       <c r="K295" s="9">
-        <f>IF(H295&lt;&gt;"",MIN(L294,(M295-J295)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I295)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I295))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I295)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I295))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I295))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I295))*(MONTH($B$34:$B$48)=MONTH(I295))*$C$34:$C$48)),"")</f>
+        <f>IF(H295&lt;&gt;"",MIN(L294,(M295-J295)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I295)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I295))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I295)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I295))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I295))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I295))*(MONTH($B$35:$B$49)=MONTH(I295))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L295" s="9">
@@ -11274,7 +11274,7 @@
         <v/>
       </c>
       <c r="K296" s="14">
-        <f>IF(H296&lt;&gt;"",MIN(L295,(M296-J296)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I296)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I296))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I296)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I296))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I296))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I296))*(MONTH($B$34:$B$48)=MONTH(I296))*$C$34:$C$48)),"")</f>
+        <f>IF(H296&lt;&gt;"",MIN(L295,(M296-J296)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I296)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I296))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I296)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I296))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I296))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I296))*(MONTH($B$35:$B$49)=MONTH(I296))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L296" s="14">
@@ -11308,7 +11308,7 @@
         <v/>
       </c>
       <c r="K297" s="9">
-        <f>IF(H297&lt;&gt;"",MIN(L296,(M297-J297)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I297)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I297))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I297)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I297))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I297))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I297))*(MONTH($B$34:$B$48)=MONTH(I297))*$C$34:$C$48)),"")</f>
+        <f>IF(H297&lt;&gt;"",MIN(L296,(M297-J297)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I297)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I297))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I297)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I297))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I297))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I297))*(MONTH($B$35:$B$49)=MONTH(I297))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L297" s="9">
@@ -11342,7 +11342,7 @@
         <v/>
       </c>
       <c r="K298" s="14">
-        <f>IF(H298&lt;&gt;"",MIN(L297,(M298-J298)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I298)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I298))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I298)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I298))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I298))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I298))*(MONTH($B$34:$B$48)=MONTH(I298))*$C$34:$C$48)),"")</f>
+        <f>IF(H298&lt;&gt;"",MIN(L297,(M298-J298)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I298)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I298))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I298)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I298))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I298))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I298))*(MONTH($B$35:$B$49)=MONTH(I298))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L298" s="14">
@@ -11376,7 +11376,7 @@
         <v/>
       </c>
       <c r="K299" s="9">
-        <f>IF(H299&lt;&gt;"",MIN(L298,(M299-J299)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I299)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I299))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I299)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I299))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I299))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I299))*(MONTH($B$34:$B$48)=MONTH(I299))*$C$34:$C$48)),"")</f>
+        <f>IF(H299&lt;&gt;"",MIN(L298,(M299-J299)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I299)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I299))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I299)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I299))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I299))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I299))*(MONTH($B$35:$B$49)=MONTH(I299))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L299" s="9">
@@ -11410,7 +11410,7 @@
         <v/>
       </c>
       <c r="K300" s="14">
-        <f>IF(H300&lt;&gt;"",MIN(L299,(M300-J300)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I300)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I300))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I300)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I300))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I300))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I300))*(MONTH($B$34:$B$48)=MONTH(I300))*$C$34:$C$48)),"")</f>
+        <f>IF(H300&lt;&gt;"",MIN(L299,(M300-J300)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I300)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I300))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I300)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I300))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I300))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I300))*(MONTH($B$35:$B$49)=MONTH(I300))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L300" s="14">
@@ -11444,7 +11444,7 @@
         <v/>
       </c>
       <c r="K301" s="9">
-        <f>IF(H301&lt;&gt;"",MIN(L300,(M301-J301)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I301)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I301))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I301)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I301))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I301))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I301))*(MONTH($B$34:$B$48)=MONTH(I301))*$C$34:$C$48)),"")</f>
+        <f>IF(H301&lt;&gt;"",MIN(L300,(M301-J301)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I301)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I301))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I301)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I301))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I301))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I301))*(MONTH($B$35:$B$49)=MONTH(I301))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L301" s="9">
@@ -11478,7 +11478,7 @@
         <v/>
       </c>
       <c r="K302" s="14">
-        <f>IF(H302&lt;&gt;"",MIN(L301,(M302-J302)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I302)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I302))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I302)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I302))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I302))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I302))*(MONTH($B$34:$B$48)=MONTH(I302))*$C$34:$C$48)),"")</f>
+        <f>IF(H302&lt;&gt;"",MIN(L301,(M302-J302)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I302)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I302))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I302)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I302))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I302))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I302))*(MONTH($B$35:$B$49)=MONTH(I302))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L302" s="14">
@@ -11512,7 +11512,7 @@
         <v/>
       </c>
       <c r="K303" s="9">
-        <f>IF(H303&lt;&gt;"",MIN(L302,(M303-J303)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I303)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I303))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I303)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I303))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I303))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I303))*(MONTH($B$34:$B$48)=MONTH(I303))*$C$34:$C$48)),"")</f>
+        <f>IF(H303&lt;&gt;"",MIN(L302,(M303-J303)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I303)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I303))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I303)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I303))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I303))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I303))*(MONTH($B$35:$B$49)=MONTH(I303))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L303" s="9">
@@ -11546,7 +11546,7 @@
         <v/>
       </c>
       <c r="K304" s="14">
-        <f>IF(H304&lt;&gt;"",MIN(L303,(M304-J304)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I304)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I304))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I304)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I304))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I304))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I304))*(MONTH($B$34:$B$48)=MONTH(I304))*$C$34:$C$48)),"")</f>
+        <f>IF(H304&lt;&gt;"",MIN(L303,(M304-J304)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I304)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I304))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I304)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I304))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I304))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I304))*(MONTH($B$35:$B$49)=MONTH(I304))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L304" s="14">
@@ -11580,7 +11580,7 @@
         <v/>
       </c>
       <c r="K305" s="9">
-        <f>IF(H305&lt;&gt;"",MIN(L304,(M305-J305)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I305)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I305))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I305)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I305))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I305))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I305))*(MONTH($B$34:$B$48)=MONTH(I305))*$C$34:$C$48)),"")</f>
+        <f>IF(H305&lt;&gt;"",MIN(L304,(M305-J305)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I305)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I305))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I305)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I305))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I305))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I305))*(MONTH($B$35:$B$49)=MONTH(I305))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L305" s="9">
@@ -11614,7 +11614,7 @@
         <v/>
       </c>
       <c r="K306" s="14">
-        <f>IF(H306&lt;&gt;"",MIN(L305,(M306-J306)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I306)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I306))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I306)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I306))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I306))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I306))*(MONTH($B$34:$B$48)=MONTH(I306))*$C$34:$C$48)),"")</f>
+        <f>IF(H306&lt;&gt;"",MIN(L305,(M306-J306)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I306)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I306))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I306)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I306))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I306))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I306))*(MONTH($B$35:$B$49)=MONTH(I306))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L306" s="14">
@@ -11648,7 +11648,7 @@
         <v/>
       </c>
       <c r="K307" s="9">
-        <f>IF(H307&lt;&gt;"",MIN(L306,(M307-J307)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I307)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I307))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I307)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I307))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I307))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I307))*(MONTH($B$34:$B$48)=MONTH(I307))*$C$34:$C$48)),"")</f>
+        <f>IF(H307&lt;&gt;"",MIN(L306,(M307-J307)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I307)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I307))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I307)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I307))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I307))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I307))*(MONTH($B$35:$B$49)=MONTH(I307))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L307" s="9">
@@ -11682,7 +11682,7 @@
         <v/>
       </c>
       <c r="K308" s="14">
-        <f>IF(H308&lt;&gt;"",MIN(L307,(M308-J308)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I308)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I308))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I308)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I308))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I308))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I308))*(MONTH($B$34:$B$48)=MONTH(I308))*$C$34:$C$48)),"")</f>
+        <f>IF(H308&lt;&gt;"",MIN(L307,(M308-J308)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I308)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I308))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I308)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I308))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I308))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I308))*(MONTH($B$35:$B$49)=MONTH(I308))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L308" s="14">
@@ -11716,7 +11716,7 @@
         <v/>
       </c>
       <c r="K309" s="9">
-        <f>IF(H309&lt;&gt;"",MIN(L308,(M309-J309)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I309)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I309))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I309)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I309))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I309))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I309))*(MONTH($B$34:$B$48)=MONTH(I309))*$C$34:$C$48)),"")</f>
+        <f>IF(H309&lt;&gt;"",MIN(L308,(M309-J309)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I309)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I309))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I309)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I309))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I309))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I309))*(MONTH($B$35:$B$49)=MONTH(I309))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L309" s="9">
@@ -11750,7 +11750,7 @@
         <v/>
       </c>
       <c r="K310" s="14">
-        <f>IF(H310&lt;&gt;"",MIN(L309,(M310-J310)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I310)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I310))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I310)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I310))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I310))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I310))*(MONTH($B$34:$B$48)=MONTH(I310))*$C$34:$C$48)),"")</f>
+        <f>IF(H310&lt;&gt;"",MIN(L309,(M310-J310)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I310)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I310))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I310)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I310))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I310))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I310))*(MONTH($B$35:$B$49)=MONTH(I310))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L310" s="14">
@@ -11784,7 +11784,7 @@
         <v/>
       </c>
       <c r="K311" s="9">
-        <f>IF(H311&lt;&gt;"",MIN(L310,(M311-J311)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I311)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I311))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I311)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I311))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I311))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I311))*(MONTH($B$34:$B$48)=MONTH(I311))*$C$34:$C$48)),"")</f>
+        <f>IF(H311&lt;&gt;"",MIN(L310,(M311-J311)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I311)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I311))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I311)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I311))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I311))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I311))*(MONTH($B$35:$B$49)=MONTH(I311))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L311" s="9">
@@ -11818,7 +11818,7 @@
         <v/>
       </c>
       <c r="K312" s="14">
-        <f>IF(H312&lt;&gt;"",MIN(L311,(M312-J312)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I312)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I312))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I312)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I312))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I312))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I312))*(MONTH($B$34:$B$48)=MONTH(I312))*$C$34:$C$48)),"")</f>
+        <f>IF(H312&lt;&gt;"",MIN(L311,(M312-J312)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I312)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I312))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I312)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I312))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I312))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I312))*(MONTH($B$35:$B$49)=MONTH(I312))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L312" s="14">
@@ -11852,7 +11852,7 @@
         <v/>
       </c>
       <c r="K313" s="9">
-        <f>IF(H313&lt;&gt;"",MIN(L312,(M313-J313)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I313)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I313))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I313)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I313))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I313))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I313))*(MONTH($B$34:$B$48)=MONTH(I313))*$C$34:$C$48)),"")</f>
+        <f>IF(H313&lt;&gt;"",MIN(L312,(M313-J313)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I313)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I313))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I313)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I313))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I313))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I313))*(MONTH($B$35:$B$49)=MONTH(I313))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L313" s="9">
@@ -11886,7 +11886,7 @@
         <v/>
       </c>
       <c r="K314" s="14">
-        <f>IF(H314&lt;&gt;"",MIN(L313,(M314-J314)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I314)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I314))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I314)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I314))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I314))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I314))*(MONTH($B$34:$B$48)=MONTH(I314))*$C$34:$C$48)),"")</f>
+        <f>IF(H314&lt;&gt;"",MIN(L313,(M314-J314)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I314)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I314))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I314)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I314))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I314))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I314))*(MONTH($B$35:$B$49)=MONTH(I314))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L314" s="14">
@@ -11920,7 +11920,7 @@
         <v/>
       </c>
       <c r="K315" s="9">
-        <f>IF(H315&lt;&gt;"",MIN(L314,(M315-J315)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I315)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I315))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I315)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I315))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I315))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I315))*(MONTH($B$34:$B$48)=MONTH(I315))*$C$34:$C$48)),"")</f>
+        <f>IF(H315&lt;&gt;"",MIN(L314,(M315-J315)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I315)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I315))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I315)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I315))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I315))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I315))*(MONTH($B$35:$B$49)=MONTH(I315))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L315" s="9">
@@ -11954,7 +11954,7 @@
         <v/>
       </c>
       <c r="K316" s="14">
-        <f>IF(H316&lt;&gt;"",MIN(L315,(M316-J316)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I316)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I316))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I316)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I316))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I316))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I316))*(MONTH($B$34:$B$48)=MONTH(I316))*$C$34:$C$48)),"")</f>
+        <f>IF(H316&lt;&gt;"",MIN(L315,(M316-J316)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I316)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I316))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I316)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I316))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I316))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I316))*(MONTH($B$35:$B$49)=MONTH(I316))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L316" s="14">
@@ -11988,7 +11988,7 @@
         <v/>
       </c>
       <c r="K317" s="9">
-        <f>IF(H317&lt;&gt;"",MIN(L316,(M317-J317)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I317)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I317))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I317)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I317))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I317))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I317))*(MONTH($B$34:$B$48)=MONTH(I317))*$C$34:$C$48)),"")</f>
+        <f>IF(H317&lt;&gt;"",MIN(L316,(M317-J317)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I317)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I317))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I317)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I317))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I317))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I317))*(MONTH($B$35:$B$49)=MONTH(I317))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L317" s="9">
@@ -12022,7 +12022,7 @@
         <v/>
       </c>
       <c r="K318" s="14">
-        <f>IF(H318&lt;&gt;"",MIN(L317,(M318-J318)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I318)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I318))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I318)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I318))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I318))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I318))*(MONTH($B$34:$B$48)=MONTH(I318))*$C$34:$C$48)),"")</f>
+        <f>IF(H318&lt;&gt;"",MIN(L317,(M318-J318)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I318)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I318))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I318)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I318))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I318))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I318))*(MONTH($B$35:$B$49)=MONTH(I318))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L318" s="14">
@@ -12056,7 +12056,7 @@
         <v/>
       </c>
       <c r="K319" s="9">
-        <f>IF(H319&lt;&gt;"",MIN(L318,(M319-J319)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I319)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I319))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I319)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I319))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I319))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I319))*(MONTH($B$34:$B$48)=MONTH(I319))*$C$34:$C$48)),"")</f>
+        <f>IF(H319&lt;&gt;"",MIN(L318,(M319-J319)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I319)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I319))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I319)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I319))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I319))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I319))*(MONTH($B$35:$B$49)=MONTH(I319))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L319" s="9">
@@ -12090,7 +12090,7 @@
         <v/>
       </c>
       <c r="K320" s="14">
-        <f>IF(H320&lt;&gt;"",MIN(L319,(M320-J320)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I320)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I320))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I320)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I320))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I320))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I320))*(MONTH($B$34:$B$48)=MONTH(I320))*$C$34:$C$48)),"")</f>
+        <f>IF(H320&lt;&gt;"",MIN(L319,(M320-J320)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I320)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I320))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I320)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I320))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I320))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I320))*(MONTH($B$35:$B$49)=MONTH(I320))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L320" s="14">
@@ -12124,7 +12124,7 @@
         <v/>
       </c>
       <c r="K321" s="9">
-        <f>IF(H321&lt;&gt;"",MIN(L320,(M321-J321)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I321)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I321))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I321)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I321))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I321))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I321))*(MONTH($B$34:$B$48)=MONTH(I321))*$C$34:$C$48)),"")</f>
+        <f>IF(H321&lt;&gt;"",MIN(L320,(M321-J321)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I321)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I321))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I321)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I321))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I321))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I321))*(MONTH($B$35:$B$49)=MONTH(I321))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L321" s="9">
@@ -12158,7 +12158,7 @@
         <v/>
       </c>
       <c r="K322" s="14">
-        <f>IF(H322&lt;&gt;"",MIN(L321,(M322-J322)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I322)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I322))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I322)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I322))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I322))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I322))*(MONTH($B$34:$B$48)=MONTH(I322))*$C$34:$C$48)),"")</f>
+        <f>IF(H322&lt;&gt;"",MIN(L321,(M322-J322)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I322)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I322))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I322)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I322))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I322))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I322))*(MONTH($B$35:$B$49)=MONTH(I322))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L322" s="14">
@@ -12192,7 +12192,7 @@
         <v/>
       </c>
       <c r="K323" s="9">
-        <f>IF(H323&lt;&gt;"",MIN(L322,(M323-J323)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I323)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I323))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I323)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I323))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I323))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I323))*(MONTH($B$34:$B$48)=MONTH(I323))*$C$34:$C$48)),"")</f>
+        <f>IF(H323&lt;&gt;"",MIN(L322,(M323-J323)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I323)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I323))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I323)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I323))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I323))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I323))*(MONTH($B$35:$B$49)=MONTH(I323))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L323" s="9">
@@ -12226,7 +12226,7 @@
         <v/>
       </c>
       <c r="K324" s="14">
-        <f>IF(H324&lt;&gt;"",MIN(L323,(M324-J324)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I324)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I324))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I324)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I324))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I324))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I324))*(MONTH($B$34:$B$48)=MONTH(I324))*$C$34:$C$48)),"")</f>
+        <f>IF(H324&lt;&gt;"",MIN(L323,(M324-J324)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I324)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I324))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I324)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I324))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I324))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I324))*(MONTH($B$35:$B$49)=MONTH(I324))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L324" s="14">
@@ -12260,7 +12260,7 @@
         <v/>
       </c>
       <c r="K325" s="9">
-        <f>IF(H325&lt;&gt;"",MIN(L324,(M325-J325)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I325)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I325))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I325)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I325))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I325))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I325))*(MONTH($B$34:$B$48)=MONTH(I325))*$C$34:$C$48)),"")</f>
+        <f>IF(H325&lt;&gt;"",MIN(L324,(M325-J325)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I325)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I325))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I325)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I325))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I325))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I325))*(MONTH($B$35:$B$49)=MONTH(I325))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L325" s="9">
@@ -12294,7 +12294,7 @@
         <v/>
       </c>
       <c r="K326" s="14">
-        <f>IF(H326&lt;&gt;"",MIN(L325,(M326-J326)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I326)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I326))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I326)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I326))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I326))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I326))*(MONTH($B$34:$B$48)=MONTH(I326))*$C$34:$C$48)),"")</f>
+        <f>IF(H326&lt;&gt;"",MIN(L325,(M326-J326)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I326)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I326))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I326)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I326))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I326))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I326))*(MONTH($B$35:$B$49)=MONTH(I326))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L326" s="14">
@@ -12328,7 +12328,7 @@
         <v/>
       </c>
       <c r="K327" s="9">
-        <f>IF(H327&lt;&gt;"",MIN(L326,(M327-J327)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I327)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I327))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I327)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I327))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I327))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I327))*(MONTH($B$34:$B$48)=MONTH(I327))*$C$34:$C$48)),"")</f>
+        <f>IF(H327&lt;&gt;"",MIN(L326,(M327-J327)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I327)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I327))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I327)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I327))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I327))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I327))*(MONTH($B$35:$B$49)=MONTH(I327))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L327" s="9">
@@ -12362,7 +12362,7 @@
         <v/>
       </c>
       <c r="K328" s="14">
-        <f>IF(H328&lt;&gt;"",MIN(L327,(M328-J328)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I328)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I328))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I328)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I328))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I328))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I328))*(MONTH($B$34:$B$48)=MONTH(I328))*$C$34:$C$48)),"")</f>
+        <f>IF(H328&lt;&gt;"",MIN(L327,(M328-J328)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I328)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I328))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I328)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I328))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I328))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I328))*(MONTH($B$35:$B$49)=MONTH(I328))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L328" s="14">
@@ -12396,7 +12396,7 @@
         <v/>
       </c>
       <c r="K329" s="9">
-        <f>IF(H329&lt;&gt;"",MIN(L328,(M329-J329)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I329)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I329))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I329)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I329))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I329))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I329))*(MONTH($B$34:$B$48)=MONTH(I329))*$C$34:$C$48)),"")</f>
+        <f>IF(H329&lt;&gt;"",MIN(L328,(M329-J329)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I329)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I329))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I329)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I329))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I329))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I329))*(MONTH($B$35:$B$49)=MONTH(I329))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L329" s="9">
@@ -12430,7 +12430,7 @@
         <v/>
       </c>
       <c r="K330" s="14">
-        <f>IF(H330&lt;&gt;"",MIN(L329,(M330-J330)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I330)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I330))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I330)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I330))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I330))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I330))*(MONTH($B$34:$B$48)=MONTH(I330))*$C$34:$C$48)),"")</f>
+        <f>IF(H330&lt;&gt;"",MIN(L329,(M330-J330)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I330)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I330))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I330)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I330))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I330))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I330))*(MONTH($B$35:$B$49)=MONTH(I330))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L330" s="14">
@@ -12464,7 +12464,7 @@
         <v/>
       </c>
       <c r="K331" s="9">
-        <f>IF(H331&lt;&gt;"",MIN(L330,(M331-J331)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I331)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I331))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I331)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I331))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I331))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I331))*(MONTH($B$34:$B$48)=MONTH(I331))*$C$34:$C$48)),"")</f>
+        <f>IF(H331&lt;&gt;"",MIN(L330,(M331-J331)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I331)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I331))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I331)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I331))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I331))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I331))*(MONTH($B$35:$B$49)=MONTH(I331))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L331" s="9">
@@ -12498,7 +12498,7 @@
         <v/>
       </c>
       <c r="K332" s="14">
-        <f>IF(H332&lt;&gt;"",MIN(L331,(M332-J332)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I332)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I332))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I332)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I332))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I332))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I332))*(MONTH($B$34:$B$48)=MONTH(I332))*$C$34:$C$48)),"")</f>
+        <f>IF(H332&lt;&gt;"",MIN(L331,(M332-J332)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I332)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I332))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I332)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I332))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I332))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I332))*(MONTH($B$35:$B$49)=MONTH(I332))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L332" s="14">
@@ -12532,7 +12532,7 @@
         <v/>
       </c>
       <c r="K333" s="9">
-        <f>IF(H333&lt;&gt;"",MIN(L332,(M333-J333)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I333)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I333))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I333)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I333))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I333))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I333))*(MONTH($B$34:$B$48)=MONTH(I333))*$C$34:$C$48)),"")</f>
+        <f>IF(H333&lt;&gt;"",MIN(L332,(M333-J333)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I333)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I333))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I333)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I333))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I333))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I333))*(MONTH($B$35:$B$49)=MONTH(I333))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L333" s="9">
@@ -12566,7 +12566,7 @@
         <v/>
       </c>
       <c r="K334" s="14">
-        <f>IF(H334&lt;&gt;"",MIN(L333,(M334-J334)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I334)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I334))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I334)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I334))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I334))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I334))*(MONTH($B$34:$B$48)=MONTH(I334))*$C$34:$C$48)),"")</f>
+        <f>IF(H334&lt;&gt;"",MIN(L333,(M334-J334)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I334)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I334))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I334)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I334))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I334))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I334))*(MONTH($B$35:$B$49)=MONTH(I334))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L334" s="14">
@@ -12600,7 +12600,7 @@
         <v/>
       </c>
       <c r="K335" s="9">
-        <f>IF(H335&lt;&gt;"",MIN(L334,(M335-J335)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I335)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I335))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I335)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I335))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I335))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I335))*(MONTH($B$34:$B$48)=MONTH(I335))*$C$34:$C$48)),"")</f>
+        <f>IF(H335&lt;&gt;"",MIN(L334,(M335-J335)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I335)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I335))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I335)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I335))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I335))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I335))*(MONTH($B$35:$B$49)=MONTH(I335))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L335" s="9">
@@ -12634,7 +12634,7 @@
         <v/>
       </c>
       <c r="K336" s="14">
-        <f>IF(H336&lt;&gt;"",MIN(L335,(M336-J336)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I336)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I336))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I336)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I336))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I336))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I336))*(MONTH($B$34:$B$48)=MONTH(I336))*$C$34:$C$48)),"")</f>
+        <f>IF(H336&lt;&gt;"",MIN(L335,(M336-J336)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I336)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I336))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I336)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I336))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I336))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I336))*(MONTH($B$35:$B$49)=MONTH(I336))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L336" s="14">
@@ -12668,7 +12668,7 @@
         <v/>
       </c>
       <c r="K337" s="9">
-        <f>IF(H337&lt;&gt;"",MIN(L336,(M337-J337)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I337)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I337))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I337)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I337))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I337))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I337))*(MONTH($B$34:$B$48)=MONTH(I337))*$C$34:$C$48)),"")</f>
+        <f>IF(H337&lt;&gt;"",MIN(L336,(M337-J337)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I337)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I337))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I337)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I337))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I337))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I337))*(MONTH($B$35:$B$49)=MONTH(I337))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L337" s="9">
@@ -12702,7 +12702,7 @@
         <v/>
       </c>
       <c r="K338" s="14">
-        <f>IF(H338&lt;&gt;"",MIN(L337,(M338-J338)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I338)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I338))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I338)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I338))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I338))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I338))*(MONTH($B$34:$B$48)=MONTH(I338))*$C$34:$C$48)),"")</f>
+        <f>IF(H338&lt;&gt;"",MIN(L337,(M338-J338)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I338)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I338))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I338)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I338))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I338))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I338))*(MONTH($B$35:$B$49)=MONTH(I338))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L338" s="14">
@@ -12736,7 +12736,7 @@
         <v/>
       </c>
       <c r="K339" s="9">
-        <f>IF(H339&lt;&gt;"",MIN(L338,(M339-J339)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I339)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I339))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I339)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I339))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I339))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I339))*(MONTH($B$34:$B$48)=MONTH(I339))*$C$34:$C$48)),"")</f>
+        <f>IF(H339&lt;&gt;"",MIN(L338,(M339-J339)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I339)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I339))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I339)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I339))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I339))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I339))*(MONTH($B$35:$B$49)=MONTH(I339))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L339" s="9">
@@ -12770,7 +12770,7 @@
         <v/>
       </c>
       <c r="K340" s="14">
-        <f>IF(H340&lt;&gt;"",MIN(L339,(M340-J340)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I340)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I340))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I340)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I340))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I340))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I340))*(MONTH($B$34:$B$48)=MONTH(I340))*$C$34:$C$48)),"")</f>
+        <f>IF(H340&lt;&gt;"",MIN(L339,(M340-J340)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I340)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I340))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I340)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I340))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I340))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I340))*(MONTH($B$35:$B$49)=MONTH(I340))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L340" s="14">
@@ -12804,7 +12804,7 @@
         <v/>
       </c>
       <c r="K341" s="9">
-        <f>IF(H341&lt;&gt;"",MIN(L340,(M341-J341)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I341)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I341))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I341)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I341))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I341))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I341))*(MONTH($B$34:$B$48)=MONTH(I341))*$C$34:$C$48)),"")</f>
+        <f>IF(H341&lt;&gt;"",MIN(L340,(M341-J341)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I341)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I341))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I341)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I341))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I341))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I341))*(MONTH($B$35:$B$49)=MONTH(I341))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L341" s="9">
@@ -12838,7 +12838,7 @@
         <v/>
       </c>
       <c r="K342" s="14">
-        <f>IF(H342&lt;&gt;"",MIN(L341,(M342-J342)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I342)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I342))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I342)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I342))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I342))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I342))*(MONTH($B$34:$B$48)=MONTH(I342))*$C$34:$C$48)),"")</f>
+        <f>IF(H342&lt;&gt;"",MIN(L341,(M342-J342)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I342)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I342))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I342)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I342))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I342))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I342))*(MONTH($B$35:$B$49)=MONTH(I342))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L342" s="14">
@@ -12872,7 +12872,7 @@
         <v/>
       </c>
       <c r="K343" s="9">
-        <f>IF(H343&lt;&gt;"",MIN(L342,(M343-J343)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I343)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I343))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I343)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I343))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I343))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I343))*(MONTH($B$34:$B$48)=MONTH(I343))*$C$34:$C$48)),"")</f>
+        <f>IF(H343&lt;&gt;"",MIN(L342,(M343-J343)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I343)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I343))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I343)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I343))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I343))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I343))*(MONTH($B$35:$B$49)=MONTH(I343))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L343" s="9">
@@ -12906,7 +12906,7 @@
         <v/>
       </c>
       <c r="K344" s="14">
-        <f>IF(H344&lt;&gt;"",MIN(L343,(M344-J344)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I344)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I344))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I344)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I344))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I344))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I344))*(MONTH($B$34:$B$48)=MONTH(I344))*$C$34:$C$48)),"")</f>
+        <f>IF(H344&lt;&gt;"",MIN(L343,(M344-J344)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I344)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I344))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I344)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I344))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I344))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I344))*(MONTH($B$35:$B$49)=MONTH(I344))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L344" s="14">
@@ -12940,7 +12940,7 @@
         <v/>
       </c>
       <c r="K345" s="9">
-        <f>IF(H345&lt;&gt;"",MIN(L344,(M345-J345)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I345)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I345))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I345)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I345))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I345))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I345))*(MONTH($B$34:$B$48)=MONTH(I345))*$C$34:$C$48)),"")</f>
+        <f>IF(H345&lt;&gt;"",MIN(L344,(M345-J345)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I345)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I345))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I345)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I345))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I345))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I345))*(MONTH($B$35:$B$49)=MONTH(I345))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L345" s="9">
@@ -12974,7 +12974,7 @@
         <v/>
       </c>
       <c r="K346" s="14">
-        <f>IF(H346&lt;&gt;"",MIN(L345,(M346-J346)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I346)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I346))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I346)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I346))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I346))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I346))*(MONTH($B$34:$B$48)=MONTH(I346))*$C$34:$C$48)),"")</f>
+        <f>IF(H346&lt;&gt;"",MIN(L345,(M346-J346)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I346)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I346))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I346)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I346))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I346))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I346))*(MONTH($B$35:$B$49)=MONTH(I346))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L346" s="14">
@@ -13008,7 +13008,7 @@
         <v/>
       </c>
       <c r="K347" s="9">
-        <f>IF(H347&lt;&gt;"",MIN(L346,(M347-J347)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I347)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I347))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I347)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I347))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I347))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I347))*(MONTH($B$34:$B$48)=MONTH(I347))*$C$34:$C$48)),"")</f>
+        <f>IF(H347&lt;&gt;"",MIN(L346,(M347-J347)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I347)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I347))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I347)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I347))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I347))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I347))*(MONTH($B$35:$B$49)=MONTH(I347))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L347" s="9">
@@ -13042,7 +13042,7 @@
         <v/>
       </c>
       <c r="K348" s="14">
-        <f>IF(H348&lt;&gt;"",MIN(L347,(M348-J348)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I348)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I348))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I348)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I348))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I348))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I348))*(MONTH($B$34:$B$48)=MONTH(I348))*$C$34:$C$48)),"")</f>
+        <f>IF(H348&lt;&gt;"",MIN(L347,(M348-J348)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I348)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I348))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I348)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I348))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I348))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I348))*(MONTH($B$35:$B$49)=MONTH(I348))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L348" s="14">
@@ -13076,7 +13076,7 @@
         <v/>
       </c>
       <c r="K349" s="9">
-        <f>IF(H349&lt;&gt;"",MIN(L348,(M349-J349)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I349)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I349))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I349)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I349))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I349))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I349))*(MONTH($B$34:$B$48)=MONTH(I349))*$C$34:$C$48)),"")</f>
+        <f>IF(H349&lt;&gt;"",MIN(L348,(M349-J349)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I349)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I349))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I349)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I349))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I349))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I349))*(MONTH($B$35:$B$49)=MONTH(I349))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L349" s="9">
@@ -13110,7 +13110,7 @@
         <v/>
       </c>
       <c r="K350" s="14">
-        <f>IF(H350&lt;&gt;"",MIN(L349,(M350-J350)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I350)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I350))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I350)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I350))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I350))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I350))*(MONTH($B$34:$B$48)=MONTH(I350))*$C$34:$C$48)),"")</f>
+        <f>IF(H350&lt;&gt;"",MIN(L349,(M350-J350)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I350)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I350))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I350)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I350))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I350))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I350))*(MONTH($B$35:$B$49)=MONTH(I350))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L350" s="14">
@@ -13144,7 +13144,7 @@
         <v/>
       </c>
       <c r="K351" s="9">
-        <f>IF(H351&lt;&gt;"",MIN(L350,(M351-J351)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I351)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I351))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I351)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I351))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I351))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I351))*(MONTH($B$34:$B$48)=MONTH(I351))*$C$34:$C$48)),"")</f>
+        <f>IF(H351&lt;&gt;"",MIN(L350,(M351-J351)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I351)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I351))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I351)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I351))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I351))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I351))*(MONTH($B$35:$B$49)=MONTH(I351))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L351" s="9">
@@ -13178,7 +13178,7 @@
         <v/>
       </c>
       <c r="K352" s="14">
-        <f>IF(H352&lt;&gt;"",MIN(L351,(M352-J352)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I352)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I352))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I352)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I352))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I352))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I352))*(MONTH($B$34:$B$48)=MONTH(I352))*$C$34:$C$48)),"")</f>
+        <f>IF(H352&lt;&gt;"",MIN(L351,(M352-J352)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I352)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I352))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I352)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I352))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I352))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I352))*(MONTH($B$35:$B$49)=MONTH(I352))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L352" s="14">
@@ -13212,7 +13212,7 @@
         <v/>
       </c>
       <c r="K353" s="9">
-        <f>IF(H353&lt;&gt;"",MIN(L352,(M353-J353)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I353)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I353))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I353)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I353))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I353))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I353))*(MONTH($B$34:$B$48)=MONTH(I353))*$C$34:$C$48)),"")</f>
+        <f>IF(H353&lt;&gt;"",MIN(L352,(M353-J353)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I353)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I353))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I353)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I353))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I353))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I353))*(MONTH($B$35:$B$49)=MONTH(I353))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L353" s="9">
@@ -13246,7 +13246,7 @@
         <v/>
       </c>
       <c r="K354" s="14">
-        <f>IF(H354&lt;&gt;"",MIN(L353,(M354-J354)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I354)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I354))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I354)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I354))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I354))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I354))*(MONTH($B$34:$B$48)=MONTH(I354))*$C$34:$C$48)),"")</f>
+        <f>IF(H354&lt;&gt;"",MIN(L353,(M354-J354)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I354)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I354))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I354)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I354))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I354))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I354))*(MONTH($B$35:$B$49)=MONTH(I354))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L354" s="14">
@@ -13280,7 +13280,7 @@
         <v/>
       </c>
       <c r="K355" s="9">
-        <f>IF(H355&lt;&gt;"",MIN(L354,(M355-J355)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I355)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I355))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I355)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I355))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I355))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I355))*(MONTH($B$34:$B$48)=MONTH(I355))*$C$34:$C$48)),"")</f>
+        <f>IF(H355&lt;&gt;"",MIN(L354,(M355-J355)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I355)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I355))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I355)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I355))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I355))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I355))*(MONTH($B$35:$B$49)=MONTH(I355))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L355" s="9">
@@ -13314,7 +13314,7 @@
         <v/>
       </c>
       <c r="K356" s="14">
-        <f>IF(H356&lt;&gt;"",MIN(L355,(M356-J356)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I356)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I356))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I356)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I356))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I356))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I356))*(MONTH($B$34:$B$48)=MONTH(I356))*$C$34:$C$48)),"")</f>
+        <f>IF(H356&lt;&gt;"",MIN(L355,(M356-J356)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I356)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I356))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I356)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I356))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I356))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I356))*(MONTH($B$35:$B$49)=MONTH(I356))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L356" s="14">
@@ -13348,7 +13348,7 @@
         <v/>
       </c>
       <c r="K357" s="9">
-        <f>IF(H357&lt;&gt;"",MIN(L356,(M357-J357)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I357)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I357))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I357)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I357))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I357))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I357))*(MONTH($B$34:$B$48)=MONTH(I357))*$C$34:$C$48)),"")</f>
+        <f>IF(H357&lt;&gt;"",MIN(L356,(M357-J357)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I357)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I357))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I357)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I357))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I357))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I357))*(MONTH($B$35:$B$49)=MONTH(I357))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L357" s="9">
@@ -13382,7 +13382,7 @@
         <v/>
       </c>
       <c r="K358" s="14">
-        <f>IF(H358&lt;&gt;"",MIN(L357,(M358-J358)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I358)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I358))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I358)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I358))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I358))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I358))*(MONTH($B$34:$B$48)=MONTH(I358))*$C$34:$C$48)),"")</f>
+        <f>IF(H358&lt;&gt;"",MIN(L357,(M358-J358)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I358)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I358))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I358)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I358))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I358))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I358))*(MONTH($B$35:$B$49)=MONTH(I358))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L358" s="14">
@@ -13416,7 +13416,7 @@
         <v/>
       </c>
       <c r="K359" s="9">
-        <f>IF(H359&lt;&gt;"",MIN(L358,(M359-J359)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I359)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I359))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I359)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I359))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I359))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I359))*(MONTH($B$34:$B$48)=MONTH(I359))*$C$34:$C$48)),"")</f>
+        <f>IF(H359&lt;&gt;"",MIN(L358,(M359-J359)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I359)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I359))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I359)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I359))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I359))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I359))*(MONTH($B$35:$B$49)=MONTH(I359))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L359" s="9">
@@ -13450,7 +13450,7 @@
         <v/>
       </c>
       <c r="K360" s="14">
-        <f>IF(H360&lt;&gt;"",MIN(L359,(M360-J360)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I360)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I360))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I360)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I360))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I360))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I360))*(MONTH($B$34:$B$48)=MONTH(I360))*$C$34:$C$48)),"")</f>
+        <f>IF(H360&lt;&gt;"",MIN(L359,(M360-J360)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I360)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I360))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I360)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I360))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I360))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I360))*(MONTH($B$35:$B$49)=MONTH(I360))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L360" s="14">
@@ -13484,7 +13484,7 @@
         <v/>
       </c>
       <c r="K361" s="9">
-        <f>IF(H361&lt;&gt;"",MIN(L360,(M361-J361)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I361)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I361))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I361)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I361))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I361))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I361))*(MONTH($B$34:$B$48)=MONTH(I361))*$C$34:$C$48)),"")</f>
+        <f>IF(H361&lt;&gt;"",MIN(L360,(M361-J361)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I361)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I361))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I361)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I361))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I361))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I361))*(MONTH($B$35:$B$49)=MONTH(I361))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L361" s="9">
@@ -13518,7 +13518,7 @@
         <v/>
       </c>
       <c r="K362" s="14">
-        <f>IF(H362&lt;&gt;"",MIN(L361,(M362-J362)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I362)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I362))*($E$21:$E$30="Monthly")*$D$21:$D$30)+SUMPRODUCT(($B$21:$B$30&lt;&gt;"")*($B$21:$B$30&lt;=I362)*(($C$21:$C$30="")+($C$21:$C$30&lt;&gt;"")*($C$21:$C$30&gt;=I362))*($E$21:$E$30="Annual")*(MONTH($B$21:$B$30)=MONTH(I362))*$D$21:$D$30)+SUMPRODUCT(($B$34:$B$48&lt;&gt;"")*(YEAR($B$34:$B$48)=YEAR(I362))*(MONTH($B$34:$B$48)=MONTH(I362))*$C$34:$C$48)),"")</f>
+        <f>IF(H362&lt;&gt;"",MIN(L361,(M362-J362)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I362)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I362))*($E$22:$E$31="Monthly")*$D$22:$D$31)+SUMPRODUCT(($B$22:$B$31&lt;&gt;"")*($B$22:$B$31&lt;=I362)*(($C$22:$C$31="")+($C$22:$C$31&lt;&gt;"")*($C$22:$C$31&gt;=I362))*($E$22:$E$31="Annual")*(MONTH($B$22:$B$31)=MONTH(I362))*$D$22:$D$31)+SUMPRODUCT(($B$35:$B$49&lt;&gt;"")*(YEAR($B$35:$B$49)=YEAR(I362))*(MONTH($B$35:$B$49)=MONTH(I362))*$C$35:$C$49)),"")</f>
         <v/>
       </c>
       <c r="L362" s="14">
@@ -13540,14 +13540,14 @@
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A32:C32"/>
-    <mergeCell ref="A19:E19"/>
+    <mergeCell ref="A33:C33"/>
+    <mergeCell ref="A20:E20"/>
     <mergeCell ref="H1:L1"/>
     <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A9:B9"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="E21:E30" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Frequency" error="Please select Monthly or Annual" type="list">
+    <dataValidation sqref="E22:E31" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Frequency" error="Please select Monthly or Annual" type="list">
       <formula1>"Monthly,Annual"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>